<commit_message>
Refactor the whole code
</commit_message>
<xml_diff>
--- a/results_fcgma/ResultsCompMethod.xlsx
+++ b/results_fcgma/ResultsCompMethod.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,85 +438,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[[1. 0. 0. ... 0. 0. 0.]
- [0. 0. 1. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- ...
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]]</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>571.9532470703125</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>[547.602294921875, 552.4946899414062, 552.4946899414062, 552.4946899414062, 552.4946899414062, 554.5687866210938, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 570.8800659179688, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.838623046875, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125, 571.9532470703125]</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>[[1. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 1. ... 0. 0. 0.]
- ...
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]]</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>574.4638671875</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>[547.602294921875, 547.602294921875, 548.5890502929688, 554.3598022460938, 554.8607177734375, 554.8607177734375, 554.8607177734375, 554.8607177734375, 554.8607177734375, 557.3465576171875, 557.3465576171875, 560.3350830078125, 560.3350830078125, 563.3157348632812, 563.3157348632812, 563.3157348632812, 563.3157348632812, 563.3157348632812, 563.3157348632812, 563.3157348632812, 563.3157348632812, 563.3157348632812, 563.3157348632812, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 568.5697021484375, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 570.4391479492188, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875, 574.4638671875]</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>[[1. 0. 0. ... 0. 0. 0.]
- [0. 0. 1. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- ...
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]]</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>576.7672119140625</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>[547.602294921875, 547.602294921875, 553.8333129882812, 554.8280029296875, 554.8280029296875, 554.8280029296875, 554.8280029296875, 554.8280029296875, 559.8421630859375, 559.8421630859375, 559.8421630859375, 559.8421630859375, 559.851806640625, 559.851806640625, 559.851806640625, 559.851806640625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625, 576.7672119140625]</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>[[0. 1. 0. ... 0. 0. 0.]
+          <t>[[0. 0. 0. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]
  ...
@@ -525,168 +447,12 @@
  [0. 0. 0. ... 0. 0. 0.]]</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>574.0414428710938</v>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="C2" t="n">
+        <v>10.33769989013672</v>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
-          <t>[547.602294921875, 547.602294921875, 547.602294921875, 547.602294921875, 551.9946899414062, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 560.4426879882812, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 562.060791015625, 564.5723266601562, 564.5723266601562, 564.5723266601562, 564.5723266601562, 564.5723266601562, 564.5723266601562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 565.3174438476562, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938, 574.0414428710938]</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>[[1. 0. 0. ... 0. 0. 0.]
- [0. 0. 1. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- ...
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]]</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>579.9100341796875</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>[547.602294921875, 547.602294921875, 547.7874755859375, 551.4197998046875, 551.9417724609375, 551.9417724609375, 551.9417724609375, 558.9391479492188, 558.9391479492188, 558.9391479492188, 558.9391479492188, 560.42333984375, 560.42333984375, 560.42333984375, 560.42333984375, 560.42333984375, 560.42333984375, 560.42333984375, 560.42333984375, 560.42333984375, 560.42333984375, 560.42333984375, 561.5220947265625, 561.5220947265625, 561.5220947265625, 561.5220947265625, 561.5220947265625, 561.5687866210938, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 573.7760009765625, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875, 579.9100341796875]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>[[1. 0. 0. ... 0. 0. 0.]
- [0. 1. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- ...
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]]</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>578.6516723632812</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>[547.602294921875, 547.602294921875, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.4744262695312, 559.7645263671875, 559.7645263671875, 559.7645263671875, 559.7645263671875, 559.7645263671875, 559.7645263671875, 559.7645263671875, 559.7645263671875, 559.7645263671875, 559.7645263671875, 559.7645263671875, 559.7645263671875, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812, 578.6516723632812]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>[[1. 0. 0. ... 0. 0. 0.]
- [0. 1. 0. ... 0. 0. 0.]
- [0. 0. 1. ... 0. 0. 0.]
- ...
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]]</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>570.275146484375</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>[547.602294921875, 547.602294921875, 547.602294921875, 550.811279296875, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 562.9365234375, 565.5970458984375, 565.5970458984375, 565.5970458984375, 565.5970458984375, 565.5970458984375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375, 570.275146484375]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>[[1. 0. 0. ... 0. 0. 0.]
- [0. 1. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- ...
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]]</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>583.7380981445312</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>[547.602294921875, 556.0873413085938, 556.0873413085938, 565.8218994140625, 565.8218994140625, 565.8218994140625, 565.8218994140625, 565.8218994140625, 565.8218994140625, 565.8218994140625, 565.8218994140625, 565.8218994140625, 565.8218994140625, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 566.447998046875, 569.034423828125, 569.034423828125, 569.034423828125, 569.034423828125, 569.034423828125, 569.034423828125, 569.034423828125, 569.034423828125, 569.034423828125, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 571.2980346679688, 572.2998046875, 572.2998046875, 572.2998046875, 572.2998046875, 572.2998046875, 572.2998046875, 572.2998046875, 572.2998046875, 572.2998046875, 572.2998046875, 572.2998046875, 576.736328125, 576.736328125, 576.736328125, 576.736328125, 576.736328125, 576.736328125, 576.736328125, 576.736328125, 576.736328125, 579.7389526367188, 579.7389526367188, 579.7389526367188, 579.7389526367188, 580.239013671875, 580.239013671875, 580.239013671875, 582.738037109375, 582.738037109375, 582.738037109375, 582.738037109375, 582.738037109375, 583.238037109375, 583.238037109375, 583.238037109375, 583.2380981445312, 583.7380981445312, 583.7380981445312]</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>[[0. 1. 0. ... 0. 0. 0.]
- [0. 0. 1. ... 0. 0. 0.]
- [1. 0. 0. ... 0. 0. 0.]
- ...
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]]</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>579.3695068359375</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>[547.602294921875, 547.602294921875, 550.52294921875, 550.7716064453125, 551.6693115234375, 552.6834106445312, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 563.397705078125, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375, 579.3695068359375]</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>[[1. 0. 0. ... 0. 0. 0.]
- [0. 1. 0. ... 0. 0. 0.]
- [0. 0. 1. ... 0. 0. 0.]
- ...
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]]</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>570.43212890625</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>[547.602294921875, 547.602294921875, 552.0379028320312, 552.0379028320312, 552.0379028320312, 552.0379028320312, 553.4664916992188, 553.4664916992188, 562.41357421875, 562.41357421875, 562.41357421875, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 564.9805908203125, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625, 570.43212890625]</t>
+          <t>[6.964300155639648, 6.971400260925293, 7.488400459289551, 7.488400459289551, 7.488400459289551, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.635500431060791, 7.635500431060791, 7.683699607849121, 7.683699607849121, 7.683699607849121, 7.683699607849121, 8.038800239562988, 8.038800239562988, 8.086099624633789, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.526300430297852, 8.526300430297852, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.724699974060059, 8.724699974060059, 8.724699974060059, 8.724699974060059, 8.846700668334961, 8.846700668334961, 8.847900390625, 8.847900390625, 8.939499855041504, 8.957099914550781, 8.9822998046875, 8.9822998046875, 8.9822998046875, 9.024499893188477, 9.047100067138672, 9.047100067138672, 9.122400283813477, 9.122400283813477, 9.122400283813477, 9.14739990234375, 9.14739990234375, 9.163100242614746, 9.170499801635742, 9.17609977722168, 9.217399597167969, 9.363900184631348, 9.363900184631348, 9.363900184631348, 9.406400680541992, 9.443599700927734, 9.443599700927734, 9.463900566101074, 9.463900566101074, 9.50100040435791, 9.54010009765625, 9.651800155639648, 9.67449951171875, 9.67449951171875, 9.791799545288086, 9.801000595092773, 9.801000595092773, 9.828399658203125, 9.828399658203125, 9.895099639892578, 9.910400390625, 9.910400390625, 9.910900115966797, 9.911800384521484, 10.04740047454834, 10.04740047454834, 10.064599990844727, 10.064599990844727, 10.064599990844727, 10.146900177001953, 10.146900177001953, 10.153200149536133, 10.170499801635742, 10.170499801635742, 10.181499481201172, 10.194900512695312, 10.23390007019043, 10.263200759887695, 10.263400077819824, 10.274101257324219, 10.274101257324219, 10.280399322509766, 10.337699890136719]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the latest result of mayfly algorithm
</commit_message>
<xml_diff>
--- a/results_fcgma/ResultsCompMethod.xlsx
+++ b/results_fcgma/ResultsCompMethod.xlsx
@@ -439,7 +439,7 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>[[0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
+ [0. 0. 1. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]
  ...
  [0. 0. 0. ... 0. 0. 0.]
@@ -448,11 +448,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.33769989013672</v>
+        <v>44.91519927978516</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[6.964300155639648, 6.971400260925293, 7.488400459289551, 7.488400459289551, 7.488400459289551, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.635500431060791, 7.635500431060791, 7.683699607849121, 7.683699607849121, 7.683699607849121, 7.683699607849121, 8.038800239562988, 8.038800239562988, 8.086099624633789, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.526300430297852, 8.526300430297852, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.724699974060059, 8.724699974060059, 8.724699974060059, 8.724699974060059, 8.846700668334961, 8.846700668334961, 8.847900390625, 8.847900390625, 8.939499855041504, 8.957099914550781, 8.9822998046875, 8.9822998046875, 8.9822998046875, 9.024499893188477, 9.047100067138672, 9.047100067138672, 9.122400283813477, 9.122400283813477, 9.122400283813477, 9.14739990234375, 9.14739990234375, 9.163100242614746, 9.170499801635742, 9.17609977722168, 9.217399597167969, 9.363900184631348, 9.363900184631348, 9.363900184631348, 9.406400680541992, 9.443599700927734, 9.443599700927734, 9.463900566101074, 9.463900566101074, 9.50100040435791, 9.54010009765625, 9.651800155639648, 9.67449951171875, 9.67449951171875, 9.791799545288086, 9.801000595092773, 9.801000595092773, 9.828399658203125, 9.828399658203125, 9.895099639892578, 9.910400390625, 9.910400390625, 9.910900115966797, 9.911800384521484, 10.04740047454834, 10.04740047454834, 10.064599990844727, 10.064599990844727, 10.064599990844727, 10.146900177001953, 10.146900177001953, 10.153200149536133, 10.170499801635742, 10.170499801635742, 10.181499481201172, 10.194900512695312, 10.23390007019043, 10.263200759887695, 10.263400077819824, 10.274101257324219, 10.274101257324219, 10.280399322509766, 10.337699890136719]</t>
+          <t>[25.464200973510742, 25.464200973510742, 25.48550033569336, 25.692399978637695, 26.002899169921875, 26.002899169921875, 26.133899688720703, 26.329498291015625, 26.329498291015625, 26.329498291015625, 26.329498291015625, 26.340301513671875, 26.42930030822754, 26.42930030822754, 26.42930030822754, 26.527301788330078, 26.684398651123047, 26.968299865722656, 26.968299865722656, 26.968299865722656, 26.968299865722656, 26.968299865722656, 27.01609992980957, 27.11050033569336, 27.454801559448242, 27.454801559448242, 27.454801559448242, 27.523601531982422, 27.541698455810547, 27.541698455810547, 27.541698455810547, 27.99880027770996, 27.99880027770996, 27.99880027770996, 27.99880027770996, 27.99880027770996, 28.095802307128906, 28.61240005493164, 28.61240005493164, 28.864700317382812, 28.864700317382812, 28.864700317382812, 28.864700317382812, 28.864700317382812, 29.00309944152832, 29.00309944152832, 29.00309944152832, 29.03839874267578, 29.484098434448242, 29.510799407958984, 29.510799407958984, 29.69499969482422, 29.69499969482422, 30.123199462890625, 30.123199462890625, 30.123199462890625, 30.123199462890625, 30.123199462890625, 30.448301315307617, 30.448301315307617, 30.448301315307617, 30.448301315307617, 30.448301315307617, 30.50040054321289, 30.519500732421875, 30.646800994873047, 30.646800994873047, 30.646800994873047, 30.830799102783203, 30.843399047851562, 30.98040008544922, 31.06570053100586, 31.068599700927734, 31.29800033569336, 31.29800033569336, 31.29800033569336, 31.29800033569336, 31.396800994873047, 31.6260986328125, 31.6260986328125, 31.6260986328125, 31.6260986328125, 31.66080093383789, 31.66080093383789, 31.66080093383789, 31.881099700927734, 31.881099700927734, 31.924701690673828, 31.924701690673828, 32.22740173339844, 32.22740173339844, 32.22740173339844, 32.33210372924805, 32.33210372924805, 32.3838996887207, 32.65229797363281, 32.65229797363281, 32.65229797363281, 32.704200744628906, 32.85499954223633, 32.85499954223633, 32.85499954223633, 32.85499954223633, 32.85499954223633, 32.86869812011719, 32.924800872802734, 32.924800872802734, 33.060001373291016, 33.07080078125, 33.07080078125, 33.131202697753906, 33.131202697753906, 33.131202697753906, 33.14140319824219, 33.23310089111328, 33.23310089111328, 33.23310089111328, 33.239402770996094, 33.2843017578125, 33.343299865722656, 33.344200134277344, 33.36119842529297, 33.39739990234375, 33.39739990234375, 33.39739990234375, 33.39739990234375, 33.39739990234375, 33.490997314453125, 33.490997314453125, 33.56209945678711, 33.582801818847656, 33.582801818847656, 33.707401275634766, 33.767398834228516, 33.767398834228516, 33.791900634765625, 33.791900634765625, 33.791900634765625, 33.84880065917969, 33.861900329589844, 33.861900329589844, 33.89649963378906, 33.89649963378906, 33.9276008605957, 33.9276008605957, 33.92770004272461, 33.92770004272461, 33.96500015258789, 33.96500015258789, 33.96500015258789, 33.970802307128906, 33.97169876098633, 33.971797943115234, 34.00080108642578, 34.03120040893555, 34.03120040893555, 34.06880187988281, 34.06880187988281, 34.07390213012695, 34.07390213012695, 34.07390213012695, 34.11159896850586, 34.17539978027344, 34.17539978027344, 34.17539978027344, 34.18450164794922, 34.19750213623047, 34.220001220703125, 34.246700286865234, 34.246700286865234, 34.25, 34.2776985168457, 34.2776985168457, 34.2776985168457, 34.32469940185547, 34.329200744628906, 34.342201232910156, 34.38159942626953, 34.38159942626953, 34.38159942626953, 34.38629913330078, 34.38629913330078, 34.41350173950195, 34.43219757080078, 34.43219757080078, 34.53300094604492, 34.53300094604492, 34.53300094604492, 34.63850021362305, 34.69490051269531, 34.72730255126953, 34.72730255126953, 34.72730255126953, 34.72730255126953, 34.72730255126953, 34.77429962158203, 34.80000305175781, 34.82429885864258, 34.8754997253418, 34.8754997253418, 34.8754997253418, 34.8754997253418, 34.87900161743164, 34.87900161743164, 34.88890075683594, 34.89350128173828, 34.90409851074219, 34.965599060058594, 34.965599060058594, 34.97480010986328, 34.97480010986328, 35.030601501464844, 35.030601501464844, 35.030601501464844, 35.030601501464844, 35.030601501464844, 35.04610061645508, 35.04610061645508, 35.085201263427734, 35.085201263427734, 35.08700180053711, 35.18010330200195, 35.18010330200195, 35.19499969482422, 35.19499969482422, 35.19499969482422, 35.26470184326172, 35.26470184326172, 35.26570129394531, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.36309814453125, 35.36309814453125, 35.44349670410156, 35.44349670410156, 35.46039581298828, 35.46039581298828, 35.55139923095703, 35.55139923095703, 35.56999969482422, 35.63290023803711, 35.71310043334961, 35.71310043334961, 35.7218017578125, 35.742000579833984, 35.742000579833984, 35.742000579833984, 35.804100036621094, 35.88420104980469, 35.88420104980469, 35.949798583984375, 35.949798583984375, 35.949798583984375, 35.949798583984375, 36.053199768066406, 36.055999755859375, 36.055999755859375, 36.057899475097656, 36.10230255126953, 36.10230255126953, 36.10309982299805, 36.10309982299805, 36.13140106201172, 36.13140106201172, 36.13140106201172, 36.192100524902344, 36.21150207519531, 36.21150207519531, 36.212799072265625, 36.212799072265625, 36.212799072265625, 36.22899627685547, 36.277400970458984, 36.332801818847656, 36.36069869995117, 36.417598724365234, 36.436302185058594, 36.456298828125, 36.456298828125, 36.475196838378906, 36.475196838378906, 36.48400115966797, 36.5432014465332, 36.57350158691406, 36.57350158691406, 36.57350158691406, 36.70030212402344, 36.70030212402344, 36.724098205566406, 36.724098205566406, 36.740501403808594, 36.78280258178711, 36.923500061035156, 36.923500061035156, 36.923500061035156, 36.923500061035156, 36.923500061035156, 36.93709945678711, 36.93709945678711, 36.95669937133789, 36.96580123901367, 37.01679992675781, 37.03689956665039, 37.03689956665039, 37.067298889160156, 37.067298889160156, 37.07109832763672, 37.07109832763672, 37.168399810791016, 37.28239822387695, 37.28239822387695, 37.31439971923828, 37.32460021972656, 37.32460021972656, 37.332801818847656, 37.352699279785156, 37.352699279785156, 37.4109992980957, 37.4109992980957, 37.414100646972656, 37.414100646972656, 37.430198669433594, 37.430198669433594, 37.53410339355469, 37.53410339355469, 37.53410339355469, 37.53410339355469, 37.545997619628906, 37.545997619628906, 37.55419921875, 37.60919952392578, 37.61830139160156, 37.61830139160156, 37.61830139160156, 37.75320053100586, 37.75320053100586, 37.764400482177734, 37.764400482177734, 37.76810073852539, 37.76810073852539, 37.76810073852539, 37.84770202636719, 37.84770202636719, 37.85680389404297, 37.85680389404297, 37.865901947021484, 37.88189697265625, 37.88189697265625, 37.88189697265625, 37.88189697265625, 37.89360046386719, 37.92140197753906, 37.92140197753906, 37.92140197753906, 37.94640350341797, 37.94640350341797, 37.94640350341797, 38.036598205566406, 38.036598205566406, 38.036598205566406, 38.04900360107422, 38.060997009277344, 38.060997009277344, 38.060997009277344, 38.060997009277344, 38.0697021484375, 38.07820129394531, 38.131500244140625, 38.131500244140625, 38.14550018310547, 38.18800354003906, 38.18800354003906, 38.229400634765625, 38.229400634765625, 38.233299255371094, 38.25600051879883, 38.321197509765625, 38.321197509765625, 38.32569885253906, 38.32569885253906, 38.32569885253906, 38.32889938354492, 38.342498779296875, 38.349403381347656, 38.35060119628906, 38.35060119628906, 38.38639831542969, 38.38639831542969, 38.38639831542969, 38.429901123046875, 38.429901123046875, 38.44499969482422, 38.46410369873047, 38.46410369873047, 38.47090148925781, 38.47169876098633, 38.49789810180664, 38.5796012878418, 38.5796012878418, 38.5796012878418, 38.59320068359375, 38.59320068359375, 38.62919998168945, 38.62919998168945, 38.641300201416016, 38.641300201416016, 38.641395568847656, 38.650901794433594, 38.650901794433594, 38.65570068359375, 38.67179870605469, 38.67179870605469, 38.67469787597656, 38.680198669433594, 38.680198669433594, 38.680198669433594, 38.69020080566406, 38.69020080566406, 38.70170211791992, 38.70439910888672, 38.70439910888672, 38.70439910888672, 38.70439910888672, 38.70680236816406, 38.712799072265625, 38.75559997558594, 38.768096923828125, 38.768096923828125, 38.7760009765625, 38.77870178222656, 38.78369903564453, 38.794097900390625, 38.799102783203125, 38.799102783203125, 38.84290313720703, 38.86250305175781, 38.86250305175781, 38.8754997253418, 38.897300720214844, 38.90769958496094, 38.90769958496094, 38.94029998779297, 38.94029998779297, 38.94029998779297, 38.95399856567383, 38.970401763916016, 38.970401763916016, 38.99089813232422, 38.995201110839844, 39.07680130004883, 39.07680130004883, 39.105098724365234, 39.1702995300293, 39.19049835205078, 39.19049835205078, 39.2317008972168, 39.2317008972168, 39.26620101928711, 39.26620101928711, 39.29500198364258, 39.38960266113281, 39.393402099609375, 39.416500091552734, 39.416500091552734, 39.43429946899414, 39.43429946899414, 39.466697692871094, 39.51319885253906, 39.51319885253906, 39.51319885253906, 39.546600341796875, 39.546600341796875, 39.546600341796875, 39.593299865722656, 39.60029983520508, 39.61429977416992, 39.61869812011719, 39.62220001220703, 39.651702880859375, 39.651702880859375, 39.651702880859375, 39.651702880859375, 39.66400146484375, 39.66400146484375, 39.67720031738281, 39.68949890136719, 39.70649719238281, 39.70649719238281, 39.70840072631836, 39.70840072631836, 39.728599548339844, 39.730499267578125, 39.745399475097656, 39.745399475097656, 39.75749969482422, 39.77619934082031, 39.77619934082031, 39.77619934082031, 39.77619934082031, 39.777400970458984, 39.777400970458984, 39.777400970458984, 39.82859802246094, 39.885501861572266, 39.92759704589844, 39.938697814941406, 39.938697814941406, 39.94159698486328, 39.95349884033203, 39.95349884033203, 39.98249816894531, 39.98249816894531, 39.9911994934082, 40.026798248291016, 40.026798248291016, 40.02799987792969, 40.09120178222656, 40.09120178222656, 40.11199951171875, 40.14720153808594, 40.15159606933594, 40.22330093383789, 40.22330093383789, 40.23259735107422, 40.23979949951172, 40.27179718017578, 40.31780242919922, 40.33830261230469, 40.36219787597656, 40.389400482177734, 40.389400482177734, 40.389400482177734, 40.399898529052734, 40.40549850463867, 40.40549850463867, 40.40549850463867, 40.40549850463867, 40.417198181152344, 40.417198181152344, 40.41780090332031, 40.48080062866211, 40.48080062866211, 40.48080062866211, 40.52330017089844, 40.54180145263672, 40.577301025390625, 40.577301025390625, 40.67359924316406, 40.67359924316406, 40.763099670410156, 40.763099670410156, 40.8302001953125, 40.840599060058594, 40.840599060058594, 40.84649658203125, 40.84870147705078, 40.84870147705078, 40.84880065917969, 40.84880065917969, 40.86479949951172, 40.86479949951172, 40.86479949951172, 40.87300109863281, 40.89820098876953, 40.907798767089844, 40.907798767089844, 40.91360092163086, 40.91360092163086, 40.91360092163086, 40.9911994934082, 41.02320098876953, 41.03010177612305, 41.03010177612305, 41.055599212646484, 41.075897216796875, 41.11070251464844, 41.11070251464844, 41.1151008605957, 41.139495849609375, 41.198299407958984, 41.198299407958984, 41.198299407958984, 41.198299407958984, 41.20880126953125, 41.20880126953125, 41.22269821166992, 41.23320007324219, 41.23320007324219, 41.23320007324219, 41.2411994934082, 41.25170135498047, 41.255897521972656, 41.27110290527344, 41.27110290527344, 41.275299072265625, 41.30970001220703, 41.30970001220703, 41.30970001220703, 41.30970001220703, 41.345699310302734, 41.345699310302734, 41.345699310302734, 41.345699310302734, 41.35890197753906, 41.3922004699707, 41.3922004699707, 41.40230178833008, 41.40230178833008, 41.40230178833008, 41.40230178833008, 41.415000915527344, 41.45110321044922, 41.455299377441406, 41.47739791870117, 41.47739791870117, 41.47739791870117, 41.50339889526367, 41.50339889526367, 41.50740051269531, 41.52149963378906, 41.548797607421875, 41.548797607421875, 41.548797607421875, 41.573402404785156, 41.573402404785156, 41.574501037597656, 41.574501037597656, 41.574501037597656, 41.63800048828125, 41.63909912109375, 41.64419937133789, 41.64419937133789, 41.65769958496094, 41.689998626708984, 41.689998626708984, 41.704795837402344, 41.704795837402344, 41.704795837402344, 41.704795837402344, 41.704795837402344, 41.71039962768555, 41.72220230102539, 41.72220230102539, 41.72620391845703, 41.73270034790039, 41.750099182128906, 41.750099182128906, 41.75830078125, 41.76319885253906, 41.77149963378906, 41.77149963378906, 41.77989959716797, 41.80889892578125, 41.80889892578125, 41.80889892578125, 41.80889892578125, 41.86119842529297, 41.86119842529297, 41.91320037841797, 41.91320037841797, 41.91320037841797, 41.96689987182617, 42.01020050048828, 42.01020050048828, 42.019100189208984, 42.03820037841797, 42.042999267578125, 42.042999267578125, 42.047096252441406, 42.047096252441406, 42.097801208496094, 42.15789794921875, 42.15789794921875, 42.16200256347656, 42.16239929199219, 42.19599914550781, 42.19599914550781, 42.199501037597656, 42.20490264892578, 42.230201721191406, 42.255699157714844, 42.27110290527344, 42.272300720214844, 42.272300720214844, 42.29460144042969, 42.29710006713867, 42.29869842529297, 42.29869842529297, 42.29869842529297, 42.329803466796875, 42.354000091552734, 42.35580062866211, 42.35580062866211, 42.358299255371094, 42.359901428222656, 42.36260223388672, 42.36920166015625, 42.38330078125, 42.38330078125, 42.38330078125, 42.479400634765625, 42.479400634765625, 42.48040008544922, 42.48040008544922, 42.48040008544922, 42.48040008544922, 42.49610137939453, 42.49610137939453, 42.49610137939453, 42.49610137939453, 42.54719924926758, 42.58489990234375, 42.589500427246094, 42.59280014038086, 42.59280014038086, 42.59280014038086, 42.59280014038086, 42.59830093383789, 42.601600646972656, 42.60969924926758, 42.60969924926758, 42.6254997253418, 42.6254997253418, 42.6525993347168, 42.6525993347168, 42.6525993347168, 42.65589904785156, 42.65589904785156, 42.65589904785156, 42.667198181152344, 42.667198181152344, 42.670501708984375, 42.670501708984375, 42.670501708984375, 42.68939971923828, 42.68939971923828, 42.69270324707031, 42.69770050048828, 42.69770050048828, 42.71800231933594, 42.71800231933594, 42.71800231933594, 42.71800231933594, 42.71800231933594, 42.7224006652832, 42.74030303955078, 42.74030303955078, 42.754798889160156, 42.76599884033203, 42.768699645996094, 42.768699645996094, 42.78209686279297, 42.78209686279297, 42.82019805908203, 42.82830047607422, 42.83899688720703, 42.83899688720703, 42.83899688720703, 42.83899688720703, 42.84579849243164, 42.84579849243164, 42.94269943237305, 42.94269943237305, 43.022499084472656, 43.022499084472656, 43.022499084472656, 43.121498107910156, 43.121498107910156, 43.121498107910156, 43.16780090332031, 43.16780090332031, 43.21119689941406, 43.213600158691406, 43.221099853515625, 43.221099853515625, 43.221099853515625, 43.22630310058594, 43.24259948730469, 43.25530242919922, 43.435298919677734, 43.435298919677734, 43.435298919677734, 43.435298919677734, 43.47869873046875, 43.47869873046875, 43.47869873046875, 43.47869873046875, 43.48759841918945, 43.525001525878906, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.588802337646484, 43.603302001953125, 43.603302001953125, 43.603302001953125, 43.603302001953125, 43.603302001953125, 43.633602142333984, 43.633602142333984, 43.640899658203125, 43.679298400878906, 43.697898864746094, 43.73100280761719, 43.73100280761719, 43.7318000793457, 43.77649688720703, 43.77649688720703, 43.77939987182617, 43.77939987182617, 43.77939987182617, 43.77939987182617, 43.82209777832031, 43.843502044677734, 43.843502044677734, 43.87670135498047, 43.87670135498047, 43.87839889526367, 43.950599670410156, 43.952301025390625, 44.037200927734375, 44.03950119018555, 44.103302001953125, 44.103302001953125, 44.1239013671875, 44.1239013671875, 44.16809844970703, 44.16809844970703, 44.183101654052734, 44.183101654052734, 44.186004638671875, 44.186004638671875, 44.206398010253906, 44.206398010253906, 44.24469757080078, 44.24869918823242, 44.24869918823242, 44.281002044677734, 44.333099365234375, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.35199737548828, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.37989807128906, 44.417198181152344, 44.417198181152344, 44.417198181152344, 44.418296813964844, 44.418296813964844, 44.418296813964844, 44.418296813964844, 44.418296813964844, 44.418800354003906, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45970153808594, 44.45970153808594, 44.45970153808594, 44.45970153808594, 44.49340057373047, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.52239990234375, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.53670120239258, 44.566898345947266, 44.566898345947266, 44.566898345947266, 44.566898345947266, 44.566898345947266, 44.57200241088867, 44.57200241088867, 44.57200241088867, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.85129928588867, 44.85129928588867, 44.85129928588867, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.86759948730469, 44.86759948730469, 44.87350082397461, 44.87350082397461, 44.87350082397461, 44.87350082397461, 44.915199279785156, 44.915199279785156, 44.915199279785156, 44.915199279785156]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update latest optimizer result
</commit_message>
<xml_diff>
--- a/results_fcgma/ResultsCompMethod.xlsx
+++ b/results_fcgma/ResultsCompMethod.xlsx
@@ -444,15 +444,15 @@
  ...
  [0. 0. 0. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]]</t>
+ [0. 0. 0. ... 1. 0. 0.]]</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.33769989013672</v>
+        <v>22.17259979248047</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[6.964300155639648, 6.971400260925293, 7.488400459289551, 7.488400459289551, 7.488400459289551, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.635500431060791, 7.635500431060791, 7.683699607849121, 7.683699607849121, 7.683699607849121, 7.683699607849121, 8.038800239562988, 8.038800239562988, 8.086099624633789, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.526300430297852, 8.526300430297852, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.724699974060059, 8.724699974060059, 8.724699974060059, 8.724699974060059, 8.846700668334961, 8.846700668334961, 8.847900390625, 8.847900390625, 8.939499855041504, 8.957099914550781, 8.9822998046875, 8.9822998046875, 8.9822998046875, 9.024499893188477, 9.047100067138672, 9.047100067138672, 9.122400283813477, 9.122400283813477, 9.122400283813477, 9.14739990234375, 9.14739990234375, 9.163100242614746, 9.170499801635742, 9.17609977722168, 9.217399597167969, 9.363900184631348, 9.363900184631348, 9.363900184631348, 9.406400680541992, 9.443599700927734, 9.443599700927734, 9.463900566101074, 9.463900566101074, 9.50100040435791, 9.54010009765625, 9.651800155639648, 9.67449951171875, 9.67449951171875, 9.791799545288086, 9.801000595092773, 9.801000595092773, 9.828399658203125, 9.828399658203125, 9.895099639892578, 9.910400390625, 9.910400390625, 9.910900115966797, 9.911800384521484, 10.04740047454834, 10.04740047454834, 10.064599990844727, 10.064599990844727, 10.064599990844727, 10.146900177001953, 10.146900177001953, 10.153200149536133, 10.170499801635742, 10.170499801635742, 10.181499481201172, 10.194900512695312, 10.23390007019043, 10.263200759887695, 10.263400077819824, 10.274101257324219, 10.274101257324219, 10.280399322509766, 10.337699890136719]</t>
+          <t>[8.237699508666992, 8.237699508666992, 8.237699508666992, 8.357200622558594, 8.41919994354248, 8.41919994354248, 8.792699813842773, 8.792699813842773, 9.292499542236328, 9.292499542236328, 9.292499542236328, 9.543498992919922, 9.567499160766602, 9.567499160766602, 9.843099594116211, 9.843099594116211, 9.843099594116211, 10.014799118041992, 10.014799118041992, 10.014799118041992, 10.074100494384766, 10.074100494384766, 10.174300193786621, 10.186500549316406, 10.186500549316406, 10.186500549316406, 10.186500549316406, 10.429999351501465, 10.429999351501465, 10.429999351501465, 10.429999351501465, 10.431400299072266, 10.986400604248047, 10.986400604248047, 10.986400604248047, 11.015600204467773, 11.034699440002441, 11.230500221252441, 11.230500221252441, 11.54580020904541, 11.54580020904541, 11.54580020904541, 11.54580020904541, 11.876699447631836, 11.876699447631836, 11.893799781799316, 12.018400192260742, 12.018400192260742, 12.0733003616333, 12.0733003616333, 12.177200317382812, 12.177200317382812, 12.177200317382812, 12.280500411987305, 12.328300476074219, 12.33899974822998, 12.33899974822998, 12.342599868774414, 12.469600677490234, 12.604599952697754, 12.604599952697754, 12.604599952697754, 12.780900001525879, 12.7829008102417, 12.7829008102417, 12.7829008102417, 12.984100341796875, 12.984100341796875, 13.053199768066406, 13.053199768066406, 13.060799598693848, 13.14739990234375, 13.14739990234375, 13.186698913574219, 13.186698913574219, 13.251899719238281, 13.251899719238281, 13.251899719238281, 13.252900123596191, 13.252900123596191, 13.499200820922852, 13.499200820922852, 13.499200820922852, 13.55270004272461, 13.55270004272461, 13.592300415039062, 13.596000671386719, 13.596000671386719, 13.596000671386719, 13.639400482177734, 13.666500091552734, 13.730500221252441, 13.776700019836426, 13.85460090637207, 13.85460090637207, 13.858099937438965, 13.858099937438965, 13.858099937438965, 13.858099937438965, 13.876701354980469, 13.9468994140625, 13.947800636291504, 13.965300559997559, 14.003999710083008, 14.091401100158691, 14.110000610351562, 14.121999740600586, 14.135100364685059, 14.217599868774414, 14.313699722290039, 14.313699722290039, 14.313699722290039, 14.32819938659668, 14.350800514221191, 14.364100456237793, 14.444700241088867, 14.478800773620605, 14.478800773620605, 14.496600151062012, 14.496600151062012, 14.657100677490234, 14.672500610351562, 14.672500610351562, 14.672500610351562, 14.721400260925293, 14.760601043701172, 14.767600059509277, 14.810400009155273, 14.826900482177734, 14.826900482177734, 14.838299751281738, 14.838299751281738, 14.851500511169434, 14.863500595092773, 14.87350082397461, 14.87350082397461, 14.892601013183594, 15.006799697875977, 15.006799697875977, 15.024399757385254, 15.024399757385254, 15.046100616455078, 15.133001327514648, 15.133001327514648, 15.140399932861328, 15.140399932861328, 15.143600463867188, 15.145899772644043, 15.145899772644043, 15.173199653625488, 15.180601119995117, 15.2322998046875, 15.248300552368164, 15.25059986114502, 15.25059986114502, 15.284000396728516, 15.33440113067627, 15.381200790405273, 15.398401260375977, 15.398401260375977, 15.398401260375977, 15.398401260375977, 15.434000015258789, 15.434000015258789, 15.44420051574707, 15.478700637817383, 15.499500274658203, 15.499500274658203, 15.499600410461426, 15.531499862670898, 15.531499862670898, 15.542400360107422, 15.55579948425293, 15.55579948425293, 15.557201385498047, 15.571300506591797, 15.571300506591797, 15.60680103302002, 15.60680103302002, 15.627399444580078, 15.627399444580078, 15.665600776672363, 15.69990062713623, 15.708200454711914, 15.728200912475586, 15.728200912475586, 15.729799270629883, 15.777800559997559, 15.777800559997559, 15.777800559997559, 15.777800559997559, 15.777800559997559, 15.780800819396973, 15.780800819396973, 15.811700820922852, 15.811700820922852, 15.850201606750488, 15.850201606750488, 15.854700088500977, 15.873100280761719, 15.873200416564941, 15.873200416564941, 15.873600006103516, 15.873600006103516, 15.873600006103516, 15.898399353027344, 15.898399353027344, 15.898399353027344, 15.898399353027344, 15.898399353027344, 15.915300369262695, 15.946499824523926, 15.946499824523926, 15.949400901794434, 16.004899978637695, 16.004899978637695, 16.006500244140625, 16.006500244140625, 16.00830078125, 16.0093994140625, 16.03660011291504, 16.03660011291504, 16.03660011291504, 16.04869842529297, 16.04869842529297, 16.056800842285156, 16.0635986328125, 16.0635986328125, 16.0635986328125, 16.06570053100586, 16.06570053100586, 16.082801818847656, 16.090099334716797, 16.090099334716797, 16.090099334716797, 16.139999389648438, 16.158802032470703, 16.158802032470703, 16.1924991607666, 16.1924991607666, 16.195899963378906, 16.239501953125, 16.239501953125, 16.24540138244629, 16.24540138244629, 16.271800994873047, 16.28270149230957, 16.28270149230957, 16.34309959411621, 16.346500396728516, 16.346500396728516, 16.388099670410156, 16.388099670410156, 16.388099670410156, 16.388099670410156, 16.388099670410156, 16.388099670410156, 16.39200210571289, 16.39200210571289, 16.447399139404297, 16.447399139404297, 16.447399139404297, 16.479900360107422, 16.479900360107422, 16.479900360107422, 16.511600494384766, 16.52280044555664, 16.535900115966797, 16.535900115966797, 16.549800872802734, 16.56290054321289, 16.56290054321289, 16.59440040588379, 16.59440040588379, 16.595300674438477, 16.595300674438477, 16.606399536132812, 16.633901596069336, 16.633901596069336, 16.643199920654297, 16.664199829101562, 16.664199829101562, 16.672401428222656, 16.69260025024414, 16.69260025024414, 16.69260025024414, 16.697601318359375, 16.697601318359375, 16.701801300048828, 16.731399536132812, 16.731399536132812, 16.736400604248047, 16.736400604248047, 16.736400604248047, 16.760299682617188, 16.780200958251953, 16.780200958251953, 16.780500411987305, 16.780500411987305, 16.835901260375977, 16.835901260375977, 16.835901260375977, 16.841999053955078, 16.841999053955078, 16.89150047302246, 16.89150047302246, 16.89150047302246, 16.89150047302246, 16.89150047302246, 16.906299591064453, 16.911300659179688, 16.914701461791992, 16.914701461791992, 17.052200317382812, 17.052200317382812, 17.052200317382812, 17.058700561523438, 17.05900001525879, 17.05900001525879, 17.05900001525879, 17.05900001525879, 17.071701049804688, 17.079700469970703, 17.110300064086914, 17.15380096435547, 17.192298889160156, 17.192298889160156, 17.192298889160156, 17.19260025024414, 17.19260025024414, 17.236499786376953, 17.291900634765625, 17.329200744628906, 17.343101501464844, 17.365800857543945, 17.365800857543945, 17.365800857543945, 17.368499755859375, 17.368499755859375, 17.420101165771484, 17.420101165771484, 17.430599212646484, 17.44610023498535, 17.44849967956543, 17.452301025390625, 17.452301025390625, 17.452600479125977, 17.452600479125977, 17.452600479125977, 17.452600479125977, 17.452600479125977, 17.452600479125977, 17.490001678466797, 17.490001678466797, 17.49919891357422, 17.506000518798828, 17.506000518798828, 17.514202117919922, 17.53569984436035, 17.55550193786621, 17.556901931762695, 17.556901931762695, 17.591800689697266, 17.591800689697266, 17.591800689697266, 17.625900268554688, 17.627700805664062, 17.633100509643555, 17.633100509643555, 17.65690040588379, 17.65690040588379, 17.65690040588379, 17.66230010986328, 17.66230010986328, 17.66230010986328, 17.663999557495117, 17.663999557495117, 17.663999557495117, 17.666000366210938, 17.667699813842773, 17.690399169921875, 17.690399169921875, 17.692100524902344, 17.692699432373047, 17.692699432373047, 17.702699661254883, 17.702699661254883, 17.70370101928711, 17.705402374267578, 17.707799911499023, 17.710201263427734, 17.811901092529297, 17.859500885009766, 17.859500885009766, 17.869300842285156, 17.913400650024414, 17.913400650024414, 17.92300033569336, 17.92300033569336, 17.92300033569336, 17.934600830078125, 17.934600830078125, 17.97100067138672, 17.973400115966797, 17.973400115966797, 17.973400115966797, 17.987499237060547, 17.987499237060547, 17.99020004272461, 17.99020004272461, 18.036800384521484, 18.042301177978516, 18.046300888061523, 18.052200317382812, 18.07390022277832, 18.07390022277832, 18.07390022277832, 18.07390022277832, 18.07390022277832, 18.074901580810547, 18.074901580810547, 18.074901580810547, 18.074901580810547, 18.076200485229492, 18.078899383544922, 18.10430145263672, 18.10430145263672, 18.108299255371094, 18.16119956970215, 18.16119956970215, 18.19580078125, 18.19580078125, 18.19580078125, 18.19580078125, 18.19580078125, 18.19580078125, 18.19580078125, 18.221099853515625, 18.234399795532227, 18.234399795532227, 18.234399795532227, 18.234399795532227, 18.247299194335938, 18.349300384521484, 18.349300384521484, 18.349899291992188, 18.349899291992188, 18.436199188232422, 18.464599609375, 18.464599609375, 18.48550033569336, 18.486801147460938, 18.489099502563477, 18.489099502563477, 18.489099502563477, 18.489099502563477, 18.489099502563477, 18.489500045776367, 18.512300491333008, 18.512300491333008, 18.526901245117188, 18.549400329589844, 18.549400329589844, 18.55729866027832, 18.577899932861328, 18.580299377441406, 18.582599639892578, 18.582599639892578, 18.61549949645996, 18.61549949645996, 18.627099990844727, 18.65610122680664, 18.65610122680664, 18.66809844970703, 18.66809844970703, 18.67169952392578, 18.67169952392578, 18.68120002746582, 18.68120002746582, 18.688199996948242, 18.742900848388672, 18.742900848388672, 18.828001022338867, 18.840599060058594, 18.840599060058594, 18.846399307250977, 18.850400924682617, 18.850400924682617, 18.850400924682617, 18.864500045776367, 18.892601013183594, 18.892601013183594, 18.892601013183594, 18.9424991607666, 18.9424991607666, 18.96739959716797, 19.032699584960938, 19.032699584960938, 19.060100555419922, 19.060100555419922, 19.060100555419922, 19.060100555419922, 19.063499450683594, 19.08370018005371, 19.08370018005371, 19.08370018005371, 19.08370018005371, 19.08370018005371, 19.08489990234375, 19.086898803710938, 19.121299743652344, 19.15169906616211, 19.15169906616211, 19.210599899291992, 19.210599899291992, 19.226299285888672, 19.229700088500977, 19.229700088500977, 19.229700088500977, 19.229700088500977, 19.229700088500977, 19.229700088500977, 19.229700088500977, 19.23110008239746, 19.23110008239746, 19.247398376464844, 19.25389862060547, 19.274799346923828, 19.274799346923828, 19.274799346923828, 19.274799346923828, 19.31679916381836, 19.317699432373047, 19.317699432373047, 19.31999969482422, 19.320899963378906, 19.34149932861328, 19.34149932861328, 19.34149932861328, 19.34149932861328, 19.34469985961914, 19.34469985961914, 19.34469985961914, 19.34469985961914, 19.34619903564453, 19.34910011291504, 19.389299392700195, 19.389299392700195, 19.389299392700195, 19.48550033569336, 19.48550033569336, 19.573501586914062, 19.573501586914062, 19.583900451660156, 19.583900451660156, 19.583900451660156, 19.602500915527344, 19.620498657226562, 19.63520050048828, 19.63520050048828, 19.677600860595703, 19.677600860595703, 19.677600860595703, 19.68800163269043, 19.69580078125, 19.69580078125, 19.69580078125, 19.69580078125, 19.699100494384766, 19.75629997253418, 19.75629997253418, 19.768199920654297, 19.768199920654297, 19.768199920654297, 19.768199920654297, 19.768199920654297, 19.768199920654297, 19.831199645996094, 19.831199645996094, 19.879199981689453, 19.8877010345459, 19.8877010345459, 19.90130043029785, 19.90130043029785, 19.90130043029785, 19.91230010986328, 19.91230010986328, 19.91230010986328, 19.91990089416504, 19.91990089416504, 19.92180061340332, 19.935100555419922, 19.935100555419922, 19.937000274658203, 19.937000274658203, 19.937000274658203, 19.977399826049805, 19.987499237060547, 20.02320098876953, 20.02770233154297, 20.02770233154297, 20.05769920349121, 20.05769920349121, 20.05769920349121, 20.061901092529297, 20.077999114990234, 20.105300903320312, 20.105300903320312, 20.151899337768555, 20.151899337768555, 20.193700790405273, 20.204898834228516, 20.204898834228516, 20.212299346923828, 20.243099212646484, 20.243099212646484, 20.243099212646484, 20.250499725341797, 20.260601043701172, 20.260601043701172, 20.270198822021484, 20.270198822021484, 20.270198822021484, 20.282400131225586, 20.3031005859375, 20.33340072631836, 20.33340072631836, 20.33340072631836, 20.366100311279297, 20.366100311279297, 20.37220001220703, 20.37220001220703, 20.378000259399414, 20.378000259399414, 20.400501251220703, 20.400501251220703, 20.406600952148438, 20.421100616455078, 20.421100616455078, 20.42650032043457, 20.42650032043457, 20.42650032043457, 20.427600860595703, 20.427600860595703, 20.427600860595703, 20.433000564575195, 20.504499435424805, 20.504499435424805, 20.509899139404297, 20.52359962463379, 20.524499893188477, 20.524499893188477, 20.524499893188477, 20.538999557495117, 20.555099487304688, 20.555099487304688, 20.595001220703125, 20.600399017333984, 20.601999282836914, 20.60580062866211, 20.60580062866211, 20.60580062866211, 20.60580062866211, 20.60580062866211, 20.60580062866211, 20.62700080871582, 20.62700080871582, 20.62700080871582, 20.62700080871582, 20.62700080871582, 20.62700080871582, 20.64820098876953, 20.655200958251953, 20.65679931640625, 20.663799285888672, 20.673398971557617, 20.688701629638672, 20.69409942626953, 20.69409942626953, 20.69409942626953, 20.69409942626953, 20.69409942626953, 20.69409942626953, 20.69409942626953, 20.702098846435547, 20.702098846435547, 20.702098846435547, 20.702098846435547, 20.702098846435547, 20.73069953918457, 20.757200241088867, 20.781400680541992, 20.783199310302734, 20.793701171875, 20.823299407958984, 20.823299407958984, 20.864200592041016, 20.864200592041016, 20.879798889160156, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.948200225830078, 20.948200225830078, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 21.1560001373291, 21.18090057373047, 21.18090057373047, 21.18090057373047, 21.205699920654297, 21.205699920654297, 21.205699920654297, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.22410011291504, 21.26110076904297, 21.26110076904297, 21.26110076904297, 21.332599639892578, 21.332599639892578, 21.373798370361328, 21.373798370361328, 21.37529945373535, 21.376998901367188, 21.376998901367188, 21.379499435424805, 21.386798858642578, 21.386798858642578, 21.388399124145508, 21.388399124145508, 21.388399124145508, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.440200805664062, 21.456600189208984, 21.456600189208984, 21.460800170898438, 21.460800170898438, 21.460800170898438, 21.460800170898438, 21.474599838256836, 21.47480010986328, 21.47480010986328, 21.48849868774414, 21.500999450683594, 21.500999450683594, 21.506799697875977, 21.506799697875977, 21.51099967956543, 21.512300491333008, 21.512300491333008, 21.512300491333008, 21.60270118713379, 21.603801727294922, 21.667999267578125, 21.667999267578125, 21.667999267578125, 21.680498123168945, 21.6846981048584, 21.6846981048584, 21.6846981048584, 21.6846981048584, 21.70319938659668, 21.708301544189453, 21.76650047302246, 21.783199310302734, 21.783199310302734, 21.783199310302734, 21.78369903564453, 21.789199829101562, 21.789199829101562, 21.789199829101562, 21.789199829101562, 21.789199829101562, 21.789199829101562, 21.799198150634766, 21.801700592041016, 21.801700592041016, 21.801700592041016, 21.807701110839844, 21.807701110839844, 21.81369972229004, 21.823898315429688, 21.823898315429688, 21.823898315429688, 21.823898315429688, 21.823898315429688, 21.823898315429688, 21.83839988708496, 21.83839988708496, 21.83839988708496, 21.83839988708496, 21.85580062866211, 21.85580062866211, 21.861799240112305, 21.861799240112305, 21.861799240112305, 21.864200592041016, 21.87769889831543, 21.88010025024414, 21.88010025024414, 21.89499855041504, 21.89499855041504, 21.89499855041504, 21.89499855041504, 21.89499855041504, 21.89499855041504, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.899301528930664, 21.90169906616211, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.927600860595703, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.983299255371094, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.988800048828125, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 22.071800231933594, 22.071800231933594, 22.071800231933594, 22.07509994506836, 22.07509994506836, 22.07509994506836, 22.07509994506836, 22.07509994506836, 22.13759994506836, 22.13759994506836, 22.13759994506836, 22.13759994506836, 22.13759994506836, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.16510009765625, 22.16510009765625, 22.16510009765625, 22.16510009765625, 22.16510009765625, 22.17259979248047, 22.17259979248047]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update the latest optimizer result
</commit_message>
<xml_diff>
--- a/results_fcgma/ResultsCompMethod.xlsx
+++ b/results_fcgma/ResultsCompMethod.xlsx
@@ -439,20 +439,20 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>[[0. 0. 0. ... 0. 0. 0.]
- [0. 0. 1. ... 0. 0. 0.]
+ [0. 1. 0. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]
  ...
  [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
+ [0. 0. 0. ... 0. 0. 1.]
  [0. 0. 0. ... 0. 0. 0.]]</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>44.91519927978516</v>
+        <v>50.2322998046875</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[25.464200973510742, 25.464200973510742, 25.48550033569336, 25.692399978637695, 26.002899169921875, 26.002899169921875, 26.133899688720703, 26.329498291015625, 26.329498291015625, 26.329498291015625, 26.329498291015625, 26.340301513671875, 26.42930030822754, 26.42930030822754, 26.42930030822754, 26.527301788330078, 26.684398651123047, 26.968299865722656, 26.968299865722656, 26.968299865722656, 26.968299865722656, 26.968299865722656, 27.01609992980957, 27.11050033569336, 27.454801559448242, 27.454801559448242, 27.454801559448242, 27.523601531982422, 27.541698455810547, 27.541698455810547, 27.541698455810547, 27.99880027770996, 27.99880027770996, 27.99880027770996, 27.99880027770996, 27.99880027770996, 28.095802307128906, 28.61240005493164, 28.61240005493164, 28.864700317382812, 28.864700317382812, 28.864700317382812, 28.864700317382812, 28.864700317382812, 29.00309944152832, 29.00309944152832, 29.00309944152832, 29.03839874267578, 29.484098434448242, 29.510799407958984, 29.510799407958984, 29.69499969482422, 29.69499969482422, 30.123199462890625, 30.123199462890625, 30.123199462890625, 30.123199462890625, 30.123199462890625, 30.448301315307617, 30.448301315307617, 30.448301315307617, 30.448301315307617, 30.448301315307617, 30.50040054321289, 30.519500732421875, 30.646800994873047, 30.646800994873047, 30.646800994873047, 30.830799102783203, 30.843399047851562, 30.98040008544922, 31.06570053100586, 31.068599700927734, 31.29800033569336, 31.29800033569336, 31.29800033569336, 31.29800033569336, 31.396800994873047, 31.6260986328125, 31.6260986328125, 31.6260986328125, 31.6260986328125, 31.66080093383789, 31.66080093383789, 31.66080093383789, 31.881099700927734, 31.881099700927734, 31.924701690673828, 31.924701690673828, 32.22740173339844, 32.22740173339844, 32.22740173339844, 32.33210372924805, 32.33210372924805, 32.3838996887207, 32.65229797363281, 32.65229797363281, 32.65229797363281, 32.704200744628906, 32.85499954223633, 32.85499954223633, 32.85499954223633, 32.85499954223633, 32.85499954223633, 32.86869812011719, 32.924800872802734, 32.924800872802734, 33.060001373291016, 33.07080078125, 33.07080078125, 33.131202697753906, 33.131202697753906, 33.131202697753906, 33.14140319824219, 33.23310089111328, 33.23310089111328, 33.23310089111328, 33.239402770996094, 33.2843017578125, 33.343299865722656, 33.344200134277344, 33.36119842529297, 33.39739990234375, 33.39739990234375, 33.39739990234375, 33.39739990234375, 33.39739990234375, 33.490997314453125, 33.490997314453125, 33.56209945678711, 33.582801818847656, 33.582801818847656, 33.707401275634766, 33.767398834228516, 33.767398834228516, 33.791900634765625, 33.791900634765625, 33.791900634765625, 33.84880065917969, 33.861900329589844, 33.861900329589844, 33.89649963378906, 33.89649963378906, 33.9276008605957, 33.9276008605957, 33.92770004272461, 33.92770004272461, 33.96500015258789, 33.96500015258789, 33.96500015258789, 33.970802307128906, 33.97169876098633, 33.971797943115234, 34.00080108642578, 34.03120040893555, 34.03120040893555, 34.06880187988281, 34.06880187988281, 34.07390213012695, 34.07390213012695, 34.07390213012695, 34.11159896850586, 34.17539978027344, 34.17539978027344, 34.17539978027344, 34.18450164794922, 34.19750213623047, 34.220001220703125, 34.246700286865234, 34.246700286865234, 34.25, 34.2776985168457, 34.2776985168457, 34.2776985168457, 34.32469940185547, 34.329200744628906, 34.342201232910156, 34.38159942626953, 34.38159942626953, 34.38159942626953, 34.38629913330078, 34.38629913330078, 34.41350173950195, 34.43219757080078, 34.43219757080078, 34.53300094604492, 34.53300094604492, 34.53300094604492, 34.63850021362305, 34.69490051269531, 34.72730255126953, 34.72730255126953, 34.72730255126953, 34.72730255126953, 34.72730255126953, 34.77429962158203, 34.80000305175781, 34.82429885864258, 34.8754997253418, 34.8754997253418, 34.8754997253418, 34.8754997253418, 34.87900161743164, 34.87900161743164, 34.88890075683594, 34.89350128173828, 34.90409851074219, 34.965599060058594, 34.965599060058594, 34.97480010986328, 34.97480010986328, 35.030601501464844, 35.030601501464844, 35.030601501464844, 35.030601501464844, 35.030601501464844, 35.04610061645508, 35.04610061645508, 35.085201263427734, 35.085201263427734, 35.08700180053711, 35.18010330200195, 35.18010330200195, 35.19499969482422, 35.19499969482422, 35.19499969482422, 35.26470184326172, 35.26470184326172, 35.26570129394531, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.36309814453125, 35.36309814453125, 35.44349670410156, 35.44349670410156, 35.46039581298828, 35.46039581298828, 35.55139923095703, 35.55139923095703, 35.56999969482422, 35.63290023803711, 35.71310043334961, 35.71310043334961, 35.7218017578125, 35.742000579833984, 35.742000579833984, 35.742000579833984, 35.804100036621094, 35.88420104980469, 35.88420104980469, 35.949798583984375, 35.949798583984375, 35.949798583984375, 35.949798583984375, 36.053199768066406, 36.055999755859375, 36.055999755859375, 36.057899475097656, 36.10230255126953, 36.10230255126953, 36.10309982299805, 36.10309982299805, 36.13140106201172, 36.13140106201172, 36.13140106201172, 36.192100524902344, 36.21150207519531, 36.21150207519531, 36.212799072265625, 36.212799072265625, 36.212799072265625, 36.22899627685547, 36.277400970458984, 36.332801818847656, 36.36069869995117, 36.417598724365234, 36.436302185058594, 36.456298828125, 36.456298828125, 36.475196838378906, 36.475196838378906, 36.48400115966797, 36.5432014465332, 36.57350158691406, 36.57350158691406, 36.57350158691406, 36.70030212402344, 36.70030212402344, 36.724098205566406, 36.724098205566406, 36.740501403808594, 36.78280258178711, 36.923500061035156, 36.923500061035156, 36.923500061035156, 36.923500061035156, 36.923500061035156, 36.93709945678711, 36.93709945678711, 36.95669937133789, 36.96580123901367, 37.01679992675781, 37.03689956665039, 37.03689956665039, 37.067298889160156, 37.067298889160156, 37.07109832763672, 37.07109832763672, 37.168399810791016, 37.28239822387695, 37.28239822387695, 37.31439971923828, 37.32460021972656, 37.32460021972656, 37.332801818847656, 37.352699279785156, 37.352699279785156, 37.4109992980957, 37.4109992980957, 37.414100646972656, 37.414100646972656, 37.430198669433594, 37.430198669433594, 37.53410339355469, 37.53410339355469, 37.53410339355469, 37.53410339355469, 37.545997619628906, 37.545997619628906, 37.55419921875, 37.60919952392578, 37.61830139160156, 37.61830139160156, 37.61830139160156, 37.75320053100586, 37.75320053100586, 37.764400482177734, 37.764400482177734, 37.76810073852539, 37.76810073852539, 37.76810073852539, 37.84770202636719, 37.84770202636719, 37.85680389404297, 37.85680389404297, 37.865901947021484, 37.88189697265625, 37.88189697265625, 37.88189697265625, 37.88189697265625, 37.89360046386719, 37.92140197753906, 37.92140197753906, 37.92140197753906, 37.94640350341797, 37.94640350341797, 37.94640350341797, 38.036598205566406, 38.036598205566406, 38.036598205566406, 38.04900360107422, 38.060997009277344, 38.060997009277344, 38.060997009277344, 38.060997009277344, 38.0697021484375, 38.07820129394531, 38.131500244140625, 38.131500244140625, 38.14550018310547, 38.18800354003906, 38.18800354003906, 38.229400634765625, 38.229400634765625, 38.233299255371094, 38.25600051879883, 38.321197509765625, 38.321197509765625, 38.32569885253906, 38.32569885253906, 38.32569885253906, 38.32889938354492, 38.342498779296875, 38.349403381347656, 38.35060119628906, 38.35060119628906, 38.38639831542969, 38.38639831542969, 38.38639831542969, 38.429901123046875, 38.429901123046875, 38.44499969482422, 38.46410369873047, 38.46410369873047, 38.47090148925781, 38.47169876098633, 38.49789810180664, 38.5796012878418, 38.5796012878418, 38.5796012878418, 38.59320068359375, 38.59320068359375, 38.62919998168945, 38.62919998168945, 38.641300201416016, 38.641300201416016, 38.641395568847656, 38.650901794433594, 38.650901794433594, 38.65570068359375, 38.67179870605469, 38.67179870605469, 38.67469787597656, 38.680198669433594, 38.680198669433594, 38.680198669433594, 38.69020080566406, 38.69020080566406, 38.70170211791992, 38.70439910888672, 38.70439910888672, 38.70439910888672, 38.70439910888672, 38.70680236816406, 38.712799072265625, 38.75559997558594, 38.768096923828125, 38.768096923828125, 38.7760009765625, 38.77870178222656, 38.78369903564453, 38.794097900390625, 38.799102783203125, 38.799102783203125, 38.84290313720703, 38.86250305175781, 38.86250305175781, 38.8754997253418, 38.897300720214844, 38.90769958496094, 38.90769958496094, 38.94029998779297, 38.94029998779297, 38.94029998779297, 38.95399856567383, 38.970401763916016, 38.970401763916016, 38.99089813232422, 38.995201110839844, 39.07680130004883, 39.07680130004883, 39.105098724365234, 39.1702995300293, 39.19049835205078, 39.19049835205078, 39.2317008972168, 39.2317008972168, 39.26620101928711, 39.26620101928711, 39.29500198364258, 39.38960266113281, 39.393402099609375, 39.416500091552734, 39.416500091552734, 39.43429946899414, 39.43429946899414, 39.466697692871094, 39.51319885253906, 39.51319885253906, 39.51319885253906, 39.546600341796875, 39.546600341796875, 39.546600341796875, 39.593299865722656, 39.60029983520508, 39.61429977416992, 39.61869812011719, 39.62220001220703, 39.651702880859375, 39.651702880859375, 39.651702880859375, 39.651702880859375, 39.66400146484375, 39.66400146484375, 39.67720031738281, 39.68949890136719, 39.70649719238281, 39.70649719238281, 39.70840072631836, 39.70840072631836, 39.728599548339844, 39.730499267578125, 39.745399475097656, 39.745399475097656, 39.75749969482422, 39.77619934082031, 39.77619934082031, 39.77619934082031, 39.77619934082031, 39.777400970458984, 39.777400970458984, 39.777400970458984, 39.82859802246094, 39.885501861572266, 39.92759704589844, 39.938697814941406, 39.938697814941406, 39.94159698486328, 39.95349884033203, 39.95349884033203, 39.98249816894531, 39.98249816894531, 39.9911994934082, 40.026798248291016, 40.026798248291016, 40.02799987792969, 40.09120178222656, 40.09120178222656, 40.11199951171875, 40.14720153808594, 40.15159606933594, 40.22330093383789, 40.22330093383789, 40.23259735107422, 40.23979949951172, 40.27179718017578, 40.31780242919922, 40.33830261230469, 40.36219787597656, 40.389400482177734, 40.389400482177734, 40.389400482177734, 40.399898529052734, 40.40549850463867, 40.40549850463867, 40.40549850463867, 40.40549850463867, 40.417198181152344, 40.417198181152344, 40.41780090332031, 40.48080062866211, 40.48080062866211, 40.48080062866211, 40.52330017089844, 40.54180145263672, 40.577301025390625, 40.577301025390625, 40.67359924316406, 40.67359924316406, 40.763099670410156, 40.763099670410156, 40.8302001953125, 40.840599060058594, 40.840599060058594, 40.84649658203125, 40.84870147705078, 40.84870147705078, 40.84880065917969, 40.84880065917969, 40.86479949951172, 40.86479949951172, 40.86479949951172, 40.87300109863281, 40.89820098876953, 40.907798767089844, 40.907798767089844, 40.91360092163086, 40.91360092163086, 40.91360092163086, 40.9911994934082, 41.02320098876953, 41.03010177612305, 41.03010177612305, 41.055599212646484, 41.075897216796875, 41.11070251464844, 41.11070251464844, 41.1151008605957, 41.139495849609375, 41.198299407958984, 41.198299407958984, 41.198299407958984, 41.198299407958984, 41.20880126953125, 41.20880126953125, 41.22269821166992, 41.23320007324219, 41.23320007324219, 41.23320007324219, 41.2411994934082, 41.25170135498047, 41.255897521972656, 41.27110290527344, 41.27110290527344, 41.275299072265625, 41.30970001220703, 41.30970001220703, 41.30970001220703, 41.30970001220703, 41.345699310302734, 41.345699310302734, 41.345699310302734, 41.345699310302734, 41.35890197753906, 41.3922004699707, 41.3922004699707, 41.40230178833008, 41.40230178833008, 41.40230178833008, 41.40230178833008, 41.415000915527344, 41.45110321044922, 41.455299377441406, 41.47739791870117, 41.47739791870117, 41.47739791870117, 41.50339889526367, 41.50339889526367, 41.50740051269531, 41.52149963378906, 41.548797607421875, 41.548797607421875, 41.548797607421875, 41.573402404785156, 41.573402404785156, 41.574501037597656, 41.574501037597656, 41.574501037597656, 41.63800048828125, 41.63909912109375, 41.64419937133789, 41.64419937133789, 41.65769958496094, 41.689998626708984, 41.689998626708984, 41.704795837402344, 41.704795837402344, 41.704795837402344, 41.704795837402344, 41.704795837402344, 41.71039962768555, 41.72220230102539, 41.72220230102539, 41.72620391845703, 41.73270034790039, 41.750099182128906, 41.750099182128906, 41.75830078125, 41.76319885253906, 41.77149963378906, 41.77149963378906, 41.77989959716797, 41.80889892578125, 41.80889892578125, 41.80889892578125, 41.80889892578125, 41.86119842529297, 41.86119842529297, 41.91320037841797, 41.91320037841797, 41.91320037841797, 41.96689987182617, 42.01020050048828, 42.01020050048828, 42.019100189208984, 42.03820037841797, 42.042999267578125, 42.042999267578125, 42.047096252441406, 42.047096252441406, 42.097801208496094, 42.15789794921875, 42.15789794921875, 42.16200256347656, 42.16239929199219, 42.19599914550781, 42.19599914550781, 42.199501037597656, 42.20490264892578, 42.230201721191406, 42.255699157714844, 42.27110290527344, 42.272300720214844, 42.272300720214844, 42.29460144042969, 42.29710006713867, 42.29869842529297, 42.29869842529297, 42.29869842529297, 42.329803466796875, 42.354000091552734, 42.35580062866211, 42.35580062866211, 42.358299255371094, 42.359901428222656, 42.36260223388672, 42.36920166015625, 42.38330078125, 42.38330078125, 42.38330078125, 42.479400634765625, 42.479400634765625, 42.48040008544922, 42.48040008544922, 42.48040008544922, 42.48040008544922, 42.49610137939453, 42.49610137939453, 42.49610137939453, 42.49610137939453, 42.54719924926758, 42.58489990234375, 42.589500427246094, 42.59280014038086, 42.59280014038086, 42.59280014038086, 42.59280014038086, 42.59830093383789, 42.601600646972656, 42.60969924926758, 42.60969924926758, 42.6254997253418, 42.6254997253418, 42.6525993347168, 42.6525993347168, 42.6525993347168, 42.65589904785156, 42.65589904785156, 42.65589904785156, 42.667198181152344, 42.667198181152344, 42.670501708984375, 42.670501708984375, 42.670501708984375, 42.68939971923828, 42.68939971923828, 42.69270324707031, 42.69770050048828, 42.69770050048828, 42.71800231933594, 42.71800231933594, 42.71800231933594, 42.71800231933594, 42.71800231933594, 42.7224006652832, 42.74030303955078, 42.74030303955078, 42.754798889160156, 42.76599884033203, 42.768699645996094, 42.768699645996094, 42.78209686279297, 42.78209686279297, 42.82019805908203, 42.82830047607422, 42.83899688720703, 42.83899688720703, 42.83899688720703, 42.83899688720703, 42.84579849243164, 42.84579849243164, 42.94269943237305, 42.94269943237305, 43.022499084472656, 43.022499084472656, 43.022499084472656, 43.121498107910156, 43.121498107910156, 43.121498107910156, 43.16780090332031, 43.16780090332031, 43.21119689941406, 43.213600158691406, 43.221099853515625, 43.221099853515625, 43.221099853515625, 43.22630310058594, 43.24259948730469, 43.25530242919922, 43.435298919677734, 43.435298919677734, 43.435298919677734, 43.435298919677734, 43.47869873046875, 43.47869873046875, 43.47869873046875, 43.47869873046875, 43.48759841918945, 43.525001525878906, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.588802337646484, 43.603302001953125, 43.603302001953125, 43.603302001953125, 43.603302001953125, 43.603302001953125, 43.633602142333984, 43.633602142333984, 43.640899658203125, 43.679298400878906, 43.697898864746094, 43.73100280761719, 43.73100280761719, 43.7318000793457, 43.77649688720703, 43.77649688720703, 43.77939987182617, 43.77939987182617, 43.77939987182617, 43.77939987182617, 43.82209777832031, 43.843502044677734, 43.843502044677734, 43.87670135498047, 43.87670135498047, 43.87839889526367, 43.950599670410156, 43.952301025390625, 44.037200927734375, 44.03950119018555, 44.103302001953125, 44.103302001953125, 44.1239013671875, 44.1239013671875, 44.16809844970703, 44.16809844970703, 44.183101654052734, 44.183101654052734, 44.186004638671875, 44.186004638671875, 44.206398010253906, 44.206398010253906, 44.24469757080078, 44.24869918823242, 44.24869918823242, 44.281002044677734, 44.333099365234375, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.35199737548828, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.37989807128906, 44.417198181152344, 44.417198181152344, 44.417198181152344, 44.418296813964844, 44.418296813964844, 44.418296813964844, 44.418296813964844, 44.418296813964844, 44.418800354003906, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45970153808594, 44.45970153808594, 44.45970153808594, 44.45970153808594, 44.49340057373047, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.52239990234375, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.53670120239258, 44.566898345947266, 44.566898345947266, 44.566898345947266, 44.566898345947266, 44.566898345947266, 44.57200241088867, 44.57200241088867, 44.57200241088867, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.85129928588867, 44.85129928588867, 44.85129928588867, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.86759948730469, 44.86759948730469, 44.87350082397461, 44.87350082397461, 44.87350082397461, 44.87350082397461, 44.915199279785156, 44.915199279785156, 44.915199279785156, 44.915199279785156]</t>
+          <t>[31.35190200805664, 31.523000717163086, 31.523000717163086, 31.590299606323242, 31.590299606323242, 31.590299606323242, 31.590299606323242, 31.590299606323242, 31.69900131225586, 31.743301391601562, 31.91230010986328, 31.91230010986328, 32.05059814453125, 32.05059814453125, 32.05059814453125, 32.07429885864258, 32.43190002441406, 32.43190002441406, 32.65800094604492, 32.65800094604492, 32.65800094604492, 32.65800094604492, 32.65800094604492, 32.65800094604492, 32.9911994934082, 32.9911994934082, 32.9911994934082, 32.9911994934082, 33.067100524902344, 33.22169876098633, 33.324100494384766, 33.324100494384766, 33.77360153198242, 33.77360153198242, 33.77360153198242, 33.77360153198242, 34.15019989013672, 34.15019989013672, 34.15019989013672, 34.15019989013672, 34.17959976196289, 34.26020050048828, 34.26020050048828, 34.277801513671875, 34.277801513671875, 34.277801513671875, 34.277801513671875, 34.277801513671875, 34.277801513671875, 34.368900299072266, 34.368900299072266, 34.41830062866211, 34.41830062866211, 34.41830062866211, 34.63859939575195, 34.63859939575195, 34.63859939575195, 34.63859939575195, 34.74869918823242, 34.74869918823242, 34.77300262451172, 34.83829879760742, 34.98919677734375, 35.0077018737793, 35.212501525878906, 35.37969970703125, 35.37969970703125, 35.37969970703125, 35.37969970703125, 35.37969970703125, 35.631195068359375, 35.95269775390625, 35.97610092163086, 35.97610092163086, 36.448299407958984, 36.448299407958984, 36.448299407958984, 36.62730026245117, 36.62730026245117, 36.62730026245117, 36.783599853515625, 36.78770065307617, 36.84379959106445, 36.84379959106445, 37.00160217285156, 37.00160217285156, 37.00160217285156, 37.146400451660156, 37.146400451660156, 37.146400451660156, 37.146400451660156, 37.22249984741211, 37.320396423339844, 37.320396423339844, 37.66709899902344, 37.66709899902344, 37.74639892578125, 37.849098205566406, 37.849098205566406, 37.85980224609375, 37.85980224609375, 38.065399169921875, 38.065399169921875, 38.065399169921875, 38.20459747314453, 38.28139877319336, 38.28139877319336, 38.40449905395508, 38.40449905395508, 38.437198638916016, 38.437198638916016, 38.641300201416016, 38.641300201416016, 38.73820114135742, 38.73820114135742, 38.73820114135742, 38.819801330566406, 38.927001953125, 38.93220138549805, 38.93220138549805, 38.93260192871094, 39.14699935913086, 39.14699935913086, 39.14699935913086, 39.253997802734375, 39.26070022583008, 39.26070022583008, 39.310203552246094, 39.341697692871094, 39.36650085449219, 39.36650085449219, 39.370399475097656, 39.370399475097656, 39.37879943847656, 39.49690246582031, 39.49690246582031, 39.529701232910156, 39.529701232910156, 39.529701232910156, 39.529701232910156, 39.529701232910156, 39.54290008544922, 39.55950164794922, 39.63459777832031, 39.658302307128906, 39.658302307128906, 39.683998107910156, 39.683998107910156, 39.70289993286133, 39.72529983520508, 39.72529983520508, 39.7598991394043, 39.873802185058594, 39.873802185058594, 39.873802185058594, 39.95829772949219, 39.95829772949219, 39.95829772949219, 39.965797424316406, 40.007999420166016, 40.007999420166016, 40.00979995727539, 40.01799774169922, 40.10960006713867, 40.156097412109375, 40.229000091552734, 40.229000091552734, 40.264503479003906, 40.264503479003906, 40.280799865722656, 40.35710144042969, 40.35710144042969, 40.42190170288086, 40.438899993896484, 40.438899993896484, 40.45790100097656, 40.472900390625, 40.472900390625, 40.617496490478516, 40.617496490478516, 40.617496490478516, 40.617496490478516, 40.68770217895508, 40.73379898071289, 40.73379898071289, 40.73379898071289, 40.790802001953125, 40.790802001953125, 40.81739807128906, 40.81739807128906, 40.819000244140625, 41.01259994506836, 41.01259994506836, 41.01259994506836, 41.01259994506836, 41.04820251464844, 41.05229949951172, 41.06310272216797, 41.08619689941406, 41.122802734375, 41.193599700927734, 41.208900451660156, 41.27210235595703, 41.36050033569336, 41.36050033569336, 41.387298583984375, 41.387298583984375, 41.387298583984375, 41.387298583984375, 41.387298583984375, 41.403099060058594, 41.403099060058594, 41.46659851074219, 41.46659851074219, 41.524200439453125, 41.524200439453125, 41.524200439453125, 41.64699935913086, 41.64699935913086, 41.64699935913086, 41.64699935913086, 41.64699935913086, 41.65639877319336, 41.69219970703125, 41.70909881591797, 41.70909881591797, 41.75910186767578, 41.75910186767578, 41.777000427246094, 41.822998046875, 41.822998046875, 41.82400131225586, 41.871002197265625, 41.92790222167969, 41.92790222167969, 41.939598083496094, 41.95130157470703, 41.95130157470703, 41.993099212646484, 41.993099212646484, 42.023399353027344, 42.04170227050781, 42.04170227050781, 42.04240036010742, 42.04240036010742, 42.08439636230469, 42.10540008544922, 42.11840057373047, 42.11840057373047, 42.18009948730469, 42.18009948730469, 42.18009948730469, 42.25330352783203, 42.26129913330078, 42.315399169921875, 42.33300018310547, 42.33300018310547, 42.333702087402344, 42.333702087402344, 42.33440399169922, 42.34280014038086, 42.34280014038086, 42.36689758300781, 42.40599822998047, 42.40599822998047, 42.40599822998047, 42.447601318359375, 42.447601318359375, 42.447601318359375, 42.450599670410156, 42.50619888305664, 42.50619888305664, 42.509498596191406, 42.51519775390625, 42.567100524902344, 42.567100524902344, 42.567100524902344, 42.567100524902344, 42.57019805908203, 42.57019805908203, 42.617000579833984, 42.617000579833984, 42.617000579833984, 42.634498596191406, 42.63669967651367, 42.63669967651367, 42.64240264892578, 42.658302307128906, 42.67359924316406, 42.67490005493164, 42.733699798583984, 42.733699798583984, 42.74899673461914, 42.75029754638672, 42.796302795410156, 42.82170104980469, 42.82170104980469, 42.82170104980469, 42.84389877319336, 42.84389877319336, 42.855499267578125, 42.92900085449219, 42.98680114746094, 43.10700225830078, 43.10700225830078, 43.10700225830078, 43.12879943847656, 43.12879943847656, 43.13710021972656, 43.17420196533203, 43.17420196533203, 43.220001220703125, 43.259803771972656, 43.259803771972656, 43.259803771972656, 43.264102935791016, 43.291297912597656, 43.291297912597656, 43.34020233154297, 43.4098014831543, 43.44519805908203, 43.523399353027344, 43.53940200805664, 43.53940200805664, 43.61399841308594, 43.642799377441406, 43.642799377441406, 43.659996032714844, 43.69129943847656, 43.72079849243164, 43.75969696044922, 43.75969696044922, 43.76570129394531, 43.76570129394531, 43.774200439453125, 43.82630157470703, 43.82630157470703, 43.83140182495117, 43.87419891357422, 43.87419891357422, 43.91510009765625, 43.91659927368164, 43.91659927368164, 43.939697265625, 43.939697265625, 43.960899353027344, 43.960899353027344, 44.001800537109375, 44.001800537109375, 44.010799407958984, 44.010799407958984, 44.0192985534668, 44.021400451660156, 44.021400451660156, 44.03179931640625, 44.03179931640625, 44.10559844970703, 44.10559844970703, 44.106903076171875, 44.139198303222656, 44.16960144042969, 44.17749786376953, 44.19929885864258, 44.20030212402344, 44.20030212402344, 44.21209716796875, 44.23870086669922, 44.23870086669922, 44.23870086669922, 44.23870086669922, 44.25309753417969, 44.25309753417969, 44.370399475097656, 44.370399475097656, 44.39099884033203, 44.39099884033203, 44.3922004699707, 44.41379928588867, 44.41659927368164, 44.42150115966797, 44.42759704589844, 44.43790054321289, 44.43790054321289, 44.441200256347656, 44.441200256347656, 44.481300354003906, 44.486202239990234, 44.486202239990234, 44.486202239990234, 44.557899475097656, 44.557899475097656, 44.574501037597656, 44.62940216064453, 44.62940216064453, 44.6510009765625, 44.6510009765625, 44.654197692871094, 44.654197692871094, 44.654197692871094, 44.654197692871094, 44.654197692871094, 44.73040008544922, 44.73040008544922, 44.75790023803711, 44.784202575683594, 44.820098876953125, 44.820098876953125, 44.877201080322266, 44.877201080322266, 44.877201080322266, 44.91510009765625, 44.9552001953125, 44.9552001953125, 44.995201110839844, 44.99800109863281, 44.99800109863281, 45.00870132446289, 45.036903381347656, 45.04629898071289, 45.04629898071289, 45.07569885253906, 45.07569885253906, 45.07740020751953, 45.100799560546875, 45.100799560546875, 45.12969970703125, 45.13800048828125, 45.13800048828125, 45.13800048828125, 45.13800048828125, 45.13800048828125, 45.14830017089844, 45.14830017089844, 45.16059875488281, 45.16059875488281, 45.161800384521484, 45.19169998168945, 45.19169998168945, 45.19839859008789, 45.19839859008789, 45.19839859008789, 45.212501525878906, 45.235496520996094, 45.235496520996094, 45.23860168457031, 45.250099182128906, 45.256099700927734, 45.263099670410156, 45.263099670410156, 45.32630157470703, 45.32630157470703, 45.32630157470703, 45.35820007324219, 45.41619873046875, 45.41619873046875, 45.41619873046875, 45.430301666259766, 45.430301666259766, 45.430301666259766, 45.442501068115234, 45.50360107421875, 45.518001556396484, 45.54719924926758, 45.54719924926758, 45.57209777832031, 45.57209777832031, 45.575199127197266, 45.597999572753906, 45.597999572753906, 45.597999572753906, 45.60110092163086, 45.63140106201172, 45.634700775146484, 45.65019989013672, 45.65019989013672, 45.68370056152344, 45.694698333740234, 45.694698333740234, 45.70539855957031, 45.70539855957031, 45.75309753417969, 45.78730010986328, 45.79669952392578, 45.8031005859375, 45.831398010253906, 45.831398010253906, 45.86940002441406, 45.896202087402344, 45.896202087402344, 45.896202087402344, 45.9176025390625, 45.9176025390625, 45.97840118408203, 45.97840118408203, 45.97840118408203, 45.994197845458984, 46.024200439453125, 46.024200439453125, 46.024200439453125, 46.03030014038086, 46.03030014038086, 46.03030014038086, 46.03209686279297, 46.03209686279297, 46.035301208496094, 46.035301208496094, 46.03879928588867, 46.03879928588867, 46.03879928588867, 46.03879928588867, 46.03879928588867, 46.03879928588867, 46.09819793701172, 46.099700927734375, 46.10639953613281, 46.13850021362305, 46.13909912109375, 46.13909912109375, 46.13909912109375, 46.14950180053711, 46.17829895019531, 46.246498107910156, 46.246498107910156, 46.29629898071289, 46.301795959472656, 46.301795959472656, 46.301795959472656, 46.33940124511719, 46.33940124511719, 46.35169982910156, 46.39540100097656, 46.39820098876953, 46.39820098876953, 46.42259979248047, 46.442298889160156, 46.442298889160156, 46.44300079345703, 46.44300079345703, 46.44300079345703, 46.44300079345703, 46.458499908447266, 46.458499908447266, 46.45909881591797, 46.588600158691406, 46.634700775146484, 46.64630126953125, 46.64970016479492, 46.64970016479492, 46.69350051879883, 46.69350051879883, 46.69350051879883, 46.69350051879883, 46.69350051879883, 46.70750045776367, 46.72270202636719, 46.726600646972656, 46.72669982910156, 46.7572021484375, 46.7572021484375, 46.76380157470703, 46.80329895019531, 46.80329895019531, 46.80329895019531, 46.80329895019531, 46.80329895019531, 46.80329895019531, 46.83830261230469, 46.83830261230469, 46.84170150756836, 46.86830139160156, 46.90620040893555, 46.98149871826172, 46.98149871826172, 47.016300201416016, 47.016300201416016, 47.016300201416016, 47.01930236816406, 47.027400970458984, 47.037200927734375, 47.037200927734375, 47.04139709472656, 47.05120086669922, 47.05120086669922, 47.05120086669922, 47.05120086669922, 47.06949996948242, 47.06949996948242, 47.147098541259766, 47.149200439453125, 47.3140983581543, 47.3140983581543, 47.318397521972656, 47.32849884033203, 47.34700012207031, 47.34700012207031, 47.34700012207031, 47.34700012207031, 47.354698181152344, 47.39120101928711, 47.39120101928711, 47.394500732421875, 47.4468994140625, 47.48179626464844, 47.48179626464844, 47.48179626464844, 47.50640106201172, 47.50640106201172, 47.51900100708008, 47.560699462890625, 47.560699462890625, 47.56420135498047, 47.586700439453125, 47.586700439453125, 47.589996337890625, 47.594398498535156, 47.594398498535156, 47.594398498535156, 47.65839767456055, 47.715301513671875, 47.74340057373047, 47.74340057373047, 47.746700286865234, 47.746700286865234, 47.77090072631836, 47.78369903564453, 47.78369903564453, 47.8135986328125, 47.827598571777344, 47.827598571777344, 47.830902099609375, 47.830902099609375, 47.84619903564453, 47.84619903564453, 47.84769821166992, 47.8494987487793, 47.855499267578125, 47.87459945678711, 47.87459945678711, 47.87459945678711, 47.886802673339844, 47.90769958496094, 47.90769958496094, 47.90769958496094, 47.91699981689453, 47.91699981689453, 47.920501708984375, 47.920501708984375, 47.948299407958984, 47.948299407958984, 47.948299407958984, 48.06120300292969, 48.06120300292969, 48.0869026184082, 48.0869026184082, 48.117698669433594, 48.12580108642578, 48.1525993347168, 48.1781005859375, 48.1781005859375, 48.23699951171875, 48.23699951171875, 48.29909896850586, 48.320098876953125, 48.320098876953125, 48.320098876953125, 48.32939910888672, 48.33290100097656, 48.37739944458008, 48.38209915161133, 48.3916015625, 48.39509963989258, 48.39509963989258, 48.39509963989258, 48.41189956665039, 48.427799224853516, 48.458099365234375, 48.458099365234375, 48.458099365234375, 48.47229766845703, 48.49120330810547, 48.492698669433594, 48.492698669433594, 48.49850082397461, 48.5098991394043, 48.530799865722656, 48.532901763916016, 48.532901763916016, 48.54560089111328, 48.54560089111328, 48.54560089111328, 48.54560089111328, 48.54560089111328, 48.555198669433594, 48.555198669433594, 48.555198669433594, 48.555198669433594, 48.566497802734375, 48.57609939575195, 48.59600067138672, 48.59600067138672, 48.655399322509766, 48.655399322509766, 48.683799743652344, 48.683799743652344, 48.683799743652344, 48.683799743652344, 48.683799743652344, 48.75490188598633, 48.756797790527344, 48.79520034790039, 48.79520034790039, 48.79520034790039, 48.811500549316406, 48.820701599121094, 48.820701599121094, 48.84459686279297, 48.84459686279297, 48.84459686279297, 48.871803283691406, 48.893402099609375, 48.907501220703125, 48.94129943847656, 48.94129943847656, 48.943599700927734, 48.94439697265625, 48.94439697265625, 48.94439697265625, 48.94670104980469, 49.02360153198242, 49.02360153198242, 49.09040069580078, 49.09040069580078, 49.09040069580078, 49.099300384521484, 49.1056022644043, 49.1056022644043, 49.1056022644043, 49.1056022644043, 49.1056022644043, 49.1255989074707, 49.1255989074707, 49.1255989074707, 49.14240264892578, 49.14240264892578, 49.19490051269531, 49.19490051269531, 49.19490051269531, 49.23500061035156, 49.23500061035156, 49.23500061035156, 49.23500061035156, 49.23500061035156, 49.26179885864258, 49.28280258178711, 49.3291015625, 49.331199645996094, 49.39209747314453, 49.39209747314453, 49.417999267578125, 49.42040252685547, 49.42040252685547, 49.44860076904297, 49.450897216796875, 49.450897216796875, 49.450897216796875, 49.480098724365234, 49.480098724365234, 49.480098724365234, 49.50619888305664, 49.50849914550781, 49.50849914550781, 49.50849914550781, 49.50849914550781, 49.50849914550781, 49.529998779296875, 49.529998779296875, 49.529998779296875, 49.55609893798828, 49.55609893798828, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.623600006103516, 49.623600006103516, 49.623600006103516, 49.62730026245117, 49.62730026245117, 49.62730026245117, 49.689701080322266, 49.689701080322266, 49.69340133666992, 49.69770050048828, 49.7150993347168, 49.75140380859375, 49.78499984741211, 49.78499984741211, 49.831398010253906, 49.85869598388672, 49.85960006713867, 49.86499786376953, 49.86989974975586, 49.86989974975586, 49.86989974975586, 49.8948974609375, 49.8948974609375, 49.902099609375, 49.90370178222656, 49.90370178222656, 49.90370178222656, 49.90370178222656, 49.90370178222656, 49.90580368041992, 49.90739822387695, 49.913299560546875, 49.913299560546875, 49.919097900390625, 49.92449951171875, 49.92449951171875, 49.93890380859375, 49.93890380859375, 49.93890380859375, 49.94070053100586, 49.942298889160156, 50.00749969482422, 50.00749969482422, 50.00749969482422, 50.01900100708008, 50.01900100708008, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.03179931640625, 50.03179931640625, 50.03179931640625, 50.03179931640625, 50.03179931640625, 50.03179931640625, 50.03179931640625, 50.033599853515625, 50.0697021484375, 50.0697021484375, 50.0697021484375, 50.0697021484375, 50.0697021484375, 50.0697021484375, 50.0697021484375, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11669921875, 50.11669921875, 50.11669921875, 50.11869812011719, 50.11869812011719, 50.11869812011719, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13209915161133, 50.18080139160156, 50.18080139160156, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Change this repo into full post-T paralell runs
</commit_message>
<xml_diff>
--- a/results_fcgma/ResultsCompMethod.xlsx
+++ b/results_fcgma/ResultsCompMethod.xlsx
@@ -439,7 +439,7 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>[[0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
+ [0. 0. 1. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]
  ...
  [0. 0. 0. ... 0. 0. 0.]
@@ -448,11 +448,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.33769989013672</v>
+        <v>44.91519927978516</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[6.964300155639648, 6.971400260925293, 7.488400459289551, 7.488400459289551, 7.488400459289551, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.634200096130371, 7.635500431060791, 7.635500431060791, 7.683699607849121, 7.683699607849121, 7.683699607849121, 7.683699607849121, 8.038800239562988, 8.038800239562988, 8.086099624633789, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.277400016784668, 8.526300430297852, 8.526300430297852, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.528800010681152, 8.724699974060059, 8.724699974060059, 8.724699974060059, 8.724699974060059, 8.846700668334961, 8.846700668334961, 8.847900390625, 8.847900390625, 8.939499855041504, 8.957099914550781, 8.9822998046875, 8.9822998046875, 8.9822998046875, 9.024499893188477, 9.047100067138672, 9.047100067138672, 9.122400283813477, 9.122400283813477, 9.122400283813477, 9.14739990234375, 9.14739990234375, 9.163100242614746, 9.170499801635742, 9.17609977722168, 9.217399597167969, 9.363900184631348, 9.363900184631348, 9.363900184631348, 9.406400680541992, 9.443599700927734, 9.443599700927734, 9.463900566101074, 9.463900566101074, 9.50100040435791, 9.54010009765625, 9.651800155639648, 9.67449951171875, 9.67449951171875, 9.791799545288086, 9.801000595092773, 9.801000595092773, 9.828399658203125, 9.828399658203125, 9.895099639892578, 9.910400390625, 9.910400390625, 9.910900115966797, 9.911800384521484, 10.04740047454834, 10.04740047454834, 10.064599990844727, 10.064599990844727, 10.064599990844727, 10.146900177001953, 10.146900177001953, 10.153200149536133, 10.170499801635742, 10.170499801635742, 10.181499481201172, 10.194900512695312, 10.23390007019043, 10.263200759887695, 10.263400077819824, 10.274101257324219, 10.274101257324219, 10.280399322509766, 10.337699890136719]</t>
+          <t>[25.464200973510742, 25.464200973510742, 25.48550033569336, 25.692399978637695, 26.002899169921875, 26.002899169921875, 26.133899688720703, 26.329498291015625, 26.329498291015625, 26.329498291015625, 26.329498291015625, 26.340301513671875, 26.42930030822754, 26.42930030822754, 26.42930030822754, 26.527301788330078, 26.684398651123047, 26.968299865722656, 26.968299865722656, 26.968299865722656, 26.968299865722656, 26.968299865722656, 27.01609992980957, 27.11050033569336, 27.454801559448242, 27.454801559448242, 27.454801559448242, 27.523601531982422, 27.541698455810547, 27.541698455810547, 27.541698455810547, 27.99880027770996, 27.99880027770996, 27.99880027770996, 27.99880027770996, 27.99880027770996, 28.095802307128906, 28.61240005493164, 28.61240005493164, 28.864700317382812, 28.864700317382812, 28.864700317382812, 28.864700317382812, 28.864700317382812, 29.00309944152832, 29.00309944152832, 29.00309944152832, 29.03839874267578, 29.484098434448242, 29.510799407958984, 29.510799407958984, 29.69499969482422, 29.69499969482422, 30.123199462890625, 30.123199462890625, 30.123199462890625, 30.123199462890625, 30.123199462890625, 30.448301315307617, 30.448301315307617, 30.448301315307617, 30.448301315307617, 30.448301315307617, 30.50040054321289, 30.519500732421875, 30.646800994873047, 30.646800994873047, 30.646800994873047, 30.830799102783203, 30.843399047851562, 30.98040008544922, 31.06570053100586, 31.068599700927734, 31.29800033569336, 31.29800033569336, 31.29800033569336, 31.29800033569336, 31.396800994873047, 31.6260986328125, 31.6260986328125, 31.6260986328125, 31.6260986328125, 31.66080093383789, 31.66080093383789, 31.66080093383789, 31.881099700927734, 31.881099700927734, 31.924701690673828, 31.924701690673828, 32.22740173339844, 32.22740173339844, 32.22740173339844, 32.33210372924805, 32.33210372924805, 32.3838996887207, 32.65229797363281, 32.65229797363281, 32.65229797363281, 32.704200744628906, 32.85499954223633, 32.85499954223633, 32.85499954223633, 32.85499954223633, 32.85499954223633, 32.86869812011719, 32.924800872802734, 32.924800872802734, 33.060001373291016, 33.07080078125, 33.07080078125, 33.131202697753906, 33.131202697753906, 33.131202697753906, 33.14140319824219, 33.23310089111328, 33.23310089111328, 33.23310089111328, 33.239402770996094, 33.2843017578125, 33.343299865722656, 33.344200134277344, 33.36119842529297, 33.39739990234375, 33.39739990234375, 33.39739990234375, 33.39739990234375, 33.39739990234375, 33.490997314453125, 33.490997314453125, 33.56209945678711, 33.582801818847656, 33.582801818847656, 33.707401275634766, 33.767398834228516, 33.767398834228516, 33.791900634765625, 33.791900634765625, 33.791900634765625, 33.84880065917969, 33.861900329589844, 33.861900329589844, 33.89649963378906, 33.89649963378906, 33.9276008605957, 33.9276008605957, 33.92770004272461, 33.92770004272461, 33.96500015258789, 33.96500015258789, 33.96500015258789, 33.970802307128906, 33.97169876098633, 33.971797943115234, 34.00080108642578, 34.03120040893555, 34.03120040893555, 34.06880187988281, 34.06880187988281, 34.07390213012695, 34.07390213012695, 34.07390213012695, 34.11159896850586, 34.17539978027344, 34.17539978027344, 34.17539978027344, 34.18450164794922, 34.19750213623047, 34.220001220703125, 34.246700286865234, 34.246700286865234, 34.25, 34.2776985168457, 34.2776985168457, 34.2776985168457, 34.32469940185547, 34.329200744628906, 34.342201232910156, 34.38159942626953, 34.38159942626953, 34.38159942626953, 34.38629913330078, 34.38629913330078, 34.41350173950195, 34.43219757080078, 34.43219757080078, 34.53300094604492, 34.53300094604492, 34.53300094604492, 34.63850021362305, 34.69490051269531, 34.72730255126953, 34.72730255126953, 34.72730255126953, 34.72730255126953, 34.72730255126953, 34.77429962158203, 34.80000305175781, 34.82429885864258, 34.8754997253418, 34.8754997253418, 34.8754997253418, 34.8754997253418, 34.87900161743164, 34.87900161743164, 34.88890075683594, 34.89350128173828, 34.90409851074219, 34.965599060058594, 34.965599060058594, 34.97480010986328, 34.97480010986328, 35.030601501464844, 35.030601501464844, 35.030601501464844, 35.030601501464844, 35.030601501464844, 35.04610061645508, 35.04610061645508, 35.085201263427734, 35.085201263427734, 35.08700180053711, 35.18010330200195, 35.18010330200195, 35.19499969482422, 35.19499969482422, 35.19499969482422, 35.26470184326172, 35.26470184326172, 35.26570129394531, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.342002868652344, 35.36309814453125, 35.36309814453125, 35.44349670410156, 35.44349670410156, 35.46039581298828, 35.46039581298828, 35.55139923095703, 35.55139923095703, 35.56999969482422, 35.63290023803711, 35.71310043334961, 35.71310043334961, 35.7218017578125, 35.742000579833984, 35.742000579833984, 35.742000579833984, 35.804100036621094, 35.88420104980469, 35.88420104980469, 35.949798583984375, 35.949798583984375, 35.949798583984375, 35.949798583984375, 36.053199768066406, 36.055999755859375, 36.055999755859375, 36.057899475097656, 36.10230255126953, 36.10230255126953, 36.10309982299805, 36.10309982299805, 36.13140106201172, 36.13140106201172, 36.13140106201172, 36.192100524902344, 36.21150207519531, 36.21150207519531, 36.212799072265625, 36.212799072265625, 36.212799072265625, 36.22899627685547, 36.277400970458984, 36.332801818847656, 36.36069869995117, 36.417598724365234, 36.436302185058594, 36.456298828125, 36.456298828125, 36.475196838378906, 36.475196838378906, 36.48400115966797, 36.5432014465332, 36.57350158691406, 36.57350158691406, 36.57350158691406, 36.70030212402344, 36.70030212402344, 36.724098205566406, 36.724098205566406, 36.740501403808594, 36.78280258178711, 36.923500061035156, 36.923500061035156, 36.923500061035156, 36.923500061035156, 36.923500061035156, 36.93709945678711, 36.93709945678711, 36.95669937133789, 36.96580123901367, 37.01679992675781, 37.03689956665039, 37.03689956665039, 37.067298889160156, 37.067298889160156, 37.07109832763672, 37.07109832763672, 37.168399810791016, 37.28239822387695, 37.28239822387695, 37.31439971923828, 37.32460021972656, 37.32460021972656, 37.332801818847656, 37.352699279785156, 37.352699279785156, 37.4109992980957, 37.4109992980957, 37.414100646972656, 37.414100646972656, 37.430198669433594, 37.430198669433594, 37.53410339355469, 37.53410339355469, 37.53410339355469, 37.53410339355469, 37.545997619628906, 37.545997619628906, 37.55419921875, 37.60919952392578, 37.61830139160156, 37.61830139160156, 37.61830139160156, 37.75320053100586, 37.75320053100586, 37.764400482177734, 37.764400482177734, 37.76810073852539, 37.76810073852539, 37.76810073852539, 37.84770202636719, 37.84770202636719, 37.85680389404297, 37.85680389404297, 37.865901947021484, 37.88189697265625, 37.88189697265625, 37.88189697265625, 37.88189697265625, 37.89360046386719, 37.92140197753906, 37.92140197753906, 37.92140197753906, 37.94640350341797, 37.94640350341797, 37.94640350341797, 38.036598205566406, 38.036598205566406, 38.036598205566406, 38.04900360107422, 38.060997009277344, 38.060997009277344, 38.060997009277344, 38.060997009277344, 38.0697021484375, 38.07820129394531, 38.131500244140625, 38.131500244140625, 38.14550018310547, 38.18800354003906, 38.18800354003906, 38.229400634765625, 38.229400634765625, 38.233299255371094, 38.25600051879883, 38.321197509765625, 38.321197509765625, 38.32569885253906, 38.32569885253906, 38.32569885253906, 38.32889938354492, 38.342498779296875, 38.349403381347656, 38.35060119628906, 38.35060119628906, 38.38639831542969, 38.38639831542969, 38.38639831542969, 38.429901123046875, 38.429901123046875, 38.44499969482422, 38.46410369873047, 38.46410369873047, 38.47090148925781, 38.47169876098633, 38.49789810180664, 38.5796012878418, 38.5796012878418, 38.5796012878418, 38.59320068359375, 38.59320068359375, 38.62919998168945, 38.62919998168945, 38.641300201416016, 38.641300201416016, 38.641395568847656, 38.650901794433594, 38.650901794433594, 38.65570068359375, 38.67179870605469, 38.67179870605469, 38.67469787597656, 38.680198669433594, 38.680198669433594, 38.680198669433594, 38.69020080566406, 38.69020080566406, 38.70170211791992, 38.70439910888672, 38.70439910888672, 38.70439910888672, 38.70439910888672, 38.70680236816406, 38.712799072265625, 38.75559997558594, 38.768096923828125, 38.768096923828125, 38.7760009765625, 38.77870178222656, 38.78369903564453, 38.794097900390625, 38.799102783203125, 38.799102783203125, 38.84290313720703, 38.86250305175781, 38.86250305175781, 38.8754997253418, 38.897300720214844, 38.90769958496094, 38.90769958496094, 38.94029998779297, 38.94029998779297, 38.94029998779297, 38.95399856567383, 38.970401763916016, 38.970401763916016, 38.99089813232422, 38.995201110839844, 39.07680130004883, 39.07680130004883, 39.105098724365234, 39.1702995300293, 39.19049835205078, 39.19049835205078, 39.2317008972168, 39.2317008972168, 39.26620101928711, 39.26620101928711, 39.29500198364258, 39.38960266113281, 39.393402099609375, 39.416500091552734, 39.416500091552734, 39.43429946899414, 39.43429946899414, 39.466697692871094, 39.51319885253906, 39.51319885253906, 39.51319885253906, 39.546600341796875, 39.546600341796875, 39.546600341796875, 39.593299865722656, 39.60029983520508, 39.61429977416992, 39.61869812011719, 39.62220001220703, 39.651702880859375, 39.651702880859375, 39.651702880859375, 39.651702880859375, 39.66400146484375, 39.66400146484375, 39.67720031738281, 39.68949890136719, 39.70649719238281, 39.70649719238281, 39.70840072631836, 39.70840072631836, 39.728599548339844, 39.730499267578125, 39.745399475097656, 39.745399475097656, 39.75749969482422, 39.77619934082031, 39.77619934082031, 39.77619934082031, 39.77619934082031, 39.777400970458984, 39.777400970458984, 39.777400970458984, 39.82859802246094, 39.885501861572266, 39.92759704589844, 39.938697814941406, 39.938697814941406, 39.94159698486328, 39.95349884033203, 39.95349884033203, 39.98249816894531, 39.98249816894531, 39.9911994934082, 40.026798248291016, 40.026798248291016, 40.02799987792969, 40.09120178222656, 40.09120178222656, 40.11199951171875, 40.14720153808594, 40.15159606933594, 40.22330093383789, 40.22330093383789, 40.23259735107422, 40.23979949951172, 40.27179718017578, 40.31780242919922, 40.33830261230469, 40.36219787597656, 40.389400482177734, 40.389400482177734, 40.389400482177734, 40.399898529052734, 40.40549850463867, 40.40549850463867, 40.40549850463867, 40.40549850463867, 40.417198181152344, 40.417198181152344, 40.41780090332031, 40.48080062866211, 40.48080062866211, 40.48080062866211, 40.52330017089844, 40.54180145263672, 40.577301025390625, 40.577301025390625, 40.67359924316406, 40.67359924316406, 40.763099670410156, 40.763099670410156, 40.8302001953125, 40.840599060058594, 40.840599060058594, 40.84649658203125, 40.84870147705078, 40.84870147705078, 40.84880065917969, 40.84880065917969, 40.86479949951172, 40.86479949951172, 40.86479949951172, 40.87300109863281, 40.89820098876953, 40.907798767089844, 40.907798767089844, 40.91360092163086, 40.91360092163086, 40.91360092163086, 40.9911994934082, 41.02320098876953, 41.03010177612305, 41.03010177612305, 41.055599212646484, 41.075897216796875, 41.11070251464844, 41.11070251464844, 41.1151008605957, 41.139495849609375, 41.198299407958984, 41.198299407958984, 41.198299407958984, 41.198299407958984, 41.20880126953125, 41.20880126953125, 41.22269821166992, 41.23320007324219, 41.23320007324219, 41.23320007324219, 41.2411994934082, 41.25170135498047, 41.255897521972656, 41.27110290527344, 41.27110290527344, 41.275299072265625, 41.30970001220703, 41.30970001220703, 41.30970001220703, 41.30970001220703, 41.345699310302734, 41.345699310302734, 41.345699310302734, 41.345699310302734, 41.35890197753906, 41.3922004699707, 41.3922004699707, 41.40230178833008, 41.40230178833008, 41.40230178833008, 41.40230178833008, 41.415000915527344, 41.45110321044922, 41.455299377441406, 41.47739791870117, 41.47739791870117, 41.47739791870117, 41.50339889526367, 41.50339889526367, 41.50740051269531, 41.52149963378906, 41.548797607421875, 41.548797607421875, 41.548797607421875, 41.573402404785156, 41.573402404785156, 41.574501037597656, 41.574501037597656, 41.574501037597656, 41.63800048828125, 41.63909912109375, 41.64419937133789, 41.64419937133789, 41.65769958496094, 41.689998626708984, 41.689998626708984, 41.704795837402344, 41.704795837402344, 41.704795837402344, 41.704795837402344, 41.704795837402344, 41.71039962768555, 41.72220230102539, 41.72220230102539, 41.72620391845703, 41.73270034790039, 41.750099182128906, 41.750099182128906, 41.75830078125, 41.76319885253906, 41.77149963378906, 41.77149963378906, 41.77989959716797, 41.80889892578125, 41.80889892578125, 41.80889892578125, 41.80889892578125, 41.86119842529297, 41.86119842529297, 41.91320037841797, 41.91320037841797, 41.91320037841797, 41.96689987182617, 42.01020050048828, 42.01020050048828, 42.019100189208984, 42.03820037841797, 42.042999267578125, 42.042999267578125, 42.047096252441406, 42.047096252441406, 42.097801208496094, 42.15789794921875, 42.15789794921875, 42.16200256347656, 42.16239929199219, 42.19599914550781, 42.19599914550781, 42.199501037597656, 42.20490264892578, 42.230201721191406, 42.255699157714844, 42.27110290527344, 42.272300720214844, 42.272300720214844, 42.29460144042969, 42.29710006713867, 42.29869842529297, 42.29869842529297, 42.29869842529297, 42.329803466796875, 42.354000091552734, 42.35580062866211, 42.35580062866211, 42.358299255371094, 42.359901428222656, 42.36260223388672, 42.36920166015625, 42.38330078125, 42.38330078125, 42.38330078125, 42.479400634765625, 42.479400634765625, 42.48040008544922, 42.48040008544922, 42.48040008544922, 42.48040008544922, 42.49610137939453, 42.49610137939453, 42.49610137939453, 42.49610137939453, 42.54719924926758, 42.58489990234375, 42.589500427246094, 42.59280014038086, 42.59280014038086, 42.59280014038086, 42.59280014038086, 42.59830093383789, 42.601600646972656, 42.60969924926758, 42.60969924926758, 42.6254997253418, 42.6254997253418, 42.6525993347168, 42.6525993347168, 42.6525993347168, 42.65589904785156, 42.65589904785156, 42.65589904785156, 42.667198181152344, 42.667198181152344, 42.670501708984375, 42.670501708984375, 42.670501708984375, 42.68939971923828, 42.68939971923828, 42.69270324707031, 42.69770050048828, 42.69770050048828, 42.71800231933594, 42.71800231933594, 42.71800231933594, 42.71800231933594, 42.71800231933594, 42.7224006652832, 42.74030303955078, 42.74030303955078, 42.754798889160156, 42.76599884033203, 42.768699645996094, 42.768699645996094, 42.78209686279297, 42.78209686279297, 42.82019805908203, 42.82830047607422, 42.83899688720703, 42.83899688720703, 42.83899688720703, 42.83899688720703, 42.84579849243164, 42.84579849243164, 42.94269943237305, 42.94269943237305, 43.022499084472656, 43.022499084472656, 43.022499084472656, 43.121498107910156, 43.121498107910156, 43.121498107910156, 43.16780090332031, 43.16780090332031, 43.21119689941406, 43.213600158691406, 43.221099853515625, 43.221099853515625, 43.221099853515625, 43.22630310058594, 43.24259948730469, 43.25530242919922, 43.435298919677734, 43.435298919677734, 43.435298919677734, 43.435298919677734, 43.47869873046875, 43.47869873046875, 43.47869873046875, 43.47869873046875, 43.48759841918945, 43.525001525878906, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.55149841308594, 43.588802337646484, 43.603302001953125, 43.603302001953125, 43.603302001953125, 43.603302001953125, 43.603302001953125, 43.633602142333984, 43.633602142333984, 43.640899658203125, 43.679298400878906, 43.697898864746094, 43.73100280761719, 43.73100280761719, 43.7318000793457, 43.77649688720703, 43.77649688720703, 43.77939987182617, 43.77939987182617, 43.77939987182617, 43.77939987182617, 43.82209777832031, 43.843502044677734, 43.843502044677734, 43.87670135498047, 43.87670135498047, 43.87839889526367, 43.950599670410156, 43.952301025390625, 44.037200927734375, 44.03950119018555, 44.103302001953125, 44.103302001953125, 44.1239013671875, 44.1239013671875, 44.16809844970703, 44.16809844970703, 44.183101654052734, 44.183101654052734, 44.186004638671875, 44.186004638671875, 44.206398010253906, 44.206398010253906, 44.24469757080078, 44.24869918823242, 44.24869918823242, 44.281002044677734, 44.333099365234375, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.33709716796875, 44.35199737548828, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.35599899291992, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.359703063964844, 44.37989807128906, 44.417198181152344, 44.417198181152344, 44.417198181152344, 44.418296813964844, 44.418296813964844, 44.418296813964844, 44.418296813964844, 44.418296813964844, 44.418800354003906, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45399856567383, 44.45970153808594, 44.45970153808594, 44.45970153808594, 44.45970153808594, 44.49340057373047, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.49909973144531, 44.52239990234375, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.528099060058594, 44.53670120239258, 44.566898345947266, 44.566898345947266, 44.566898345947266, 44.566898345947266, 44.566898345947266, 44.57200241088867, 44.57200241088867, 44.57200241088867, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.70770263671875, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.71240234375, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.77910232543945, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.821903228759766, 44.85129928588867, 44.85129928588867, 44.85129928588867, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.857200622558594, 44.86759948730469, 44.86759948730469, 44.87350082397461, 44.87350082397461, 44.87350082397461, 44.87350082397461, 44.915199279785156, 44.915199279785156, 44.915199279785156, 44.915199279785156]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Upload latest optimizer 1000 iteration results
</commit_message>
<xml_diff>
--- a/results_fcgma/ResultsCompMethod.xlsx
+++ b/results_fcgma/ResultsCompMethod.xlsx
@@ -439,20 +439,20 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>[[0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 0.]
+ [0. 1. 0. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]
  ...
  [0. 0. 0. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 1. 0. 0.]]</t>
+ [0. 0. 0. ... 0. 0. 0.]]</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22.17259979248047</v>
+        <v>35.38909912109375</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[8.237699508666992, 8.237699508666992, 8.237699508666992, 8.357200622558594, 8.41919994354248, 8.41919994354248, 8.792699813842773, 8.792699813842773, 9.292499542236328, 9.292499542236328, 9.292499542236328, 9.543498992919922, 9.567499160766602, 9.567499160766602, 9.843099594116211, 9.843099594116211, 9.843099594116211, 10.014799118041992, 10.014799118041992, 10.014799118041992, 10.074100494384766, 10.074100494384766, 10.174300193786621, 10.186500549316406, 10.186500549316406, 10.186500549316406, 10.186500549316406, 10.429999351501465, 10.429999351501465, 10.429999351501465, 10.429999351501465, 10.431400299072266, 10.986400604248047, 10.986400604248047, 10.986400604248047, 11.015600204467773, 11.034699440002441, 11.230500221252441, 11.230500221252441, 11.54580020904541, 11.54580020904541, 11.54580020904541, 11.54580020904541, 11.876699447631836, 11.876699447631836, 11.893799781799316, 12.018400192260742, 12.018400192260742, 12.0733003616333, 12.0733003616333, 12.177200317382812, 12.177200317382812, 12.177200317382812, 12.280500411987305, 12.328300476074219, 12.33899974822998, 12.33899974822998, 12.342599868774414, 12.469600677490234, 12.604599952697754, 12.604599952697754, 12.604599952697754, 12.780900001525879, 12.7829008102417, 12.7829008102417, 12.7829008102417, 12.984100341796875, 12.984100341796875, 13.053199768066406, 13.053199768066406, 13.060799598693848, 13.14739990234375, 13.14739990234375, 13.186698913574219, 13.186698913574219, 13.251899719238281, 13.251899719238281, 13.251899719238281, 13.252900123596191, 13.252900123596191, 13.499200820922852, 13.499200820922852, 13.499200820922852, 13.55270004272461, 13.55270004272461, 13.592300415039062, 13.596000671386719, 13.596000671386719, 13.596000671386719, 13.639400482177734, 13.666500091552734, 13.730500221252441, 13.776700019836426, 13.85460090637207, 13.85460090637207, 13.858099937438965, 13.858099937438965, 13.858099937438965, 13.858099937438965, 13.876701354980469, 13.9468994140625, 13.947800636291504, 13.965300559997559, 14.003999710083008, 14.091401100158691, 14.110000610351562, 14.121999740600586, 14.135100364685059, 14.217599868774414, 14.313699722290039, 14.313699722290039, 14.313699722290039, 14.32819938659668, 14.350800514221191, 14.364100456237793, 14.444700241088867, 14.478800773620605, 14.478800773620605, 14.496600151062012, 14.496600151062012, 14.657100677490234, 14.672500610351562, 14.672500610351562, 14.672500610351562, 14.721400260925293, 14.760601043701172, 14.767600059509277, 14.810400009155273, 14.826900482177734, 14.826900482177734, 14.838299751281738, 14.838299751281738, 14.851500511169434, 14.863500595092773, 14.87350082397461, 14.87350082397461, 14.892601013183594, 15.006799697875977, 15.006799697875977, 15.024399757385254, 15.024399757385254, 15.046100616455078, 15.133001327514648, 15.133001327514648, 15.140399932861328, 15.140399932861328, 15.143600463867188, 15.145899772644043, 15.145899772644043, 15.173199653625488, 15.180601119995117, 15.2322998046875, 15.248300552368164, 15.25059986114502, 15.25059986114502, 15.284000396728516, 15.33440113067627, 15.381200790405273, 15.398401260375977, 15.398401260375977, 15.398401260375977, 15.398401260375977, 15.434000015258789, 15.434000015258789, 15.44420051574707, 15.478700637817383, 15.499500274658203, 15.499500274658203, 15.499600410461426, 15.531499862670898, 15.531499862670898, 15.542400360107422, 15.55579948425293, 15.55579948425293, 15.557201385498047, 15.571300506591797, 15.571300506591797, 15.60680103302002, 15.60680103302002, 15.627399444580078, 15.627399444580078, 15.665600776672363, 15.69990062713623, 15.708200454711914, 15.728200912475586, 15.728200912475586, 15.729799270629883, 15.777800559997559, 15.777800559997559, 15.777800559997559, 15.777800559997559, 15.777800559997559, 15.780800819396973, 15.780800819396973, 15.811700820922852, 15.811700820922852, 15.850201606750488, 15.850201606750488, 15.854700088500977, 15.873100280761719, 15.873200416564941, 15.873200416564941, 15.873600006103516, 15.873600006103516, 15.873600006103516, 15.898399353027344, 15.898399353027344, 15.898399353027344, 15.898399353027344, 15.898399353027344, 15.915300369262695, 15.946499824523926, 15.946499824523926, 15.949400901794434, 16.004899978637695, 16.004899978637695, 16.006500244140625, 16.006500244140625, 16.00830078125, 16.0093994140625, 16.03660011291504, 16.03660011291504, 16.03660011291504, 16.04869842529297, 16.04869842529297, 16.056800842285156, 16.0635986328125, 16.0635986328125, 16.0635986328125, 16.06570053100586, 16.06570053100586, 16.082801818847656, 16.090099334716797, 16.090099334716797, 16.090099334716797, 16.139999389648438, 16.158802032470703, 16.158802032470703, 16.1924991607666, 16.1924991607666, 16.195899963378906, 16.239501953125, 16.239501953125, 16.24540138244629, 16.24540138244629, 16.271800994873047, 16.28270149230957, 16.28270149230957, 16.34309959411621, 16.346500396728516, 16.346500396728516, 16.388099670410156, 16.388099670410156, 16.388099670410156, 16.388099670410156, 16.388099670410156, 16.388099670410156, 16.39200210571289, 16.39200210571289, 16.447399139404297, 16.447399139404297, 16.447399139404297, 16.479900360107422, 16.479900360107422, 16.479900360107422, 16.511600494384766, 16.52280044555664, 16.535900115966797, 16.535900115966797, 16.549800872802734, 16.56290054321289, 16.56290054321289, 16.59440040588379, 16.59440040588379, 16.595300674438477, 16.595300674438477, 16.606399536132812, 16.633901596069336, 16.633901596069336, 16.643199920654297, 16.664199829101562, 16.664199829101562, 16.672401428222656, 16.69260025024414, 16.69260025024414, 16.69260025024414, 16.697601318359375, 16.697601318359375, 16.701801300048828, 16.731399536132812, 16.731399536132812, 16.736400604248047, 16.736400604248047, 16.736400604248047, 16.760299682617188, 16.780200958251953, 16.780200958251953, 16.780500411987305, 16.780500411987305, 16.835901260375977, 16.835901260375977, 16.835901260375977, 16.841999053955078, 16.841999053955078, 16.89150047302246, 16.89150047302246, 16.89150047302246, 16.89150047302246, 16.89150047302246, 16.906299591064453, 16.911300659179688, 16.914701461791992, 16.914701461791992, 17.052200317382812, 17.052200317382812, 17.052200317382812, 17.058700561523438, 17.05900001525879, 17.05900001525879, 17.05900001525879, 17.05900001525879, 17.071701049804688, 17.079700469970703, 17.110300064086914, 17.15380096435547, 17.192298889160156, 17.192298889160156, 17.192298889160156, 17.19260025024414, 17.19260025024414, 17.236499786376953, 17.291900634765625, 17.329200744628906, 17.343101501464844, 17.365800857543945, 17.365800857543945, 17.365800857543945, 17.368499755859375, 17.368499755859375, 17.420101165771484, 17.420101165771484, 17.430599212646484, 17.44610023498535, 17.44849967956543, 17.452301025390625, 17.452301025390625, 17.452600479125977, 17.452600479125977, 17.452600479125977, 17.452600479125977, 17.452600479125977, 17.452600479125977, 17.490001678466797, 17.490001678466797, 17.49919891357422, 17.506000518798828, 17.506000518798828, 17.514202117919922, 17.53569984436035, 17.55550193786621, 17.556901931762695, 17.556901931762695, 17.591800689697266, 17.591800689697266, 17.591800689697266, 17.625900268554688, 17.627700805664062, 17.633100509643555, 17.633100509643555, 17.65690040588379, 17.65690040588379, 17.65690040588379, 17.66230010986328, 17.66230010986328, 17.66230010986328, 17.663999557495117, 17.663999557495117, 17.663999557495117, 17.666000366210938, 17.667699813842773, 17.690399169921875, 17.690399169921875, 17.692100524902344, 17.692699432373047, 17.692699432373047, 17.702699661254883, 17.702699661254883, 17.70370101928711, 17.705402374267578, 17.707799911499023, 17.710201263427734, 17.811901092529297, 17.859500885009766, 17.859500885009766, 17.869300842285156, 17.913400650024414, 17.913400650024414, 17.92300033569336, 17.92300033569336, 17.92300033569336, 17.934600830078125, 17.934600830078125, 17.97100067138672, 17.973400115966797, 17.973400115966797, 17.973400115966797, 17.987499237060547, 17.987499237060547, 17.99020004272461, 17.99020004272461, 18.036800384521484, 18.042301177978516, 18.046300888061523, 18.052200317382812, 18.07390022277832, 18.07390022277832, 18.07390022277832, 18.07390022277832, 18.07390022277832, 18.074901580810547, 18.074901580810547, 18.074901580810547, 18.074901580810547, 18.076200485229492, 18.078899383544922, 18.10430145263672, 18.10430145263672, 18.108299255371094, 18.16119956970215, 18.16119956970215, 18.19580078125, 18.19580078125, 18.19580078125, 18.19580078125, 18.19580078125, 18.19580078125, 18.19580078125, 18.221099853515625, 18.234399795532227, 18.234399795532227, 18.234399795532227, 18.234399795532227, 18.247299194335938, 18.349300384521484, 18.349300384521484, 18.349899291992188, 18.349899291992188, 18.436199188232422, 18.464599609375, 18.464599609375, 18.48550033569336, 18.486801147460938, 18.489099502563477, 18.489099502563477, 18.489099502563477, 18.489099502563477, 18.489099502563477, 18.489500045776367, 18.512300491333008, 18.512300491333008, 18.526901245117188, 18.549400329589844, 18.549400329589844, 18.55729866027832, 18.577899932861328, 18.580299377441406, 18.582599639892578, 18.582599639892578, 18.61549949645996, 18.61549949645996, 18.627099990844727, 18.65610122680664, 18.65610122680664, 18.66809844970703, 18.66809844970703, 18.67169952392578, 18.67169952392578, 18.68120002746582, 18.68120002746582, 18.688199996948242, 18.742900848388672, 18.742900848388672, 18.828001022338867, 18.840599060058594, 18.840599060058594, 18.846399307250977, 18.850400924682617, 18.850400924682617, 18.850400924682617, 18.864500045776367, 18.892601013183594, 18.892601013183594, 18.892601013183594, 18.9424991607666, 18.9424991607666, 18.96739959716797, 19.032699584960938, 19.032699584960938, 19.060100555419922, 19.060100555419922, 19.060100555419922, 19.060100555419922, 19.063499450683594, 19.08370018005371, 19.08370018005371, 19.08370018005371, 19.08370018005371, 19.08370018005371, 19.08489990234375, 19.086898803710938, 19.121299743652344, 19.15169906616211, 19.15169906616211, 19.210599899291992, 19.210599899291992, 19.226299285888672, 19.229700088500977, 19.229700088500977, 19.229700088500977, 19.229700088500977, 19.229700088500977, 19.229700088500977, 19.229700088500977, 19.23110008239746, 19.23110008239746, 19.247398376464844, 19.25389862060547, 19.274799346923828, 19.274799346923828, 19.274799346923828, 19.274799346923828, 19.31679916381836, 19.317699432373047, 19.317699432373047, 19.31999969482422, 19.320899963378906, 19.34149932861328, 19.34149932861328, 19.34149932861328, 19.34149932861328, 19.34469985961914, 19.34469985961914, 19.34469985961914, 19.34469985961914, 19.34619903564453, 19.34910011291504, 19.389299392700195, 19.389299392700195, 19.389299392700195, 19.48550033569336, 19.48550033569336, 19.573501586914062, 19.573501586914062, 19.583900451660156, 19.583900451660156, 19.583900451660156, 19.602500915527344, 19.620498657226562, 19.63520050048828, 19.63520050048828, 19.677600860595703, 19.677600860595703, 19.677600860595703, 19.68800163269043, 19.69580078125, 19.69580078125, 19.69580078125, 19.69580078125, 19.699100494384766, 19.75629997253418, 19.75629997253418, 19.768199920654297, 19.768199920654297, 19.768199920654297, 19.768199920654297, 19.768199920654297, 19.768199920654297, 19.831199645996094, 19.831199645996094, 19.879199981689453, 19.8877010345459, 19.8877010345459, 19.90130043029785, 19.90130043029785, 19.90130043029785, 19.91230010986328, 19.91230010986328, 19.91230010986328, 19.91990089416504, 19.91990089416504, 19.92180061340332, 19.935100555419922, 19.935100555419922, 19.937000274658203, 19.937000274658203, 19.937000274658203, 19.977399826049805, 19.987499237060547, 20.02320098876953, 20.02770233154297, 20.02770233154297, 20.05769920349121, 20.05769920349121, 20.05769920349121, 20.061901092529297, 20.077999114990234, 20.105300903320312, 20.105300903320312, 20.151899337768555, 20.151899337768555, 20.193700790405273, 20.204898834228516, 20.204898834228516, 20.212299346923828, 20.243099212646484, 20.243099212646484, 20.243099212646484, 20.250499725341797, 20.260601043701172, 20.260601043701172, 20.270198822021484, 20.270198822021484, 20.270198822021484, 20.282400131225586, 20.3031005859375, 20.33340072631836, 20.33340072631836, 20.33340072631836, 20.366100311279297, 20.366100311279297, 20.37220001220703, 20.37220001220703, 20.378000259399414, 20.378000259399414, 20.400501251220703, 20.400501251220703, 20.406600952148438, 20.421100616455078, 20.421100616455078, 20.42650032043457, 20.42650032043457, 20.42650032043457, 20.427600860595703, 20.427600860595703, 20.427600860595703, 20.433000564575195, 20.504499435424805, 20.504499435424805, 20.509899139404297, 20.52359962463379, 20.524499893188477, 20.524499893188477, 20.524499893188477, 20.538999557495117, 20.555099487304688, 20.555099487304688, 20.595001220703125, 20.600399017333984, 20.601999282836914, 20.60580062866211, 20.60580062866211, 20.60580062866211, 20.60580062866211, 20.60580062866211, 20.60580062866211, 20.62700080871582, 20.62700080871582, 20.62700080871582, 20.62700080871582, 20.62700080871582, 20.62700080871582, 20.64820098876953, 20.655200958251953, 20.65679931640625, 20.663799285888672, 20.673398971557617, 20.688701629638672, 20.69409942626953, 20.69409942626953, 20.69409942626953, 20.69409942626953, 20.69409942626953, 20.69409942626953, 20.69409942626953, 20.702098846435547, 20.702098846435547, 20.702098846435547, 20.702098846435547, 20.702098846435547, 20.73069953918457, 20.757200241088867, 20.781400680541992, 20.783199310302734, 20.793701171875, 20.823299407958984, 20.823299407958984, 20.864200592041016, 20.864200592041016, 20.879798889160156, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.9093017578125, 20.948200225830078, 20.948200225830078, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 20.956199645996094, 21.1560001373291, 21.18090057373047, 21.18090057373047, 21.18090057373047, 21.205699920654297, 21.205699920654297, 21.205699920654297, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.211700439453125, 21.22410011291504, 21.26110076904297, 21.26110076904297, 21.26110076904297, 21.332599639892578, 21.332599639892578, 21.373798370361328, 21.373798370361328, 21.37529945373535, 21.376998901367188, 21.376998901367188, 21.379499435424805, 21.386798858642578, 21.386798858642578, 21.388399124145508, 21.388399124145508, 21.388399124145508, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.39259910583496, 21.440200805664062, 21.456600189208984, 21.456600189208984, 21.460800170898438, 21.460800170898438, 21.460800170898438, 21.460800170898438, 21.474599838256836, 21.47480010986328, 21.47480010986328, 21.48849868774414, 21.500999450683594, 21.500999450683594, 21.506799697875977, 21.506799697875977, 21.51099967956543, 21.512300491333008, 21.512300491333008, 21.512300491333008, 21.60270118713379, 21.603801727294922, 21.667999267578125, 21.667999267578125, 21.667999267578125, 21.680498123168945, 21.6846981048584, 21.6846981048584, 21.6846981048584, 21.6846981048584, 21.70319938659668, 21.708301544189453, 21.76650047302246, 21.783199310302734, 21.783199310302734, 21.783199310302734, 21.78369903564453, 21.789199829101562, 21.789199829101562, 21.789199829101562, 21.789199829101562, 21.789199829101562, 21.789199829101562, 21.799198150634766, 21.801700592041016, 21.801700592041016, 21.801700592041016, 21.807701110839844, 21.807701110839844, 21.81369972229004, 21.823898315429688, 21.823898315429688, 21.823898315429688, 21.823898315429688, 21.823898315429688, 21.823898315429688, 21.83839988708496, 21.83839988708496, 21.83839988708496, 21.83839988708496, 21.85580062866211, 21.85580062866211, 21.861799240112305, 21.861799240112305, 21.861799240112305, 21.864200592041016, 21.87769889831543, 21.88010025024414, 21.88010025024414, 21.89499855041504, 21.89499855041504, 21.89499855041504, 21.89499855041504, 21.89499855041504, 21.89499855041504, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.8966007232666, 21.899301528930664, 21.90169906616211, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.92409896850586, 21.927600860595703, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.933300018310547, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.944299697875977, 21.983299255371094, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.984798431396484, 21.988800048828125, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 21.994800567626953, 22.071800231933594, 22.071800231933594, 22.071800231933594, 22.07509994506836, 22.07509994506836, 22.07509994506836, 22.07509994506836, 22.07509994506836, 22.13759994506836, 22.13759994506836, 22.13759994506836, 22.13759994506836, 22.13759994506836, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.146499633789062, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.157800674438477, 22.16510009765625, 22.16510009765625, 22.16510009765625, 22.16510009765625, 22.16510009765625, 22.17259979248047, 22.17259979248047]</t>
+          <t>[20.500900268554688, 20.597900390625, 20.717498779296875, 21.809999465942383, 21.809999465942383, 21.809999465942383, 21.809999465942383, 21.809999465942383, 21.809999465942383, 21.809999465942383, 22.23910140991211, 22.23910140991211, 22.983301162719727, 22.983301162719727, 23.25389862060547, 23.25389862060547, 23.25389862060547, 23.344799041748047, 23.700700759887695, 23.700700759887695, 23.700700759887695, 23.700700759887695, 23.700700759887695, 23.700700759887695, 23.804100036621094, 24.034399032592773, 24.034399032592773, 24.034399032592773, 24.034399032592773, 24.034399032592773, 24.03499984741211, 24.121299743652344, 24.200698852539062, 24.200698852539062, 24.36009979248047, 24.53569984436035, 24.53569984436035, 24.56999969482422, 24.56999969482422, 24.797000885009766, 24.797000885009766, 24.797000885009766, 24.797000885009766, 24.797000885009766, 24.797000885009766, 24.965900421142578, 24.974700927734375, 24.974700927734375, 25.023700714111328, 25.072799682617188, 25.082000732421875, 25.191099166870117, 25.191099166870117, 25.32489776611328, 25.32489776611328, 25.35540008544922, 25.398300170898438, 25.398300170898438, 25.44110107421875, 25.44110107421875, 25.669300079345703, 25.669300079345703, 25.675498962402344, 25.702999114990234, 25.702999114990234, 25.707799911499023, 25.963600158691406, 25.963600158691406, 25.963600158691406, 26.018299102783203, 26.19580078125, 26.19580078125, 26.19580078125, 26.19580078125, 26.20090103149414, 26.284000396728516, 26.284000396728516, 26.390899658203125, 26.390899658203125, 26.489700317382812, 26.489700317382812, 26.520898818969727, 26.520898818969727, 26.520898818969727, 26.54990005493164, 26.54990005493164, 26.66119956970215, 26.66119956970215, 26.66119956970215, 26.740299224853516, 26.740299224853516, 26.762001037597656, 26.81999969482422, 26.824899673461914, 26.824899673461914, 26.904600143432617, 26.904600143432617, 26.91109848022461, 26.91109848022461, 26.997699737548828, 26.997699737548828, 26.997699737548828, 27.042800903320312, 27.045799255371094, 27.045799255371094, 27.070499420166016, 27.07469940185547, 27.084400177001953, 27.164199829101562, 27.172298431396484, 27.172298431396484, 27.186199188232422, 27.186199188232422, 27.2406005859375, 27.2406005859375, 27.2406005859375, 27.249399185180664, 27.304500579833984, 27.446001052856445, 27.51959991455078, 27.51959991455078, 27.574899673461914, 27.574899673461914, 27.574899673461914, 27.57859992980957, 27.57859992980957, 27.604000091552734, 27.604000091552734, 27.610000610351562, 27.610000610351562, 27.673500061035156, 27.673500061035156, 27.673500061035156, 27.688400268554688, 27.733299255371094, 27.733299255371094, 27.733299255371094, 27.75619888305664, 27.75619888305664, 27.77519989013672, 27.77519989013672, 27.789997100830078, 27.789997100830078, 27.829200744628906, 27.83449935913086, 27.837100982666016, 27.862600326538086, 27.862600326538086, 27.87660026550293, 27.87660026550293, 27.892898559570312, 27.892898559570312, 27.909400939941406, 27.915498733520508, 27.93939971923828, 27.96320152282715, 27.96320152282715, 27.96320152282715, 27.978900909423828, 27.978900909423828, 28.000499725341797, 28.000499725341797, 28.045101165771484, 28.045101165771484, 28.045101165771484, 28.045101165771484, 28.052701950073242, 28.052701950073242, 28.06279945373535, 28.06279945373535, 28.06279945373535, 28.11050033569336, 28.11050033569336, 28.11050033569336, 28.112098693847656, 28.12929916381836, 28.137699127197266, 28.137699127197266, 28.15489959716797, 28.15489959716797, 28.165401458740234, 28.165401458740234, 28.165401458740234, 28.16939926147461, 28.21160125732422, 28.253501892089844, 28.253501892089844, 28.253501892089844, 28.28019905090332, 28.28019905090332, 28.301898956298828, 28.327999114990234, 28.360300064086914, 28.431800842285156, 28.431800842285156, 28.431800842285156, 28.441699981689453, 28.478199005126953, 28.49810028076172, 28.49810028076172, 28.49810028076172, 28.512100219726562, 28.512100219726562, 28.512100219726562, 28.524200439453125, 28.5310001373291, 28.553800582885742, 28.553800582885742, 28.55419921875, 28.55419921875, 28.555599212646484, 28.582801818847656, 28.62019920349121, 28.62019920349121, 28.64419937133789, 28.651599884033203, 28.651599884033203, 28.744600296020508, 28.782100677490234, 28.782100677490234, 28.989700317382812, 28.989700317382812, 28.991901397705078, 28.991901397705078, 28.991901397705078, 29.041301727294922, 29.041301727294922, 29.041601181030273, 29.041601181030273, 29.057100296020508, 29.100399017333984, 29.100399017333984, 29.100399017333984, 29.103700637817383, 29.12220001220703, 29.13719940185547, 29.16860008239746, 29.16860008239746, 29.17140007019043, 29.17140007019043, 29.18120002746582, 29.18120002746582, 29.18120002746582, 29.18429946899414, 29.18429946899414, 29.188899993896484, 29.189800262451172, 29.189800262451172, 29.22439956665039, 29.243999481201172, 29.243999481201172, 29.306299209594727, 29.306299209594727, 29.321102142333984, 29.321102142333984, 29.352401733398438, 29.393199920654297, 29.393199920654297, 29.394298553466797, 29.394298553466797, 29.394298553466797, 29.39529800415039, 29.404401779174805, 29.404401779174805, 29.405799865722656, 29.410400390625, 29.42840003967285, 29.42840003967285, 29.42840003967285, 29.42840003967285, 29.434099197387695, 29.434099197387695, 29.434099197387695, 29.442100524902344, 29.48889923095703, 29.494300842285156, 29.494300842285156, 29.494300842285156, 29.50469970703125, 29.50469970703125, 29.50469970703125, 29.552200317382812, 29.552200317382812, 29.552200317382812, 29.559999465942383, 29.600900650024414, 29.651500701904297, 29.651500701904297, 29.651500701904297, 29.683799743652344, 29.683799743652344, 29.683799743652344, 29.705299377441406, 29.705299377441406, 29.744998931884766, 29.796398162841797, 29.796398162841797, 29.796398162841797, 29.796398162841797, 29.796398162841797, 29.836502075195312, 29.873300552368164, 29.873300552368164, 29.87969970703125, 29.887401580810547, 29.887401580810547, 29.887401580810547, 29.924999237060547, 29.924999237060547, 29.95149803161621, 29.95149803161621, 29.95560073852539, 29.95560073852539, 29.95560073852539, 29.95840072631836, 29.95840072631836, 30.028499603271484, 30.028499603271484, 30.028499603271484, 30.054798126220703, 30.054798126220703, 30.058700561523438, 30.062002182006836, 30.062002182006836, 30.062002182006836, 30.062002182006836, 30.09160041809082, 30.110599517822266, 30.110599517822266, 30.127599716186523, 30.127599716186523, 30.29410171508789, 30.29410171508789, 30.33270263671875, 30.33270263671875, 30.33270263671875, 30.35340118408203, 30.358800888061523, 30.358800888061523, 30.365100860595703, 30.365100860595703, 30.365100860595703, 30.366199493408203, 30.371400833129883, 30.375701904296875, 30.42660140991211, 30.432899475097656, 30.432899475097656, 30.440399169921875, 30.453998565673828, 30.48750114440918, 30.48750114440918, 30.48750114440918, 30.48750114440918, 30.491701126098633, 30.491701126098633, 30.530799865722656, 30.530799865722656, 30.532699584960938, 30.532699584960938, 30.555801391601562, 30.555801391601562, 30.585201263427734, 30.606000900268555, 30.606000900268555, 30.607200622558594, 30.637399673461914, 30.68349838256836, 30.704200744628906, 30.704200744628906, 30.70530128479004, 30.70530128479004, 30.70530128479004, 30.70530128479004, 30.71649932861328, 30.71649932861328, 30.75320053100586, 30.75320053100586, 30.775598526000977, 30.775598526000977, 30.775598526000977, 30.79020118713379, 30.8356990814209, 30.841999053955078, 30.85500144958496, 30.85500144958496, 30.85500144958496, 30.85500144958496, 30.85500144958496, 30.860000610351562, 30.880298614501953, 30.88960075378418, 30.90719985961914, 30.910200119018555, 30.910200119018555, 30.941299438476562, 30.941299438476562, 30.941299438476562, 30.941299438476562, 30.941299438476562, 30.953601837158203, 30.953601837158203, 30.953601837158203, 30.954898834228516, 30.95560073852539, 30.958301544189453, 30.958301544189453, 30.967500686645508, 30.967500686645508, 30.996400833129883, 30.99799919128418, 30.998300552368164, 31.06319808959961, 31.105199813842773, 31.125701904296875, 31.125701904296875, 31.1289005279541, 31.172998428344727, 31.19219970703125, 31.19219970703125, 31.229900360107422, 31.229900360107422, 31.229900360107422, 31.252399444580078, 31.252399444580078, 31.261898040771484, 31.261898040771484, 31.261898040771484, 31.32740020751953, 31.32740020751953, 31.327899932861328, 31.335599899291992, 31.335599899291992, 31.37150001525879, 31.402599334716797, 31.402599334716797, 31.402599334716797, 31.405900955200195, 31.405900955200195, 31.420398712158203, 31.42300033569336, 31.424100875854492, 31.461502075195312, 31.465999603271484, 31.48859977722168, 31.501300811767578, 31.501300811767578, 31.50760269165039, 31.50760269165039, 31.507701873779297, 31.507701873779297, 31.51919937133789, 31.528400421142578, 31.536502838134766, 31.54250144958496, 31.54250144958496, 31.577699661254883, 31.60900115966797, 31.60900115966797, 31.60900115966797, 31.615299224853516, 31.617300033569336, 31.617300033569336, 31.62900161743164, 31.62900161743164, 31.62900161743164, 31.65290069580078, 31.652999877929688, 31.652999877929688, 31.65489959716797, 31.65489959716797, 31.72960090637207, 31.72960090637207, 31.72960090637207, 31.72960090637207, 31.72960090637207, 31.746601104736328, 31.747699737548828, 31.78350067138672, 31.78350067138672, 31.78350067138672, 31.78350067138672, 31.885398864746094, 31.885398864746094, 31.885398864746094, 31.932598114013672, 31.932598114013672, 31.933700561523438, 31.9596004486084, 31.960599899291992, 31.960599899291992, 31.9606990814209, 31.9606990814209, 31.9606990814209, 31.977800369262695, 31.986900329589844, 31.986900329589844, 31.986900329589844, 31.99169921875, 32.01380157470703, 32.04499816894531, 32.05059814453125, 32.06300354003906, 32.073097229003906, 32.135799407958984, 32.135799407958984, 32.135799407958984, 32.135799407958984, 32.135799407958984, 32.1598014831543, 32.1598014831543, 32.1598014831543, 32.1598014831543, 32.1598014831543, 32.165000915527344, 32.165000915527344, 32.195098876953125, 32.195098876953125, 32.19620132446289, 32.21659851074219, 32.21659851074219, 32.21800231933594, 32.23729705810547, 32.26459884643555, 32.30070114135742, 32.31119918823242, 32.31119918823242, 32.32579803466797, 32.33829879760742, 32.390098571777344, 32.401702880859375, 32.401702880859375, 32.40380096435547, 32.431800842285156, 32.431800842285156, 32.431800842285156, 32.44059753417969, 32.44059753417969, 32.44059753417969, 32.44059753417969, 32.47779846191406, 32.48740005493164, 32.50090026855469, 32.53160095214844, 32.538299560546875, 32.54140090942383, 32.54140090942383, 32.57160186767578, 32.57160186767578, 32.57160186767578, 32.57440185546875, 32.578800201416016, 32.578800201416016, 32.59510040283203, 32.59510040283203, 32.59510040283203, 32.59510040283203, 32.60070037841797, 32.614200592041016, 32.614200592041016, 32.628700256347656, 32.628700256347656, 32.628700256347656, 32.635799407958984, 32.635799407958984, 32.635799407958984, 32.635799407958984, 32.635799407958984, 32.67980194091797, 32.72690200805664, 32.727901458740234, 32.80500030517578, 32.813201904296875, 32.813201904296875, 32.813201904296875, 32.859500885009766, 32.871700286865234, 32.871700286865234, 32.897499084472656, 32.897499084472656, 32.897499084472656, 32.904998779296875, 32.904998779296875, 32.93280029296875, 32.93280029296875, 32.93659973144531, 32.93659973144531, 32.94139862060547, 32.94139862060547, 33.01259994506836, 33.040401458740234, 33.040401458740234, 33.08429718017578, 33.08429718017578, 33.08429718017578, 33.08429718017578, 33.134498596191406, 33.134498596191406, 33.15290069580078, 33.15290069580078, 33.211997985839844, 33.211997985839844, 33.223899841308594, 33.223899841308594, 33.225399017333984, 33.22809982299805, 33.22809982299805, 33.22809982299805, 33.235599517822266, 33.235599517822266, 33.25559997558594, 33.266700744628906, 33.266700744628906, 33.266700744628906, 33.266700744628906, 33.3046989440918, 33.3046989440918, 33.339500427246094, 33.339500427246094, 33.38159942626953, 33.38159942626953, 33.42620086669922, 33.42620086669922, 33.446800231933594, 33.45240020751953, 33.458099365234375, 33.458099365234375, 33.4635009765625, 33.465702056884766, 33.465702056884766, 33.473899841308594, 33.473899841308594, 33.477500915527344, 33.49169921875, 33.496002197265625, 33.541297912597656, 33.54199981689453, 33.554901123046875, 33.554901123046875, 33.554901123046875, 33.554901123046875, 33.554901123046875, 33.56809997558594, 33.56809997558594, 33.58519744873047, 33.612998962402344, 33.612998962402344, 33.612998962402344, 33.61579895019531, 33.61579895019531, 33.62120056152344, 33.62120056152344, 33.630001068115234, 33.66429901123047, 33.66429901123047, 33.66429901123047, 33.676998138427734, 33.686500549316406, 33.686500549316406, 33.686500549316406, 33.686500549316406, 33.686500549316406, 33.686500549316406, 33.7135009765625, 33.7135009765625, 33.7135009765625, 33.738399505615234, 33.7588005065918, 33.79079818725586, 33.834999084472656, 33.84429931640625, 33.87160110473633, 33.88650131225586, 33.88650131225586, 33.88650131225586, 33.88650131225586, 33.901100158691406, 33.901100158691406, 33.91600036621094, 33.93410110473633, 33.965301513671875, 33.96989822387695, 33.96989822387695, 33.96989822387695, 34.00529861450195, 34.00529861450195, 34.00529861450195, 34.00529861450195, 34.00529861450195, 34.00529861450195, 34.01089859008789, 34.01089859008789, 34.01820373535156, 34.01820373535156, 34.0238037109375, 34.0238037109375, 34.0238037109375, 34.02510070800781, 34.02510070800781, 34.02510070800781, 34.033199310302734, 34.0359001159668, 34.0359001159668, 34.069801330566406, 34.069801330566406, 34.069801330566406, 34.08689880371094, 34.08689880371094, 34.08689880371094, 34.08689880371094, 34.097599029541016, 34.097599029541016, 34.097599029541016, 34.112701416015625, 34.112701416015625, 34.132598876953125, 34.132598876953125, 34.15019989013672, 34.17169952392578, 34.1776008605957, 34.199398040771484, 34.2218017578125, 34.2218017578125, 34.23529815673828, 34.23959732055664, 34.24470138549805, 34.24470138549805, 34.25029754638672, 34.25550079345703, 34.27280044555664, 34.31610107421875, 34.31610107421875, 34.31610107421875, 34.355796813964844, 34.361900329589844, 34.407501220703125, 34.407501220703125, 34.408897399902344, 34.41380310058594, 34.44050216674805, 34.44050216674805, 34.44050216674805, 34.44919967651367, 34.44919967651367, 34.46999740600586, 34.479698181152344, 34.479698181152344, 34.479698181152344, 34.488399505615234, 34.53730010986328, 34.53730010986328, 34.53779983520508, 34.548099517822266, 34.548099517822266, 34.566001892089844, 34.595298767089844, 34.595298767089844, 34.595298767089844, 34.595298767089844, 34.61949920654297, 34.61949920654297, 34.61949920654297, 34.61949920654297, 34.628204345703125, 34.65890121459961, 34.65890121459961, 34.69419860839844, 34.69419860839844, 34.69419860839844, 34.69419860839844, 34.69419860839844, 34.69419860839844, 34.69419860839844, 34.71500015258789, 34.73400115966797, 34.763702392578125, 34.80350112915039, 34.830902099609375, 34.830902099609375, 34.84239959716797, 34.84239959716797, 34.852699279785156, 34.852699279785156, 34.852699279785156, 34.852699279785156, 34.86509704589844, 34.87409973144531, 34.87879943847656, 34.87879943847656, 34.87879943847656, 34.881099700927734, 34.901702880859375, 34.901702880859375, 34.901702880859375, 34.91670227050781, 34.91670227050781, 34.91670227050781, 34.91709899902344, 34.919002532958984, 34.919002532958984, 34.919097900390625, 34.919097900390625, 34.919097900390625, 34.92009735107422, 34.92009735107422, 34.92009735107422, 34.94260025024414, 34.94350051879883, 34.94350051879883, 34.96730041503906, 34.976600646972656, 34.976600646972656, 35.004798889160156, 35.004798889160156, 35.04450225830078, 35.04450225830078, 35.04450225830078, 35.04800033569336, 35.04800033569336, 35.104000091552734, 35.104000091552734, 35.139503479003906, 35.1614990234375, 35.1614990234375, 35.16709899902344, 35.18620300292969, 35.261199951171875, 35.2671012878418, 35.2671012878418, 35.2671012878418, 35.27660369873047, 35.27660369873047, 35.29540252685547, 35.30289840698242, 35.30590057373047, 35.30590057373047, 35.30590057373047, 35.3125, 35.31380081176758, 35.31380081176758, 35.317501068115234, 35.3223991394043, 35.3223991394043, 35.3223991394043, 35.32749938964844, 35.32749938964844, 35.32749938964844, 35.32879638671875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.356201171875, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.35860061645508, 35.37120056152344, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.37379837036133, 35.383697509765625, 35.383697509765625, 35.383697509765625, 35.383697509765625, 35.38909912109375, 35.38909912109375, 35.38909912109375, 35.38909912109375, 35.38909912109375, 35.38909912109375, 35.38909912109375, 35.38909912109375, 35.38909912109375, 35.38909912109375, 35.38909912109375, 35.38909912109375]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update latest optimizer 1000 iteration results
</commit_message>
<xml_diff>
--- a/results_fcgma/ResultsCompMethod.xlsx
+++ b/results_fcgma/ResultsCompMethod.xlsx
@@ -439,20 +439,20 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>[[0. 0. 0. ... 0. 0. 0.]
- [0. 1. 0. ... 0. 0. 0.]
+ [0. 0. 1. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]
  ...
  [0. 0. 0. ... 0. 0. 0.]
- [0. 0. 0. ... 0. 0. 1.]
+ [0. 0. 0. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]]</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50.2322998046875</v>
+        <v>51.3275032043457</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[31.35190200805664, 31.523000717163086, 31.523000717163086, 31.590299606323242, 31.590299606323242, 31.590299606323242, 31.590299606323242, 31.590299606323242, 31.69900131225586, 31.743301391601562, 31.91230010986328, 31.91230010986328, 32.05059814453125, 32.05059814453125, 32.05059814453125, 32.07429885864258, 32.43190002441406, 32.43190002441406, 32.65800094604492, 32.65800094604492, 32.65800094604492, 32.65800094604492, 32.65800094604492, 32.65800094604492, 32.9911994934082, 32.9911994934082, 32.9911994934082, 32.9911994934082, 33.067100524902344, 33.22169876098633, 33.324100494384766, 33.324100494384766, 33.77360153198242, 33.77360153198242, 33.77360153198242, 33.77360153198242, 34.15019989013672, 34.15019989013672, 34.15019989013672, 34.15019989013672, 34.17959976196289, 34.26020050048828, 34.26020050048828, 34.277801513671875, 34.277801513671875, 34.277801513671875, 34.277801513671875, 34.277801513671875, 34.277801513671875, 34.368900299072266, 34.368900299072266, 34.41830062866211, 34.41830062866211, 34.41830062866211, 34.63859939575195, 34.63859939575195, 34.63859939575195, 34.63859939575195, 34.74869918823242, 34.74869918823242, 34.77300262451172, 34.83829879760742, 34.98919677734375, 35.0077018737793, 35.212501525878906, 35.37969970703125, 35.37969970703125, 35.37969970703125, 35.37969970703125, 35.37969970703125, 35.631195068359375, 35.95269775390625, 35.97610092163086, 35.97610092163086, 36.448299407958984, 36.448299407958984, 36.448299407958984, 36.62730026245117, 36.62730026245117, 36.62730026245117, 36.783599853515625, 36.78770065307617, 36.84379959106445, 36.84379959106445, 37.00160217285156, 37.00160217285156, 37.00160217285156, 37.146400451660156, 37.146400451660156, 37.146400451660156, 37.146400451660156, 37.22249984741211, 37.320396423339844, 37.320396423339844, 37.66709899902344, 37.66709899902344, 37.74639892578125, 37.849098205566406, 37.849098205566406, 37.85980224609375, 37.85980224609375, 38.065399169921875, 38.065399169921875, 38.065399169921875, 38.20459747314453, 38.28139877319336, 38.28139877319336, 38.40449905395508, 38.40449905395508, 38.437198638916016, 38.437198638916016, 38.641300201416016, 38.641300201416016, 38.73820114135742, 38.73820114135742, 38.73820114135742, 38.819801330566406, 38.927001953125, 38.93220138549805, 38.93220138549805, 38.93260192871094, 39.14699935913086, 39.14699935913086, 39.14699935913086, 39.253997802734375, 39.26070022583008, 39.26070022583008, 39.310203552246094, 39.341697692871094, 39.36650085449219, 39.36650085449219, 39.370399475097656, 39.370399475097656, 39.37879943847656, 39.49690246582031, 39.49690246582031, 39.529701232910156, 39.529701232910156, 39.529701232910156, 39.529701232910156, 39.529701232910156, 39.54290008544922, 39.55950164794922, 39.63459777832031, 39.658302307128906, 39.658302307128906, 39.683998107910156, 39.683998107910156, 39.70289993286133, 39.72529983520508, 39.72529983520508, 39.7598991394043, 39.873802185058594, 39.873802185058594, 39.873802185058594, 39.95829772949219, 39.95829772949219, 39.95829772949219, 39.965797424316406, 40.007999420166016, 40.007999420166016, 40.00979995727539, 40.01799774169922, 40.10960006713867, 40.156097412109375, 40.229000091552734, 40.229000091552734, 40.264503479003906, 40.264503479003906, 40.280799865722656, 40.35710144042969, 40.35710144042969, 40.42190170288086, 40.438899993896484, 40.438899993896484, 40.45790100097656, 40.472900390625, 40.472900390625, 40.617496490478516, 40.617496490478516, 40.617496490478516, 40.617496490478516, 40.68770217895508, 40.73379898071289, 40.73379898071289, 40.73379898071289, 40.790802001953125, 40.790802001953125, 40.81739807128906, 40.81739807128906, 40.819000244140625, 41.01259994506836, 41.01259994506836, 41.01259994506836, 41.01259994506836, 41.04820251464844, 41.05229949951172, 41.06310272216797, 41.08619689941406, 41.122802734375, 41.193599700927734, 41.208900451660156, 41.27210235595703, 41.36050033569336, 41.36050033569336, 41.387298583984375, 41.387298583984375, 41.387298583984375, 41.387298583984375, 41.387298583984375, 41.403099060058594, 41.403099060058594, 41.46659851074219, 41.46659851074219, 41.524200439453125, 41.524200439453125, 41.524200439453125, 41.64699935913086, 41.64699935913086, 41.64699935913086, 41.64699935913086, 41.64699935913086, 41.65639877319336, 41.69219970703125, 41.70909881591797, 41.70909881591797, 41.75910186767578, 41.75910186767578, 41.777000427246094, 41.822998046875, 41.822998046875, 41.82400131225586, 41.871002197265625, 41.92790222167969, 41.92790222167969, 41.939598083496094, 41.95130157470703, 41.95130157470703, 41.993099212646484, 41.993099212646484, 42.023399353027344, 42.04170227050781, 42.04170227050781, 42.04240036010742, 42.04240036010742, 42.08439636230469, 42.10540008544922, 42.11840057373047, 42.11840057373047, 42.18009948730469, 42.18009948730469, 42.18009948730469, 42.25330352783203, 42.26129913330078, 42.315399169921875, 42.33300018310547, 42.33300018310547, 42.333702087402344, 42.333702087402344, 42.33440399169922, 42.34280014038086, 42.34280014038086, 42.36689758300781, 42.40599822998047, 42.40599822998047, 42.40599822998047, 42.447601318359375, 42.447601318359375, 42.447601318359375, 42.450599670410156, 42.50619888305664, 42.50619888305664, 42.509498596191406, 42.51519775390625, 42.567100524902344, 42.567100524902344, 42.567100524902344, 42.567100524902344, 42.57019805908203, 42.57019805908203, 42.617000579833984, 42.617000579833984, 42.617000579833984, 42.634498596191406, 42.63669967651367, 42.63669967651367, 42.64240264892578, 42.658302307128906, 42.67359924316406, 42.67490005493164, 42.733699798583984, 42.733699798583984, 42.74899673461914, 42.75029754638672, 42.796302795410156, 42.82170104980469, 42.82170104980469, 42.82170104980469, 42.84389877319336, 42.84389877319336, 42.855499267578125, 42.92900085449219, 42.98680114746094, 43.10700225830078, 43.10700225830078, 43.10700225830078, 43.12879943847656, 43.12879943847656, 43.13710021972656, 43.17420196533203, 43.17420196533203, 43.220001220703125, 43.259803771972656, 43.259803771972656, 43.259803771972656, 43.264102935791016, 43.291297912597656, 43.291297912597656, 43.34020233154297, 43.4098014831543, 43.44519805908203, 43.523399353027344, 43.53940200805664, 43.53940200805664, 43.61399841308594, 43.642799377441406, 43.642799377441406, 43.659996032714844, 43.69129943847656, 43.72079849243164, 43.75969696044922, 43.75969696044922, 43.76570129394531, 43.76570129394531, 43.774200439453125, 43.82630157470703, 43.82630157470703, 43.83140182495117, 43.87419891357422, 43.87419891357422, 43.91510009765625, 43.91659927368164, 43.91659927368164, 43.939697265625, 43.939697265625, 43.960899353027344, 43.960899353027344, 44.001800537109375, 44.001800537109375, 44.010799407958984, 44.010799407958984, 44.0192985534668, 44.021400451660156, 44.021400451660156, 44.03179931640625, 44.03179931640625, 44.10559844970703, 44.10559844970703, 44.106903076171875, 44.139198303222656, 44.16960144042969, 44.17749786376953, 44.19929885864258, 44.20030212402344, 44.20030212402344, 44.21209716796875, 44.23870086669922, 44.23870086669922, 44.23870086669922, 44.23870086669922, 44.25309753417969, 44.25309753417969, 44.370399475097656, 44.370399475097656, 44.39099884033203, 44.39099884033203, 44.3922004699707, 44.41379928588867, 44.41659927368164, 44.42150115966797, 44.42759704589844, 44.43790054321289, 44.43790054321289, 44.441200256347656, 44.441200256347656, 44.481300354003906, 44.486202239990234, 44.486202239990234, 44.486202239990234, 44.557899475097656, 44.557899475097656, 44.574501037597656, 44.62940216064453, 44.62940216064453, 44.6510009765625, 44.6510009765625, 44.654197692871094, 44.654197692871094, 44.654197692871094, 44.654197692871094, 44.654197692871094, 44.73040008544922, 44.73040008544922, 44.75790023803711, 44.784202575683594, 44.820098876953125, 44.820098876953125, 44.877201080322266, 44.877201080322266, 44.877201080322266, 44.91510009765625, 44.9552001953125, 44.9552001953125, 44.995201110839844, 44.99800109863281, 44.99800109863281, 45.00870132446289, 45.036903381347656, 45.04629898071289, 45.04629898071289, 45.07569885253906, 45.07569885253906, 45.07740020751953, 45.100799560546875, 45.100799560546875, 45.12969970703125, 45.13800048828125, 45.13800048828125, 45.13800048828125, 45.13800048828125, 45.13800048828125, 45.14830017089844, 45.14830017089844, 45.16059875488281, 45.16059875488281, 45.161800384521484, 45.19169998168945, 45.19169998168945, 45.19839859008789, 45.19839859008789, 45.19839859008789, 45.212501525878906, 45.235496520996094, 45.235496520996094, 45.23860168457031, 45.250099182128906, 45.256099700927734, 45.263099670410156, 45.263099670410156, 45.32630157470703, 45.32630157470703, 45.32630157470703, 45.35820007324219, 45.41619873046875, 45.41619873046875, 45.41619873046875, 45.430301666259766, 45.430301666259766, 45.430301666259766, 45.442501068115234, 45.50360107421875, 45.518001556396484, 45.54719924926758, 45.54719924926758, 45.57209777832031, 45.57209777832031, 45.575199127197266, 45.597999572753906, 45.597999572753906, 45.597999572753906, 45.60110092163086, 45.63140106201172, 45.634700775146484, 45.65019989013672, 45.65019989013672, 45.68370056152344, 45.694698333740234, 45.694698333740234, 45.70539855957031, 45.70539855957031, 45.75309753417969, 45.78730010986328, 45.79669952392578, 45.8031005859375, 45.831398010253906, 45.831398010253906, 45.86940002441406, 45.896202087402344, 45.896202087402344, 45.896202087402344, 45.9176025390625, 45.9176025390625, 45.97840118408203, 45.97840118408203, 45.97840118408203, 45.994197845458984, 46.024200439453125, 46.024200439453125, 46.024200439453125, 46.03030014038086, 46.03030014038086, 46.03030014038086, 46.03209686279297, 46.03209686279297, 46.035301208496094, 46.035301208496094, 46.03879928588867, 46.03879928588867, 46.03879928588867, 46.03879928588867, 46.03879928588867, 46.03879928588867, 46.09819793701172, 46.099700927734375, 46.10639953613281, 46.13850021362305, 46.13909912109375, 46.13909912109375, 46.13909912109375, 46.14950180053711, 46.17829895019531, 46.246498107910156, 46.246498107910156, 46.29629898071289, 46.301795959472656, 46.301795959472656, 46.301795959472656, 46.33940124511719, 46.33940124511719, 46.35169982910156, 46.39540100097656, 46.39820098876953, 46.39820098876953, 46.42259979248047, 46.442298889160156, 46.442298889160156, 46.44300079345703, 46.44300079345703, 46.44300079345703, 46.44300079345703, 46.458499908447266, 46.458499908447266, 46.45909881591797, 46.588600158691406, 46.634700775146484, 46.64630126953125, 46.64970016479492, 46.64970016479492, 46.69350051879883, 46.69350051879883, 46.69350051879883, 46.69350051879883, 46.69350051879883, 46.70750045776367, 46.72270202636719, 46.726600646972656, 46.72669982910156, 46.7572021484375, 46.7572021484375, 46.76380157470703, 46.80329895019531, 46.80329895019531, 46.80329895019531, 46.80329895019531, 46.80329895019531, 46.80329895019531, 46.83830261230469, 46.83830261230469, 46.84170150756836, 46.86830139160156, 46.90620040893555, 46.98149871826172, 46.98149871826172, 47.016300201416016, 47.016300201416016, 47.016300201416016, 47.01930236816406, 47.027400970458984, 47.037200927734375, 47.037200927734375, 47.04139709472656, 47.05120086669922, 47.05120086669922, 47.05120086669922, 47.05120086669922, 47.06949996948242, 47.06949996948242, 47.147098541259766, 47.149200439453125, 47.3140983581543, 47.3140983581543, 47.318397521972656, 47.32849884033203, 47.34700012207031, 47.34700012207031, 47.34700012207031, 47.34700012207031, 47.354698181152344, 47.39120101928711, 47.39120101928711, 47.394500732421875, 47.4468994140625, 47.48179626464844, 47.48179626464844, 47.48179626464844, 47.50640106201172, 47.50640106201172, 47.51900100708008, 47.560699462890625, 47.560699462890625, 47.56420135498047, 47.586700439453125, 47.586700439453125, 47.589996337890625, 47.594398498535156, 47.594398498535156, 47.594398498535156, 47.65839767456055, 47.715301513671875, 47.74340057373047, 47.74340057373047, 47.746700286865234, 47.746700286865234, 47.77090072631836, 47.78369903564453, 47.78369903564453, 47.8135986328125, 47.827598571777344, 47.827598571777344, 47.830902099609375, 47.830902099609375, 47.84619903564453, 47.84619903564453, 47.84769821166992, 47.8494987487793, 47.855499267578125, 47.87459945678711, 47.87459945678711, 47.87459945678711, 47.886802673339844, 47.90769958496094, 47.90769958496094, 47.90769958496094, 47.91699981689453, 47.91699981689453, 47.920501708984375, 47.920501708984375, 47.948299407958984, 47.948299407958984, 47.948299407958984, 48.06120300292969, 48.06120300292969, 48.0869026184082, 48.0869026184082, 48.117698669433594, 48.12580108642578, 48.1525993347168, 48.1781005859375, 48.1781005859375, 48.23699951171875, 48.23699951171875, 48.29909896850586, 48.320098876953125, 48.320098876953125, 48.320098876953125, 48.32939910888672, 48.33290100097656, 48.37739944458008, 48.38209915161133, 48.3916015625, 48.39509963989258, 48.39509963989258, 48.39509963989258, 48.41189956665039, 48.427799224853516, 48.458099365234375, 48.458099365234375, 48.458099365234375, 48.47229766845703, 48.49120330810547, 48.492698669433594, 48.492698669433594, 48.49850082397461, 48.5098991394043, 48.530799865722656, 48.532901763916016, 48.532901763916016, 48.54560089111328, 48.54560089111328, 48.54560089111328, 48.54560089111328, 48.54560089111328, 48.555198669433594, 48.555198669433594, 48.555198669433594, 48.555198669433594, 48.566497802734375, 48.57609939575195, 48.59600067138672, 48.59600067138672, 48.655399322509766, 48.655399322509766, 48.683799743652344, 48.683799743652344, 48.683799743652344, 48.683799743652344, 48.683799743652344, 48.75490188598633, 48.756797790527344, 48.79520034790039, 48.79520034790039, 48.79520034790039, 48.811500549316406, 48.820701599121094, 48.820701599121094, 48.84459686279297, 48.84459686279297, 48.84459686279297, 48.871803283691406, 48.893402099609375, 48.907501220703125, 48.94129943847656, 48.94129943847656, 48.943599700927734, 48.94439697265625, 48.94439697265625, 48.94439697265625, 48.94670104980469, 49.02360153198242, 49.02360153198242, 49.09040069580078, 49.09040069580078, 49.09040069580078, 49.099300384521484, 49.1056022644043, 49.1056022644043, 49.1056022644043, 49.1056022644043, 49.1056022644043, 49.1255989074707, 49.1255989074707, 49.1255989074707, 49.14240264892578, 49.14240264892578, 49.19490051269531, 49.19490051269531, 49.19490051269531, 49.23500061035156, 49.23500061035156, 49.23500061035156, 49.23500061035156, 49.23500061035156, 49.26179885864258, 49.28280258178711, 49.3291015625, 49.331199645996094, 49.39209747314453, 49.39209747314453, 49.417999267578125, 49.42040252685547, 49.42040252685547, 49.44860076904297, 49.450897216796875, 49.450897216796875, 49.450897216796875, 49.480098724365234, 49.480098724365234, 49.480098724365234, 49.50619888305664, 49.50849914550781, 49.50849914550781, 49.50849914550781, 49.50849914550781, 49.50849914550781, 49.529998779296875, 49.529998779296875, 49.529998779296875, 49.55609893798828, 49.55609893798828, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.574501037597656, 49.623600006103516, 49.623600006103516, 49.623600006103516, 49.62730026245117, 49.62730026245117, 49.62730026245117, 49.689701080322266, 49.689701080322266, 49.69340133666992, 49.69770050048828, 49.7150993347168, 49.75140380859375, 49.78499984741211, 49.78499984741211, 49.831398010253906, 49.85869598388672, 49.85960006713867, 49.86499786376953, 49.86989974975586, 49.86989974975586, 49.86989974975586, 49.8948974609375, 49.8948974609375, 49.902099609375, 49.90370178222656, 49.90370178222656, 49.90370178222656, 49.90370178222656, 49.90370178222656, 49.90580368041992, 49.90739822387695, 49.913299560546875, 49.913299560546875, 49.919097900390625, 49.92449951171875, 49.92449951171875, 49.93890380859375, 49.93890380859375, 49.93890380859375, 49.94070053100586, 49.942298889160156, 50.00749969482422, 50.00749969482422, 50.00749969482422, 50.01900100708008, 50.01900100708008, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.0198974609375, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.02510070800781, 50.03179931640625, 50.03179931640625, 50.03179931640625, 50.03179931640625, 50.03179931640625, 50.03179931640625, 50.03179931640625, 50.033599853515625, 50.0697021484375, 50.0697021484375, 50.0697021484375, 50.0697021484375, 50.0697021484375, 50.0697021484375, 50.0697021484375, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.09000015258789, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.10919952392578, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11119842529297, 50.11669921875, 50.11669921875, 50.11669921875, 50.11869812011719, 50.11869812011719, 50.11869812011719, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.126399993896484, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13010025024414, 50.13209915161133, 50.18080139160156, 50.18080139160156, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.20389938354492, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875, 50.2322998046875]</t>
+          <t>[27.00040054321289, 27.51999855041504, 27.651599884033203, 27.930599212646484, 28.249801635742188, 28.249801635742188, 28.249801635742188, 28.249801635742188, 28.33810043334961, 29.196102142333984, 29.196102142333984, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.802900314331055, 29.802900314331055, 29.802900314331055, 29.802900314331055, 30.251001358032227, 30.561498641967773, 30.78059959411621, 30.78059959411621, 31.18670082092285, 31.331199645996094, 31.383899688720703, 31.383899688720703, 31.810699462890625, 31.89419937133789, 31.89419937133789, 32.12550354003906, 32.2035026550293, 32.60980224609375, 32.92279815673828, 32.92279815673828, 32.92279815673828, 32.92279815673828, 32.93149948120117, 32.93149948120117, 32.93149948120117, 33.12889862060547, 33.209999084472656, 33.45800018310547, 33.502403259277344, 33.502403259277344, 33.502403259277344, 33.5093994140625, 33.89929962158203, 33.89929962158203, 33.89929962158203, 33.89929962158203, 33.92559814453125, 34.108001708984375, 34.32680130004883, 34.32680130004883, 34.331199645996094, 34.6796989440918, 34.6796989440918, 34.701900482177734, 34.909202575683594, 34.909202575683594, 35.04280090332031, 35.04280090332031, 35.114097595214844, 35.114097595214844, 35.26150131225586, 35.27210235595703, 35.41720199584961, 35.57149887084961, 35.57149887084961, 35.71030044555664, 35.71030044555664, 35.858802795410156, 35.99290084838867, 36.2384033203125, 36.2384033203125, 36.2384033203125, 36.2384033203125, 36.280303955078125, 36.280303955078125, 36.283302307128906, 36.283302307128906, 36.34239959716797, 36.370201110839844, 36.44459915161133, 36.44459915161133, 36.51020050048828, 36.51020050048828, 36.561500549316406, 36.561500549316406, 36.603004455566406, 36.603004455566406, 36.603004455566406, 36.62480163574219, 36.64570236206055, 36.660797119140625, 36.660797119140625, 36.732398986816406, 36.732398986816406, 36.732398986816406, 36.84170150756836, 36.95580291748047, 36.967899322509766, 37.05950164794922, 37.05950164794922, 37.05950164794922, 37.062896728515625, 37.141998291015625, 37.27509689331055, 37.27509689331055, 37.2926025390625, 37.35639953613281, 37.35639953613281, 37.42729949951172, 37.42729949951172, 37.45840072631836, 37.45840072631836, 37.482601165771484, 37.538002014160156, 37.56230163574219, 37.56749725341797, 37.56749725341797, 37.56749725341797, 37.60340118408203, 37.60780334472656, 37.645999908447266, 37.645999908447266, 37.645999908447266, 37.65250015258789, 37.734901428222656, 37.80350112915039, 37.98210144042969, 37.98210144042969, 38.08219909667969, 38.13129806518555, 38.209800720214844, 38.21369934082031, 38.21369934082031, 38.30940246582031, 38.30940246582031, 38.33409881591797, 38.33409881591797, 38.36830139160156, 38.36830139160156, 38.36830139160156, 38.36830139160156, 38.36830139160156, 38.36830139160156, 38.42029571533203, 38.540000915527344, 38.540000915527344, 38.540000915527344, 38.583702087402344, 38.80400085449219, 38.82939910888672, 38.82939910888672, 38.86870193481445, 38.966102600097656, 38.966102600097656, 38.966102600097656, 39.14189910888672, 39.14189910888672, 39.1692008972168, 39.54399871826172, 39.54399871826172, 39.54399871826172, 39.70109939575195, 39.70109939575195, 39.70109939575195, 39.70109939575195, 39.74290466308594, 39.74290466308594, 39.74290466308594, 39.842803955078125, 39.842803955078125, 39.87459945678711, 39.87459945678711, 39.94920349121094, 39.94920349121094, 39.955902099609375, 39.978302001953125, 39.985198974609375, 40.02180099487305, 40.033103942871094, 40.033103942871094, 40.10340118408203, 40.10340118408203, 40.10340118408203, 40.112701416015625, 40.112701416015625, 40.2234001159668, 40.2234001159668, 40.250701904296875, 40.25080108642578, 40.25080108642578, 40.26340103149414, 40.3567008972168, 40.36830139160156, 40.36830139160156, 40.400001525878906, 40.486000061035156, 40.49970245361328, 40.49970245361328, 40.622802734375, 40.622802734375, 40.628700256347656, 40.628700256347656, 40.7046012878418, 40.7046012878418, 40.72880172729492, 40.731201171875, 40.747100830078125, 40.747100830078125, 40.75559997558594, 40.7692985534668, 40.8120002746582, 40.8120002746582, 40.92169952392578, 40.92169952392578, 40.955101013183594, 41.090702056884766, 41.090702056884766, 41.090702056884766, 41.090702056884766, 41.090702056884766, 41.090702056884766, 41.186195373535156, 41.23080062866211, 41.23080062866211, 41.36540222167969, 41.411800384521484, 41.467002868652344, 41.467002868652344, 41.46949768066406, 41.545196533203125, 41.545196533203125, 41.545196533203125, 41.545196533203125, 41.55549621582031, 41.55549621582031, 41.55549621582031, 41.578697204589844, 41.578697204589844, 41.62030029296875, 41.68939971923828, 41.68939971923828, 41.730098724365234, 41.730098724365234, 41.730098724365234, 41.784698486328125, 41.784698486328125, 41.784698486328125, 41.794898986816406, 41.794898986816406, 41.82550048828125, 41.82550048828125, 41.928199768066406, 41.95490264892578, 41.960304260253906, 41.99020004272461, 41.99020004272461, 42.20429992675781, 42.20429992675781, 42.20429992675781, 42.293601989746094, 42.322898864746094, 42.322898864746094, 42.38629913330078, 42.38629913330078, 42.38629913330078, 42.38629913330078, 42.419898986816406, 42.43890380859375, 42.45429992675781, 42.49399948120117, 42.49399948120117, 42.49399948120117, 42.49399948120117, 42.49399948120117, 42.49399948120117, 42.49399948120117, 42.4994010925293, 42.561302185058594, 42.6067008972168, 42.6067008972168, 42.608699798583984, 42.71289825439453, 42.743896484375, 42.75019836425781, 42.75019836425781, 42.75019836425781, 42.84990310668945, 43.04180145263672, 43.045799255371094, 43.045799255371094, 43.078800201416016, 43.153499603271484, 43.153499603271484, 43.153499603271484, 43.153499603271484, 43.18040084838867, 43.22380065917969, 43.22380065917969, 43.22380065917969, 43.233795166015625, 43.26359939575195, 43.26709747314453, 43.270301818847656, 43.270301818847656, 43.270301818847656, 43.279701232910156, 43.321800231933594, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.49939727783203, 43.5010986328125, 43.5010986328125, 43.5260009765625, 43.55940246582031, 43.57680130004883, 43.589698791503906, 43.62409973144531, 43.62409973144531, 43.625301361083984, 43.62860107421875, 43.62860107421875, 43.64939880371094, 43.69740295410156, 43.69740295410156, 43.71240234375, 43.71240234375, 43.71240234375, 43.71240234375, 43.789703369140625, 43.789703369140625, 43.789703369140625, 43.7942008972168, 43.7942008972168, 43.794403076171875, 43.80250549316406, 43.80699920654297, 43.85850143432617, 43.91339874267578, 43.93730163574219, 43.963401794433594, 43.963401794433594, 43.97010040283203, 43.97010040283203, 43.97010040283203, 44.01639938354492, 44.02439880371094, 44.02439880371094, 44.02439880371094, 44.08620071411133, 44.09920120239258, 44.12909698486328, 44.12909698486328, 44.12909698486328, 44.135498046875, 44.135498046875, 44.15660095214844, 44.18009948730469, 44.2052001953125, 44.23749923706055, 44.23749923706055, 44.26679992675781, 44.26679992675781, 44.28219985961914, 44.28219985961914, 44.28219985961914, 44.29520034790039, 44.31279754638672, 44.31549835205078, 44.34819793701172, 44.34819793701172, 44.37940216064453, 44.37940216064453, 44.39250183105469, 44.43830108642578, 44.43830108642578, 44.487300872802734, 44.487300872802734, 44.487300872802734, 44.54800033569336, 44.54800033569336, 44.595298767089844, 44.595298767089844, 44.6260986328125, 44.64690017700195, 44.64690017700195, 44.666099548339844, 44.70130157470703, 44.70130157470703, 44.72560119628906, 44.72560119628906, 45.08769989013672, 45.2025032043457, 45.3052978515625, 45.34449768066406, 45.34449768066406, 45.34449768066406, 45.34449768066406, 45.360198974609375, 45.37940216064453, 45.37940216064453, 45.3822021484375, 45.45790100097656, 45.47019958496094, 45.50669860839844, 45.55650329589844, 45.55650329589844, 45.56659698486328, 45.56659698486328, 45.57160186767578, 45.677696228027344, 45.677696228027344, 45.69300079345703, 45.70840072631836, 45.70840072631836, 45.70840072631836, 45.759498596191406, 45.825599670410156, 45.825599670410156, 45.825599670410156, 45.825599670410156, 45.833900451660156, 45.833900451660156, 45.85169982910156, 45.878700256347656, 45.8838005065918, 45.893001556396484, 45.893001556396484, 45.91379928588867, 45.92720031738281, 45.93770217895508, 45.96969985961914, 45.96969985961914, 45.989898681640625, 46.029300689697266, 46.029300689697266, 46.08689880371094, 46.08689880371094, 46.09000015258789, 46.10649871826172, 46.10649871826172, 46.117401123046875, 46.12630081176758, 46.141998291015625, 46.16790008544922, 46.182098388671875, 46.182098388671875, 46.195701599121094, 46.206298828125, 46.217796325683594, 46.25299835205078, 46.25299835205078, 46.25299835205078, 46.269996643066406, 46.32149887084961, 46.347198486328125, 46.37730026245117, 46.384002685546875, 46.384002685546875, 46.458099365234375, 46.458099365234375, 46.458099365234375, 46.458099365234375, 46.467498779296875, 46.467498779296875, 46.467498779296875, 46.467498779296875, 46.467498779296875, 46.484397888183594, 46.555702209472656, 46.627098083496094, 46.774200439453125, 46.845401763916016, 46.85310363769531, 46.85310363769531, 46.85310363769531, 46.868900299072266, 46.90950012207031, 46.90950012207031, 46.91340255737305, 46.98040008544922, 46.98040008544922, 46.989200592041016, 46.989200592041016, 47.002601623535156, 47.002601623535156, 47.08460235595703, 47.08720016479492, 47.17169952392578, 47.17169952392578, 47.17169952392578, 47.188201904296875, 47.19160079956055, 47.19160079956055, 47.20860290527344, 47.20860290527344, 47.211997985839844, 47.231101989746094, 47.231101989746094, 47.23310089111328, 47.240501403808594, 47.240501403808594, 47.268898010253906, 47.27960205078125, 47.299598693847656, 47.3218994140625, 47.326602935791016, 47.3369026184082, 47.3369026184082, 47.41680145263672, 47.42620086669922, 47.42620086669922, 47.42620086669922, 47.43090057373047, 47.47880172729492, 47.47880172729492, 47.482200622558594, 47.52000045776367, 47.528900146484375, 47.528900146484375, 47.535301208496094, 47.538902282714844, 47.538902282714844, 47.538902282714844, 47.54719924926758, 47.551700592041016, 47.55419921875, 47.565704345703125, 47.565704345703125, 47.5802001953125, 47.617698669433594, 47.617698669433594, 47.62339782714844, 47.62620162963867, 47.685699462890625, 47.687896728515625, 47.71699905395508, 47.71699905395508, 47.71710205078125, 47.73540115356445, 47.73540115356445, 47.74570083618164, 47.754302978515625, 47.754302978515625, 47.754302978515625, 47.777000427246094, 47.777000427246094, 47.777000427246094, 47.7952995300293, 47.7952995300293, 47.813697814941406, 47.81700134277344, 47.826499938964844, 47.8307991027832, 47.8307991027832, 47.85700225830078, 47.85700225830078, 47.97669982910156, 47.97669982910156, 47.988399505615234, 48.041603088378906, 48.041603088378906, 48.04930114746094, 48.10090255737305, 48.10090255737305, 48.10980224609375, 48.11750030517578, 48.1245002746582, 48.1245002746582, 48.1245002746582, 48.13999938964844, 48.13999938964844, 48.15570068359375, 48.237998962402344, 48.252899169921875, 48.2626953125, 48.2626953125, 48.268802642822266, 48.2698974609375, 48.2760009765625, 48.29050064086914, 48.3306999206543, 48.3306999206543, 48.33919906616211, 48.369300842285156, 48.369300842285156, 48.37670135498047, 48.42129898071289, 48.42129898071289, 48.42129898071289, 48.451900482177734, 48.465599060058594, 48.465599060058594, 48.465599060058594, 48.58360290527344, 48.58360290527344, 48.58360290527344, 48.597999572753906, 48.597999572753906, 48.597999572753906, 48.61250305175781, 48.61250305175781, 48.648399353027344, 48.64910125732422, 48.6599006652832, 48.67720031738281, 48.67720031738281, 48.72549819946289, 48.72549819946289, 48.72549819946289, 48.728599548339844, 48.728599548339844, 48.73570251464844, 48.73749923706055, 48.73749923706055, 48.73749923706055, 48.75230026245117, 48.75230026245117, 48.758201599121094, 48.78009796142578, 48.79199981689453, 48.79199981689453, 48.813201904296875, 48.823699951171875, 48.842002868652344, 48.842002868652344, 48.842002868652344, 48.846397399902344, 48.846397399902344, 48.846397399902344, 48.852500915527344, 48.852500915527344, 48.852500915527344, 48.852500915527344, 48.854801177978516, 48.86949920654297, 48.86949920654297, 48.87560272216797, 48.87989807128906, 48.87989807128906, 48.88390350341797, 48.891300201416016, 48.891300201416016, 48.911102294921875, 48.911102294921875, 48.911102294921875, 48.91480255126953, 48.91550064086914, 48.91729736328125, 48.960296630859375, 48.970497131347656, 48.970497131347656, 48.98429870605469, 48.98429870605469, 49.006202697753906, 49.007999420166016, 49.020599365234375, 49.029701232910156, 49.029701232910156, 49.041900634765625, 49.043701171875, 49.04810333251953, 49.053001403808594, 49.053001403808594, 49.053001403808594, 49.060401916503906, 49.06529998779297, 49.06599807739258, 49.06599807739258, 49.070701599121094, 49.15619659423828, 49.15619659423828, 49.15619659423828, 49.171199798583984, 49.17729949951172, 49.17729949951172, 49.19580078125, 49.197601318359375, 49.197601318359375, 49.198699951171875, 49.20050048828125, 49.211097717285156, 49.21139907836914, 49.2765998840332, 49.27690124511719, 49.27690124511719, 49.30030059814453, 49.314300537109375, 49.317298889160156, 49.3202018737793, 49.320899963378906, 49.320899963378906, 49.35009765625, 49.380401611328125, 49.4193000793457, 49.4193000793457, 49.430397033691406, 49.4901008605957, 49.49310302734375, 49.53559875488281, 49.54309844970703, 49.54309844970703, 49.54949951171875, 49.5625, 49.5625, 49.5625, 49.5625, 49.598201751708984, 49.598201751708984, 49.67179870605469, 49.67179870605469, 49.67179870605469, 49.7489013671875, 49.7489013671875, 49.7489013671875, 49.7489013671875, 49.7489013671875, 49.7489013671875, 49.75480270385742, 49.775001525878906, 49.775001525878906, 49.907100677490234, 49.907100677490234, 49.907100677490234, 49.93400192260742, 49.96030044555664, 49.97060012817383, 50.006500244140625, 50.006500244140625, 50.0458984375, 50.07469940185547, 50.08700180053711, 50.10660171508789, 50.109901428222656, 50.15439987182617, 50.18230056762695, 50.18230056762695, 50.20540237426758, 50.22209930419922, 50.22209930419922, 50.22209930419922, 50.23290252685547, 50.24040222167969, 50.24620056152344, 50.24620056152344, 50.24620056152344, 50.24620056152344, 50.25210189819336, 50.25210189819336, 50.26919937133789, 50.26919937133789, 50.27400207519531, 50.27400207519531, 50.27400207519531, 50.28020095825195, 50.28020095825195, 50.28450012207031, 50.29319763183594, 50.32250213623047, 50.33890151977539, 50.34989929199219, 50.35100173950195, 50.35100173950195, 50.35100173950195, 50.40739822387695, 50.40739822387695, 50.436100006103516, 50.436100006103516, 50.43769836425781, 50.43769836425781, 50.439796447753906, 50.44070053100586, 50.44070053100586, 50.44070053100586, 50.448997497558594, 50.464298248291016, 50.46500015258789, 50.52300262451172, 50.52300262451172, 50.52300262451172, 50.52370071411133, 50.541603088378906, 50.54509735107422, 50.547203063964844, 50.547698974609375, 50.547698974609375, 50.55120086669922, 50.55630111694336, 50.55630111694336, 50.55840301513672, 50.55840301513672, 50.55840301513672, 50.56919860839844, 50.56919860839844, 50.56919860839844, 50.56919860839844, 50.56919860839844, 50.56919860839844, 50.56919860839844, 50.595699310302734, 50.595699310302734, 50.60499954223633, 50.60499954223633, 50.60499954223633, 50.613399505615234, 50.620201110839844, 50.620201110839844, 50.62940216064453, 50.62940216064453, 50.644203186035156, 50.644203186035156, 50.64959716796875, 50.65599822998047, 50.697601318359375, 50.697601318359375, 50.70880126953125, 50.70880126953125, 50.72509765625, 50.730499267578125, 50.77260208129883, 50.77260208129883, 50.80860137939453, 50.84370040893555, 50.84370040893555, 50.84370040893555, 50.852901458740234, 50.888301849365234, 50.888301849365234, 50.888301849365234, 50.888301849365234, 50.888301849365234, 50.888301849365234, 50.888301849365234, 50.89229965209961, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.894203186035156, 50.89959716796875, 50.89959716796875, 50.89959716796875, 50.89959716796875, 50.915199279785156, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.925201416015625, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 51.022796630859375, 51.022796630859375, 51.022796630859375, 51.022796630859375, 51.073001861572266, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.13859558105469, 51.13859558105469, 51.13859558105469, 51.13859558105469, 51.13859558105469, 51.13859558105469, 51.14189910888672, 51.14189910888672, 51.14189910888672, 51.14189910888672, 51.14189910888672, 51.148597717285156, 51.153099060058594, 51.153099060058594, 51.159000396728516, 51.159000396728516, 51.159000396728516, 51.16830062866211, 51.16830062866211, 51.16830062866211, 51.16830062866211, 51.16830062866211, 51.18939971923828, 51.20320129394531, 51.20989990234375, 51.20989990234375, 51.20989990234375, 51.20989990234375, 51.20989990234375, 51.20989990234375, 51.23210144042969, 51.23210144042969, 51.23210144042969, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.3275032043457, 51.3275032043457, 51.3275032043457, 51.3275032043457, 51.3275032043457, 51.3275032043457, 51.3275032043457]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Save optimizer latest results
</commit_message>
<xml_diff>
--- a/results_fcgma/ResultsCompMethod.xlsx
+++ b/results_fcgma/ResultsCompMethod.xlsx
@@ -439,7 +439,7 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>[[0. 0. 0. ... 0. 0. 0.]
- [0. 0. 1. ... 0. 0. 0.]
+ [1. 0. 0. ... 0. 0. 0.]
  [0. 0. 0. ... 0. 0. 0.]
  ...
  [0. 0. 0. ... 0. 0. 0.]
@@ -448,11 +448,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>51.3275032043457</v>
+        <v>47.31919860839844</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[27.00040054321289, 27.51999855041504, 27.651599884033203, 27.930599212646484, 28.249801635742188, 28.249801635742188, 28.249801635742188, 28.249801635742188, 28.33810043334961, 29.196102142333984, 29.196102142333984, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.679698944091797, 29.802900314331055, 29.802900314331055, 29.802900314331055, 29.802900314331055, 30.251001358032227, 30.561498641967773, 30.78059959411621, 30.78059959411621, 31.18670082092285, 31.331199645996094, 31.383899688720703, 31.383899688720703, 31.810699462890625, 31.89419937133789, 31.89419937133789, 32.12550354003906, 32.2035026550293, 32.60980224609375, 32.92279815673828, 32.92279815673828, 32.92279815673828, 32.92279815673828, 32.93149948120117, 32.93149948120117, 32.93149948120117, 33.12889862060547, 33.209999084472656, 33.45800018310547, 33.502403259277344, 33.502403259277344, 33.502403259277344, 33.5093994140625, 33.89929962158203, 33.89929962158203, 33.89929962158203, 33.89929962158203, 33.92559814453125, 34.108001708984375, 34.32680130004883, 34.32680130004883, 34.331199645996094, 34.6796989440918, 34.6796989440918, 34.701900482177734, 34.909202575683594, 34.909202575683594, 35.04280090332031, 35.04280090332031, 35.114097595214844, 35.114097595214844, 35.26150131225586, 35.27210235595703, 35.41720199584961, 35.57149887084961, 35.57149887084961, 35.71030044555664, 35.71030044555664, 35.858802795410156, 35.99290084838867, 36.2384033203125, 36.2384033203125, 36.2384033203125, 36.2384033203125, 36.280303955078125, 36.280303955078125, 36.283302307128906, 36.283302307128906, 36.34239959716797, 36.370201110839844, 36.44459915161133, 36.44459915161133, 36.51020050048828, 36.51020050048828, 36.561500549316406, 36.561500549316406, 36.603004455566406, 36.603004455566406, 36.603004455566406, 36.62480163574219, 36.64570236206055, 36.660797119140625, 36.660797119140625, 36.732398986816406, 36.732398986816406, 36.732398986816406, 36.84170150756836, 36.95580291748047, 36.967899322509766, 37.05950164794922, 37.05950164794922, 37.05950164794922, 37.062896728515625, 37.141998291015625, 37.27509689331055, 37.27509689331055, 37.2926025390625, 37.35639953613281, 37.35639953613281, 37.42729949951172, 37.42729949951172, 37.45840072631836, 37.45840072631836, 37.482601165771484, 37.538002014160156, 37.56230163574219, 37.56749725341797, 37.56749725341797, 37.56749725341797, 37.60340118408203, 37.60780334472656, 37.645999908447266, 37.645999908447266, 37.645999908447266, 37.65250015258789, 37.734901428222656, 37.80350112915039, 37.98210144042969, 37.98210144042969, 38.08219909667969, 38.13129806518555, 38.209800720214844, 38.21369934082031, 38.21369934082031, 38.30940246582031, 38.30940246582031, 38.33409881591797, 38.33409881591797, 38.36830139160156, 38.36830139160156, 38.36830139160156, 38.36830139160156, 38.36830139160156, 38.36830139160156, 38.42029571533203, 38.540000915527344, 38.540000915527344, 38.540000915527344, 38.583702087402344, 38.80400085449219, 38.82939910888672, 38.82939910888672, 38.86870193481445, 38.966102600097656, 38.966102600097656, 38.966102600097656, 39.14189910888672, 39.14189910888672, 39.1692008972168, 39.54399871826172, 39.54399871826172, 39.54399871826172, 39.70109939575195, 39.70109939575195, 39.70109939575195, 39.70109939575195, 39.74290466308594, 39.74290466308594, 39.74290466308594, 39.842803955078125, 39.842803955078125, 39.87459945678711, 39.87459945678711, 39.94920349121094, 39.94920349121094, 39.955902099609375, 39.978302001953125, 39.985198974609375, 40.02180099487305, 40.033103942871094, 40.033103942871094, 40.10340118408203, 40.10340118408203, 40.10340118408203, 40.112701416015625, 40.112701416015625, 40.2234001159668, 40.2234001159668, 40.250701904296875, 40.25080108642578, 40.25080108642578, 40.26340103149414, 40.3567008972168, 40.36830139160156, 40.36830139160156, 40.400001525878906, 40.486000061035156, 40.49970245361328, 40.49970245361328, 40.622802734375, 40.622802734375, 40.628700256347656, 40.628700256347656, 40.7046012878418, 40.7046012878418, 40.72880172729492, 40.731201171875, 40.747100830078125, 40.747100830078125, 40.75559997558594, 40.7692985534668, 40.8120002746582, 40.8120002746582, 40.92169952392578, 40.92169952392578, 40.955101013183594, 41.090702056884766, 41.090702056884766, 41.090702056884766, 41.090702056884766, 41.090702056884766, 41.090702056884766, 41.186195373535156, 41.23080062866211, 41.23080062866211, 41.36540222167969, 41.411800384521484, 41.467002868652344, 41.467002868652344, 41.46949768066406, 41.545196533203125, 41.545196533203125, 41.545196533203125, 41.545196533203125, 41.55549621582031, 41.55549621582031, 41.55549621582031, 41.578697204589844, 41.578697204589844, 41.62030029296875, 41.68939971923828, 41.68939971923828, 41.730098724365234, 41.730098724365234, 41.730098724365234, 41.784698486328125, 41.784698486328125, 41.784698486328125, 41.794898986816406, 41.794898986816406, 41.82550048828125, 41.82550048828125, 41.928199768066406, 41.95490264892578, 41.960304260253906, 41.99020004272461, 41.99020004272461, 42.20429992675781, 42.20429992675781, 42.20429992675781, 42.293601989746094, 42.322898864746094, 42.322898864746094, 42.38629913330078, 42.38629913330078, 42.38629913330078, 42.38629913330078, 42.419898986816406, 42.43890380859375, 42.45429992675781, 42.49399948120117, 42.49399948120117, 42.49399948120117, 42.49399948120117, 42.49399948120117, 42.49399948120117, 42.49399948120117, 42.4994010925293, 42.561302185058594, 42.6067008972168, 42.6067008972168, 42.608699798583984, 42.71289825439453, 42.743896484375, 42.75019836425781, 42.75019836425781, 42.75019836425781, 42.84990310668945, 43.04180145263672, 43.045799255371094, 43.045799255371094, 43.078800201416016, 43.153499603271484, 43.153499603271484, 43.153499603271484, 43.153499603271484, 43.18040084838867, 43.22380065917969, 43.22380065917969, 43.22380065917969, 43.233795166015625, 43.26359939575195, 43.26709747314453, 43.270301818847656, 43.270301818847656, 43.270301818847656, 43.279701232910156, 43.321800231933594, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.36900329589844, 43.49939727783203, 43.5010986328125, 43.5010986328125, 43.5260009765625, 43.55940246582031, 43.57680130004883, 43.589698791503906, 43.62409973144531, 43.62409973144531, 43.625301361083984, 43.62860107421875, 43.62860107421875, 43.64939880371094, 43.69740295410156, 43.69740295410156, 43.71240234375, 43.71240234375, 43.71240234375, 43.71240234375, 43.789703369140625, 43.789703369140625, 43.789703369140625, 43.7942008972168, 43.7942008972168, 43.794403076171875, 43.80250549316406, 43.80699920654297, 43.85850143432617, 43.91339874267578, 43.93730163574219, 43.963401794433594, 43.963401794433594, 43.97010040283203, 43.97010040283203, 43.97010040283203, 44.01639938354492, 44.02439880371094, 44.02439880371094, 44.02439880371094, 44.08620071411133, 44.09920120239258, 44.12909698486328, 44.12909698486328, 44.12909698486328, 44.135498046875, 44.135498046875, 44.15660095214844, 44.18009948730469, 44.2052001953125, 44.23749923706055, 44.23749923706055, 44.26679992675781, 44.26679992675781, 44.28219985961914, 44.28219985961914, 44.28219985961914, 44.29520034790039, 44.31279754638672, 44.31549835205078, 44.34819793701172, 44.34819793701172, 44.37940216064453, 44.37940216064453, 44.39250183105469, 44.43830108642578, 44.43830108642578, 44.487300872802734, 44.487300872802734, 44.487300872802734, 44.54800033569336, 44.54800033569336, 44.595298767089844, 44.595298767089844, 44.6260986328125, 44.64690017700195, 44.64690017700195, 44.666099548339844, 44.70130157470703, 44.70130157470703, 44.72560119628906, 44.72560119628906, 45.08769989013672, 45.2025032043457, 45.3052978515625, 45.34449768066406, 45.34449768066406, 45.34449768066406, 45.34449768066406, 45.360198974609375, 45.37940216064453, 45.37940216064453, 45.3822021484375, 45.45790100097656, 45.47019958496094, 45.50669860839844, 45.55650329589844, 45.55650329589844, 45.56659698486328, 45.56659698486328, 45.57160186767578, 45.677696228027344, 45.677696228027344, 45.69300079345703, 45.70840072631836, 45.70840072631836, 45.70840072631836, 45.759498596191406, 45.825599670410156, 45.825599670410156, 45.825599670410156, 45.825599670410156, 45.833900451660156, 45.833900451660156, 45.85169982910156, 45.878700256347656, 45.8838005065918, 45.893001556396484, 45.893001556396484, 45.91379928588867, 45.92720031738281, 45.93770217895508, 45.96969985961914, 45.96969985961914, 45.989898681640625, 46.029300689697266, 46.029300689697266, 46.08689880371094, 46.08689880371094, 46.09000015258789, 46.10649871826172, 46.10649871826172, 46.117401123046875, 46.12630081176758, 46.141998291015625, 46.16790008544922, 46.182098388671875, 46.182098388671875, 46.195701599121094, 46.206298828125, 46.217796325683594, 46.25299835205078, 46.25299835205078, 46.25299835205078, 46.269996643066406, 46.32149887084961, 46.347198486328125, 46.37730026245117, 46.384002685546875, 46.384002685546875, 46.458099365234375, 46.458099365234375, 46.458099365234375, 46.458099365234375, 46.467498779296875, 46.467498779296875, 46.467498779296875, 46.467498779296875, 46.467498779296875, 46.484397888183594, 46.555702209472656, 46.627098083496094, 46.774200439453125, 46.845401763916016, 46.85310363769531, 46.85310363769531, 46.85310363769531, 46.868900299072266, 46.90950012207031, 46.90950012207031, 46.91340255737305, 46.98040008544922, 46.98040008544922, 46.989200592041016, 46.989200592041016, 47.002601623535156, 47.002601623535156, 47.08460235595703, 47.08720016479492, 47.17169952392578, 47.17169952392578, 47.17169952392578, 47.188201904296875, 47.19160079956055, 47.19160079956055, 47.20860290527344, 47.20860290527344, 47.211997985839844, 47.231101989746094, 47.231101989746094, 47.23310089111328, 47.240501403808594, 47.240501403808594, 47.268898010253906, 47.27960205078125, 47.299598693847656, 47.3218994140625, 47.326602935791016, 47.3369026184082, 47.3369026184082, 47.41680145263672, 47.42620086669922, 47.42620086669922, 47.42620086669922, 47.43090057373047, 47.47880172729492, 47.47880172729492, 47.482200622558594, 47.52000045776367, 47.528900146484375, 47.528900146484375, 47.535301208496094, 47.538902282714844, 47.538902282714844, 47.538902282714844, 47.54719924926758, 47.551700592041016, 47.55419921875, 47.565704345703125, 47.565704345703125, 47.5802001953125, 47.617698669433594, 47.617698669433594, 47.62339782714844, 47.62620162963867, 47.685699462890625, 47.687896728515625, 47.71699905395508, 47.71699905395508, 47.71710205078125, 47.73540115356445, 47.73540115356445, 47.74570083618164, 47.754302978515625, 47.754302978515625, 47.754302978515625, 47.777000427246094, 47.777000427246094, 47.777000427246094, 47.7952995300293, 47.7952995300293, 47.813697814941406, 47.81700134277344, 47.826499938964844, 47.8307991027832, 47.8307991027832, 47.85700225830078, 47.85700225830078, 47.97669982910156, 47.97669982910156, 47.988399505615234, 48.041603088378906, 48.041603088378906, 48.04930114746094, 48.10090255737305, 48.10090255737305, 48.10980224609375, 48.11750030517578, 48.1245002746582, 48.1245002746582, 48.1245002746582, 48.13999938964844, 48.13999938964844, 48.15570068359375, 48.237998962402344, 48.252899169921875, 48.2626953125, 48.2626953125, 48.268802642822266, 48.2698974609375, 48.2760009765625, 48.29050064086914, 48.3306999206543, 48.3306999206543, 48.33919906616211, 48.369300842285156, 48.369300842285156, 48.37670135498047, 48.42129898071289, 48.42129898071289, 48.42129898071289, 48.451900482177734, 48.465599060058594, 48.465599060058594, 48.465599060058594, 48.58360290527344, 48.58360290527344, 48.58360290527344, 48.597999572753906, 48.597999572753906, 48.597999572753906, 48.61250305175781, 48.61250305175781, 48.648399353027344, 48.64910125732422, 48.6599006652832, 48.67720031738281, 48.67720031738281, 48.72549819946289, 48.72549819946289, 48.72549819946289, 48.728599548339844, 48.728599548339844, 48.73570251464844, 48.73749923706055, 48.73749923706055, 48.73749923706055, 48.75230026245117, 48.75230026245117, 48.758201599121094, 48.78009796142578, 48.79199981689453, 48.79199981689453, 48.813201904296875, 48.823699951171875, 48.842002868652344, 48.842002868652344, 48.842002868652344, 48.846397399902344, 48.846397399902344, 48.846397399902344, 48.852500915527344, 48.852500915527344, 48.852500915527344, 48.852500915527344, 48.854801177978516, 48.86949920654297, 48.86949920654297, 48.87560272216797, 48.87989807128906, 48.87989807128906, 48.88390350341797, 48.891300201416016, 48.891300201416016, 48.911102294921875, 48.911102294921875, 48.911102294921875, 48.91480255126953, 48.91550064086914, 48.91729736328125, 48.960296630859375, 48.970497131347656, 48.970497131347656, 48.98429870605469, 48.98429870605469, 49.006202697753906, 49.007999420166016, 49.020599365234375, 49.029701232910156, 49.029701232910156, 49.041900634765625, 49.043701171875, 49.04810333251953, 49.053001403808594, 49.053001403808594, 49.053001403808594, 49.060401916503906, 49.06529998779297, 49.06599807739258, 49.06599807739258, 49.070701599121094, 49.15619659423828, 49.15619659423828, 49.15619659423828, 49.171199798583984, 49.17729949951172, 49.17729949951172, 49.19580078125, 49.197601318359375, 49.197601318359375, 49.198699951171875, 49.20050048828125, 49.211097717285156, 49.21139907836914, 49.2765998840332, 49.27690124511719, 49.27690124511719, 49.30030059814453, 49.314300537109375, 49.317298889160156, 49.3202018737793, 49.320899963378906, 49.320899963378906, 49.35009765625, 49.380401611328125, 49.4193000793457, 49.4193000793457, 49.430397033691406, 49.4901008605957, 49.49310302734375, 49.53559875488281, 49.54309844970703, 49.54309844970703, 49.54949951171875, 49.5625, 49.5625, 49.5625, 49.5625, 49.598201751708984, 49.598201751708984, 49.67179870605469, 49.67179870605469, 49.67179870605469, 49.7489013671875, 49.7489013671875, 49.7489013671875, 49.7489013671875, 49.7489013671875, 49.7489013671875, 49.75480270385742, 49.775001525878906, 49.775001525878906, 49.907100677490234, 49.907100677490234, 49.907100677490234, 49.93400192260742, 49.96030044555664, 49.97060012817383, 50.006500244140625, 50.006500244140625, 50.0458984375, 50.07469940185547, 50.08700180053711, 50.10660171508789, 50.109901428222656, 50.15439987182617, 50.18230056762695, 50.18230056762695, 50.20540237426758, 50.22209930419922, 50.22209930419922, 50.22209930419922, 50.23290252685547, 50.24040222167969, 50.24620056152344, 50.24620056152344, 50.24620056152344, 50.24620056152344, 50.25210189819336, 50.25210189819336, 50.26919937133789, 50.26919937133789, 50.27400207519531, 50.27400207519531, 50.27400207519531, 50.28020095825195, 50.28020095825195, 50.28450012207031, 50.29319763183594, 50.32250213623047, 50.33890151977539, 50.34989929199219, 50.35100173950195, 50.35100173950195, 50.35100173950195, 50.40739822387695, 50.40739822387695, 50.436100006103516, 50.436100006103516, 50.43769836425781, 50.43769836425781, 50.439796447753906, 50.44070053100586, 50.44070053100586, 50.44070053100586, 50.448997497558594, 50.464298248291016, 50.46500015258789, 50.52300262451172, 50.52300262451172, 50.52300262451172, 50.52370071411133, 50.541603088378906, 50.54509735107422, 50.547203063964844, 50.547698974609375, 50.547698974609375, 50.55120086669922, 50.55630111694336, 50.55630111694336, 50.55840301513672, 50.55840301513672, 50.55840301513672, 50.56919860839844, 50.56919860839844, 50.56919860839844, 50.56919860839844, 50.56919860839844, 50.56919860839844, 50.56919860839844, 50.595699310302734, 50.595699310302734, 50.60499954223633, 50.60499954223633, 50.60499954223633, 50.613399505615234, 50.620201110839844, 50.620201110839844, 50.62940216064453, 50.62940216064453, 50.644203186035156, 50.644203186035156, 50.64959716796875, 50.65599822998047, 50.697601318359375, 50.697601318359375, 50.70880126953125, 50.70880126953125, 50.72509765625, 50.730499267578125, 50.77260208129883, 50.77260208129883, 50.80860137939453, 50.84370040893555, 50.84370040893555, 50.84370040893555, 50.852901458740234, 50.888301849365234, 50.888301849365234, 50.888301849365234, 50.888301849365234, 50.888301849365234, 50.888301849365234, 50.888301849365234, 50.89229965209961, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.893402099609375, 50.894203186035156, 50.89959716796875, 50.89959716796875, 50.89959716796875, 50.89959716796875, 50.915199279785156, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.91539764404297, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.92469787597656, 50.925201416015625, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.94609832763672, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 50.96670150756836, 51.022796630859375, 51.022796630859375, 51.022796630859375, 51.022796630859375, 51.073001861572266, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.0740966796875, 51.13859558105469, 51.13859558105469, 51.13859558105469, 51.13859558105469, 51.13859558105469, 51.13859558105469, 51.14189910888672, 51.14189910888672, 51.14189910888672, 51.14189910888672, 51.14189910888672, 51.148597717285156, 51.153099060058594, 51.153099060058594, 51.159000396728516, 51.159000396728516, 51.159000396728516, 51.16830062866211, 51.16830062866211, 51.16830062866211, 51.16830062866211, 51.16830062866211, 51.18939971923828, 51.20320129394531, 51.20989990234375, 51.20989990234375, 51.20989990234375, 51.20989990234375, 51.20989990234375, 51.20989990234375, 51.23210144042969, 51.23210144042969, 51.23210144042969, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.24440002441406, 51.3275032043457, 51.3275032043457, 51.3275032043457, 51.3275032043457, 51.3275032043457, 51.3275032043457, 51.3275032043457]</t>
+          <t>[27.264699935913086, 27.59079933166504, 27.71940040588379, 27.791400909423828, 28.06760025024414, 28.322898864746094, 28.322898864746094, 28.322898864746094, 28.322898864746094, 28.322898864746094, 28.322898864746094, 28.47589874267578, 28.494701385498047, 28.494701385498047, 29.446300506591797, 29.446300506591797, 29.446300506591797, 29.446300506591797, 29.446300506591797, 29.446300506591797, 29.446300506591797, 29.46990203857422, 29.46990203857422, 29.72249984741211, 29.96860122680664, 29.96860122680664, 29.96860122680664, 29.96860122680664, 30.111400604248047, 30.111400604248047, 30.368297576904297, 30.447898864746094, 30.447898864746094, 30.563800811767578, 30.626399993896484, 30.639198303222656, 30.73740005493164, 30.73740005493164, 30.751998901367188, 30.751998901367188, 30.871299743652344, 31.237098693847656, 31.237098693847656, 31.237098693847656, 31.237098693847656, 31.589801788330078, 31.589801788330078, 31.70349884033203, 31.70349884033203, 31.773300170898438, 31.823400497436523, 32.16699981689453, 32.16699981689453, 32.41619873046875, 32.41619873046875, 32.41619873046875, 32.41619873046875, 32.41619873046875, 32.41619873046875, 32.46710205078125, 32.46710205078125, 32.46710205078125, 32.54969787597656, 32.54969787597656, 32.65480041503906, 32.65480041503906, 32.704200744628906, 32.704200744628906, 32.80229949951172, 32.89759826660156, 32.89759826660156, 32.89759826660156, 32.9989013671875, 33.029701232910156, 33.029701232910156, 33.049598693847656, 33.059200286865234, 33.06779861450195, 33.075401306152344, 33.075401306152344, 33.075401306152344, 33.14419937133789, 33.169498443603516, 33.20390319824219, 33.26249694824219, 33.3235969543457, 33.3235969543457, 33.372398376464844, 33.457496643066406, 33.55889892578125, 33.57969665527344, 33.598697662353516, 33.67020034790039, 33.71310043334961, 33.755401611328125, 33.88639831542969, 33.95560073852539, 33.95560073852539, 33.95560073852539, 34.0458984375, 34.0458984375, 34.0609016418457, 34.08660125732422, 34.20840072631836, 34.20840072631836, 34.211299896240234, 34.339202880859375, 34.36140060424805, 34.36140060424805, 34.36140060424805, 34.385799407958984, 34.39299774169922, 34.39299774169922, 34.45090103149414, 34.520599365234375, 34.520599365234375, 34.520599365234375, 34.520599365234375, 34.520599365234375, 34.52570343017578, 34.52570343017578, 34.531097412109375, 34.545799255371094, 34.56300354003906, 34.56300354003906, 34.56300354003906, 34.58270263671875, 34.58270263671875, 34.60060119628906, 34.75299835205078, 34.78849792480469, 34.81560134887695, 34.81560134887695, 34.81560134887695, 34.91590118408203, 35.08789825439453, 35.08789825439453, 35.08789825439453, 35.10150146484375, 35.10150146484375, 35.12710189819336, 35.15520095825195, 35.19960021972656, 35.200096130371094, 35.200096130371094, 35.27090072631836, 35.27090072631836, 35.27090072631836, 35.32040023803711, 35.32040023803711, 35.36410140991211, 35.382598876953125, 35.393898010253906, 35.413902282714844, 35.43440246582031, 35.43440246582031, 35.44559860229492, 35.44670104980469, 35.46630096435547, 35.472999572753906, 35.553001403808594, 35.553001403808594, 35.562599182128906, 35.596099853515625, 35.596099853515625, 35.64219665527344, 35.68970489501953, 35.68970489501953, 35.69750213623047, 35.7056999206543, 35.7056999206543, 35.72249984741211, 35.72249984741211, 35.785301208496094, 35.821197509765625, 35.821197509765625, 35.821197509765625, 35.869903564453125, 35.869903564453125, 35.869903564453125, 35.869903564453125, 35.869903564453125, 35.95830154418945, 35.95830154418945, 35.96149826049805, 35.964698791503906, 35.964698791503906, 36.00080108642578, 36.006202697753906, 36.03150177001953, 36.03150177001953, 36.03150177001953, 36.03369903564453, 36.03369903564453, 36.047000885009766, 36.09259796142578, 36.11330032348633, 36.11370086669922, 36.14520263671875, 36.16259765625, 36.16259765625, 36.20199966430664, 36.20949935913086, 36.20949935913086, 36.25419998168945, 36.25419998168945, 36.25669860839844, 36.3052978515625, 36.3052978515625, 36.37670135498047, 36.37670135498047, 36.37670135498047, 36.50230026245117, 36.50230026245117, 36.51799774169922, 36.51799774169922, 36.53810119628906, 36.53810119628906, 36.59700012207031, 36.59700012207031, 36.59700012207031, 36.59700012207031, 36.631099700927734, 36.79010009765625, 36.79010009765625, 36.79010009765625, 37.003299713134766, 37.003299713134766, 37.003299713134766, 37.003299713134766, 37.003299713134766, 37.025299072265625, 37.025299072265625, 37.05010223388672, 37.05010223388672, 37.08110046386719, 37.087196350097656, 37.11899948120117, 37.371803283691406, 37.37670135498047, 37.37670135498047, 37.37670135498047, 37.45020294189453, 37.52330017089844, 37.52330017089844, 37.579898834228516, 37.60409927368164, 37.60409927368164, 37.67720031738281, 37.67720031738281, 37.691200256347656, 37.743099212646484, 37.743099212646484, 37.743099212646484, 37.773597717285156, 37.77989959716797, 37.781898498535156, 37.781898498535156, 37.80839920043945, 37.81050109863281, 37.82939910888672, 37.86530303955078, 37.90310287475586, 37.935302734375, 37.99140167236328, 37.99140167236328, 38.02629852294922, 38.06880187988281, 38.122802734375, 38.122802734375, 38.1510009765625, 38.16539764404297, 38.23670196533203, 38.23670196533203, 38.23670196533203, 38.26329803466797, 38.328800201416016, 38.328800201416016, 38.38119888305664, 38.390602111816406, 38.390602111816406, 38.407798767089844, 38.407798767089844, 38.43239974975586, 38.52199935913086, 38.52199935913086, 38.52199935913086, 38.57659912109375, 38.633602142333984, 38.67359924316406, 38.68260192871094, 38.68260192871094, 38.69350051879883, 38.72819900512695, 38.72819900512695, 38.74109649658203, 38.74470138549805, 38.76429748535156, 38.76429748535156, 38.76429748535156, 38.76429748535156, 38.81520080566406, 38.81520080566406, 38.8203010559082, 38.8203010559082, 38.84020233154297, 38.842498779296875, 38.842498779296875, 38.90800094604492, 38.90800094604492, 38.928001403808594, 38.94649887084961, 38.94649887084961, 38.95750045776367, 39.057403564453125, 39.057403564453125, 39.166500091552734, 39.198097229003906, 39.198097229003906, 39.198097229003906, 39.198097229003906, 39.19830322265625, 39.25499725341797, 39.26740264892578, 39.26740264892578, 39.29119873046875, 39.31019973754883, 39.31019973754883, 39.35980224609375, 39.35980224609375, 39.38850021362305, 39.38850021362305, 39.42319869995117, 39.43050003051758, 39.43220138549805, 39.43989944458008, 39.44949722290039, 39.605098724365234, 39.605098724365234, 39.64459991455078, 39.64679718017578, 39.64679718017578, 39.64679718017578, 39.64679718017578, 39.65520095825195, 39.66440200805664, 39.6708984375, 39.6708984375, 39.67259979248047, 39.67259979248047, 39.69239807128906, 39.69239807128906, 39.692501068115234, 39.692501068115234, 39.753700256347656, 39.753700256347656, 39.75379943847656, 39.75379943847656, 39.75379943847656, 39.75640106201172, 39.85009765625, 39.85009765625, 39.852699279785156, 39.852699279785156, 39.948699951171875, 39.948699951171875, 39.9723014831543, 39.9723014831543, 40.05280303955078, 40.05280303955078, 40.05280303955078, 40.05280303955078, 40.077701568603516, 40.086700439453125, 40.09640121459961, 40.09640121459961, 40.156898498535156, 40.19620132446289, 40.21770095825195, 40.21770095825195, 40.228797912597656, 40.230201721191406, 40.235801696777344, 40.235801696777344, 40.242698669433594, 40.242698669433594, 40.242698669433594, 40.26170349121094, 40.29650115966797, 40.29650115966797, 40.32550048828125, 40.32550048828125, 40.3297004699707, 40.33580017089844, 40.33580017089844, 40.33580017089844, 40.36869812011719, 40.36869812011719, 40.36869812011719, 40.438899993896484, 40.438899993896484, 40.51350021362305, 40.53310012817383, 40.53940200805664, 40.5536994934082, 40.5536994934082, 40.55439758300781, 40.557899475097656, 40.626502990722656, 40.626502990722656, 40.65800094604492, 40.65800094604492, 40.67559814453125, 40.67559814453125, 40.689598083496094, 40.708702087402344, 40.708702087402344, 40.79010009765625, 40.79010009765625, 40.87809753417969, 40.87809753417969, 40.87809753417969, 40.87809753417969, 40.87809753417969, 40.87809753417969, 40.87809753417969, 40.87809753417969, 40.910301208496094, 40.91999816894531, 40.91999816894531, 40.93130111694336, 40.931400299072266, 40.97010040283203, 40.97949981689453, 40.97949981689453, 40.97949981689453, 40.97949981689453, 41.082000732421875, 41.082000732421875, 41.13719940185547, 41.17939758300781, 41.17939758300781, 41.23740005493164, 41.23740005493164, 41.26850128173828, 41.291099548339844, 41.39540100097656, 41.39540100097656, 41.40049743652344, 41.40049743652344, 41.42179870605469, 41.42179870605469, 41.447601318359375, 41.447601318359375, 41.45490264892578, 41.45490264892578, 41.45490264892578, 41.48040008544922, 41.535499572753906, 41.535499572753906, 41.543800354003906, 41.543800354003906, 41.55760192871094, 41.56209945678711, 41.566200256347656, 41.58060073852539, 41.591896057128906, 41.591896057128906, 41.622596740722656, 41.622596740722656, 41.6531982421875, 41.6531982421875, 41.66529846191406, 41.68280029296875, 41.68280029296875, 41.68370056152344, 41.70399856567383, 41.70399856567383, 41.70399856567383, 41.76390075683594, 41.78960037231445, 41.80179977416992, 41.81019592285156, 41.81449890136719, 41.81449890136719, 41.863399505615234, 41.87300109863281, 41.88990020751953, 41.89070129394531, 41.91680145263672, 41.936500549316406, 41.936500549316406, 41.936500549316406, 41.93769836425781, 41.94059753417969, 41.95659637451172, 41.998802185058594, 41.998802185058594, 41.998802185058594, 42.03919982910156, 42.05550003051758, 42.05550003051758, 42.05550003051758, 42.05550003051758, 42.08180236816406, 42.108001708984375, 42.11009979248047, 42.11009979248047, 42.198699951171875, 42.22570037841797, 42.22570037841797, 42.311302185058594, 42.311302185058594, 42.32889938354492, 42.32889938354492, 42.32889938354492, 42.3400993347168, 42.36069869995117, 42.38050079345703, 42.407100677490234, 42.41389846801758, 42.450599670410156, 42.60369873046875, 42.64139938354492, 42.6870002746582, 42.6870002746582, 42.68920135498047, 42.68920135498047, 42.731101989746094, 42.731101989746094, 42.74909973144531, 42.74909973144531, 42.75899887084961, 42.75899887084961, 42.813499450683594, 42.813499450683594, 42.86149978637695, 42.867698669433594, 42.872802734375, 42.881797790527344, 42.88800048828125, 42.95589828491211, 42.95589828491211, 42.976600646972656, 42.987998962402344, 43.05099868774414, 43.066200256347656, 43.066200256347656, 43.066200256347656, 43.121002197265625, 43.121002197265625, 43.122901916503906, 43.122901916503906, 43.147300720214844, 43.15260314941406, 43.15260314941406, 43.173004150390625, 43.1781005859375, 43.1781005859375, 43.197601318359375, 43.22270202636719, 43.262901306152344, 43.262901306152344, 43.26449966430664, 43.26449966430664, 43.26449966430664, 43.336402893066406, 43.336402893066406, 43.34040069580078, 43.354400634765625, 43.3577995300293, 43.3577995300293, 43.515403747558594, 43.515403747558594, 43.55480194091797, 43.555397033691406, 43.555397033691406, 43.555397033691406, 43.555397033691406, 43.555397033691406, 43.555397033691406, 43.598899841308594, 43.598899841308594, 43.60639953613281, 43.61070251464844, 43.61070251464844, 43.61070251464844, 43.613101959228516, 43.650001525878906, 43.67879867553711, 43.733299255371094, 43.733299255371094, 43.805397033691406, 43.805397033691406, 43.827301025390625, 43.827301025390625, 43.827301025390625, 43.827301025390625, 43.827301025390625, 43.91050338745117, 43.93060302734375, 43.93880081176758, 43.93880081176758, 43.93880081176758, 43.95390319824219, 43.982200622558594, 43.982200622558594, 44.01210021972656, 44.01210021972656, 44.01210021972656, 44.018798828125, 44.018798828125, 44.02090072631836, 44.02090072631836, 44.04100036621094, 44.04100036621094, 44.04100036621094, 44.04100036621094, 44.04100036621094, 44.27189636230469, 44.301597595214844, 44.301597595214844, 44.301597595214844, 44.30270004272461, 44.30270004272461, 44.30270004272461, 44.30270004272461, 44.30270004272461, 44.30270004272461, 44.30550003051758, 44.30550003051758, 44.35169982910156, 44.353797912597656, 44.353797912597656, 44.41189956665039, 44.424400329589844, 44.424400329589844, 44.42509841918945, 44.43659973144531, 44.46870040893555, 44.52320098876953, 44.52320098876953, 44.52389907836914, 44.52389907836914, 44.52549743652344, 44.52549743652344, 44.52549743652344, 44.52549743652344, 44.59579849243164, 44.59579849243164, 44.61750030517578, 44.63199996948242, 44.63199996948242, 44.665496826171875, 44.665496826171875, 44.672698974609375, 44.696502685546875, 44.696502685546875, 44.70600128173828, 44.70600128173828, 44.741600036621094, 44.741600036621094, 44.741600036621094, 44.741600036621094, 44.76799774169922, 44.771697998046875, 44.836700439453125, 44.845802307128906, 44.869598388671875, 44.869598388671875, 44.869598388671875, 44.869598388671875, 44.869598388671875, 44.88140106201172, 44.88570022583008, 44.88610076904297, 44.90079879760742, 44.91270065307617, 44.91270065307617, 44.94309997558594, 44.94309997558594, 44.968101501464844, 44.98619842529297, 44.997798919677734, 44.997798919677734, 45.034202575683594, 45.056297302246094, 45.056297302246094, 45.10020065307617, 45.10020065307617, 45.10020065307617, 45.1068000793457, 45.1068000793457, 45.16790008544922, 45.16790008544922, 45.16790008544922, 45.173500061035156, 45.173500061035156, 45.24209976196289, 45.24209976196289, 45.25029754638672, 45.25029754638672, 45.253997802734375, 45.32469940185547, 45.33100128173828, 45.33100128173828, 45.347496032714844, 45.347496032714844, 45.35029983520508, 45.36170196533203, 45.41210174560547, 45.46549987792969, 45.476402282714844, 45.49720001220703, 45.49720001220703, 45.527801513671875, 45.527801513671875, 45.527801513671875, 45.53099822998047, 45.53099822998047, 45.53099822998047, 45.593997955322266, 45.593997955322266, 45.64240264892578, 45.64240264892578, 45.64670181274414, 45.64670181274414, 45.652000427246094, 45.679100036621094, 45.679100036621094, 45.688697814941406, 45.69609832763672, 45.69609832763672, 45.703697204589844, 45.703697204589844, 45.73609924316406, 45.78810119628906, 45.78810119628906, 45.78810119628906, 45.78810119628906, 45.805599212646484, 45.805599212646484, 45.805599212646484, 45.805599212646484, 45.821800231933594, 45.833396911621094, 45.833396911621094, 45.83899688720703, 45.86219787597656, 45.86219787597656, 45.86650085449219, 45.86650085449219, 45.86650085449219, 45.87940216064453, 45.900299072265625, 45.90800094604492, 45.95180130004883, 45.95180130004883, 45.97719955444336, 45.97719955444336, 45.97719955444336, 45.97719955444336, 46.00379943847656, 46.00379943847656, 46.00520324707031, 46.009498596191406, 46.027400970458984, 46.027400970458984, 46.027400970458984, 46.027400970458984, 46.027400970458984, 46.027400970458984, 46.027400970458984, 46.027400970458984, 46.027400970458984, 46.027400970458984, 46.03820037841797, 46.03820037841797, 46.05950164794922, 46.081298828125, 46.081600189208984, 46.08509826660156, 46.10230255126953, 46.10230255126953, 46.10230255126953, 46.10919952392578, 46.17070007324219, 46.18790054321289, 46.18790054321289, 46.198699951171875, 46.198699951171875, 46.212100982666016, 46.222900390625, 46.23659896850586, 46.23659896850586, 46.23659896850586, 46.23659896850586, 46.240997314453125, 46.285499572753906, 46.285499572753906, 46.285499572753906, 46.285499572753906, 46.30180358886719, 46.3052978515625, 46.3052978515625, 46.3052978515625, 46.3052978515625, 46.30590057373047, 46.336204528808594, 46.368499755859375, 46.42890167236328, 46.42890167236328, 46.45289611816406, 46.468299865722656, 46.468299865722656, 46.468299865722656, 46.48200225830078, 46.48959732055664, 46.563499450683594, 46.563499450683594, 46.563499450683594, 46.56780242919922, 46.58380126953125, 46.61499786376953, 46.61499786376953, 46.64459991455078, 46.65079879760742, 46.65530014038086, 46.67279815673828, 46.67279815673828, 46.70039749145508, 46.714202880859375, 46.74690246582031, 46.74690246582031, 46.75600051879883, 46.75600051879883, 46.75600051879883, 46.766700744628906, 46.766700744628906, 46.766700744628906, 46.766700744628906, 46.766700744628906, 46.766700744628906, 46.766700744628906, 46.766700744628906, 46.766700744628906, 46.766700744628906, 46.822200775146484, 46.822200775146484, 46.822200775146484, 46.822200775146484, 46.82379913330078, 46.86199951171875, 46.870399475097656, 46.870399475097656, 46.87969970703125, 46.889198303222656, 46.889198303222656, 46.889198303222656, 46.889198303222656, 46.889198303222656, 46.889198303222656, 46.889198303222656, 46.89259719848633, 46.89259719848633, 46.89259719848633, 46.903297424316406, 46.903297424316406, 46.903297424316406, 46.903297424316406, 46.903297424316406, 46.903297424316406, 46.903297424316406, 46.903297424316406, 46.903297424316406, 46.903297424316406, 46.903297424316406, 46.990196228027344, 46.990196228027344, 46.998600006103516, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.082801818847656, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.10130310058594, 47.11470031738281, 47.11470031738281, 47.11470031738281, 47.11470031738281, 47.11470031738281, 47.11470031738281, 47.11470031738281, 47.11470031738281, 47.11470031738281, 47.11470031738281, 47.11470031738281, 47.11470031738281, 47.1239013671875, 47.1239013671875, 47.1239013671875, 47.1239013671875, 47.1239013671875, 47.1239013671875, 47.1239013671875, 47.1239013671875, 47.169097900390625, 47.169097900390625, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.20650100708008, 47.2213020324707, 47.2213020324707, 47.2213020324707, 47.2213020324707, 47.2213020324707, 47.2213020324707, 47.26360321044922, 47.31919860839844, 47.31919860839844, 47.31919860839844, 47.31919860839844, 47.31919860839844, 47.31919860839844, 47.31919860839844, 47.31919860839844, 47.31919860839844, 47.31919860839844]</t>
         </is>
       </c>
     </row>

</xml_diff>